<commit_message>
feat(crm): adiciona indicadores do pagador
</commit_message>
<xml_diff>
--- a/outputs/relatorio-cotacoes-fernanda-2026-07-07-a-2026-07-31.xlsx
+++ b/outputs/relatorio-cotacoes-fernanda-2026-07-07-a-2026-07-31.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ganhos" sheetId="1" r:id="R951641a0a9b14acb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Não ganhos" sheetId="2" r:id="R3a90ac19e9fc4651"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revisão" sheetId="3" r:id="R263ce13768d7464e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ganhos" sheetId="1" r:id="Rb41017288f5b4342"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Não ganhos" sheetId="2" r:id="R09ea195e873840ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revisão" sheetId="3" r:id="R75189d45f6854b12"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,10 +15,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="200" formatCode="#,##0.00"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="dd/mm/yyyy"/>
+    <x:numFmt numFmtId="203" formatCode="#,##0"/>
   </x:numFmts>
   <x:fonts count="6">
     <x:font>
@@ -113,7 +114,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="39">
+  <x:cellXfs count="42">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -149,6 +150,13 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="5" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -437,6 +445,8 @@
     <x:col min="10" max="10" width="23" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="58" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="15" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -548,6 +558,12 @@
       <x:c r="L11" s="17" t="str">
         <x:v>Observação</x:v>
       </x:c>
+      <x:c r="M11" s="17" t="str">
+        <x:v>Tabela Preço</x:v>
+      </x:c>
+      <x:c r="N11" s="17" t="str">
+        <x:v>CTes Ultimos 6 meses</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="13" t="str">
@@ -586,6 +602,12 @@
       <x:c r="L12" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M12" s="23" t="str">
+        <x:v>não</x:v>
+      </x:c>
+      <x:c r="N12" s="25" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="13" t="str">
@@ -624,6 +646,12 @@
       <x:c r="L13" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M13" s="23" t="str">
+        <x:v>não</x:v>
+      </x:c>
+      <x:c r="N13" s="25" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="13" t="str">
@@ -662,6 +690,12 @@
       <x:c r="L14" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M14" s="23" t="str">
+        <x:v>não</x:v>
+      </x:c>
+      <x:c r="N14" s="25" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="13" t="str">
@@ -700,6 +734,12 @@
       <x:c r="L15" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M15" s="23" t="str">
+        <x:v>sim</x:v>
+      </x:c>
+      <x:c r="N15" s="25" t="n">
+        <x:v>55</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="13" t="str">
@@ -738,6 +778,12 @@
       <x:c r="L16" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M16" s="23" t="str">
+        <x:v>sim</x:v>
+      </x:c>
+      <x:c r="N16" s="25" t="n">
+        <x:v>587</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="13" t="str">
@@ -776,6 +822,12 @@
       <x:c r="L17" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M17" s="23" t="str">
+        <x:v>não</x:v>
+      </x:c>
+      <x:c r="N17" s="25" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="13" t="str">
@@ -814,6 +866,12 @@
       <x:c r="L18" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M18" s="23" t="str">
+        <x:v>sim</x:v>
+      </x:c>
+      <x:c r="N18" s="25" t="n">
+        <x:v>30</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="13" t="str">
@@ -852,6 +910,12 @@
       <x:c r="L19" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M19" s="23" t="str">
+        <x:v>não</x:v>
+      </x:c>
+      <x:c r="N19" s="25" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="13" t="str">
@@ -890,6 +954,12 @@
       <x:c r="L20" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M20" s="23" t="str">
+        <x:v>sim</x:v>
+      </x:c>
+      <x:c r="N20" s="25" t="n">
+        <x:v>25</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="13" t="str">
@@ -928,6 +998,12 @@
       <x:c r="L21" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M21" s="23" t="str">
+        <x:v>sim</x:v>
+      </x:c>
+      <x:c r="N21" s="25" t="n">
+        <x:v>55</x:v>
+      </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="13" t="str">
@@ -966,6 +1042,12 @@
       <x:c r="L22" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M22" s="23" t="str">
+        <x:v>não</x:v>
+      </x:c>
+      <x:c r="N22" s="25" t="n">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="13" t="str">
@@ -1004,6 +1086,12 @@
       <x:c r="L23" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M23" s="23" t="str">
+        <x:v>não</x:v>
+      </x:c>
+      <x:c r="N23" s="25" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="13" t="str">
@@ -1042,6 +1130,12 @@
       <x:c r="L24" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M24" s="23" t="str">
+        <x:v>sim</x:v>
+      </x:c>
+      <x:c r="N24" s="25" t="n">
+        <x:v>55</x:v>
+      </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="13" t="str">
@@ -1080,6 +1174,12 @@
       <x:c r="L25" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M25" s="23" t="str">
+        <x:v>não</x:v>
+      </x:c>
+      <x:c r="N25" s="25" t="n">
+        <x:v>6</x:v>
+      </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="13" t="str">
@@ -1118,6 +1218,12 @@
       <x:c r="L26" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M26" s="23" t="str">
+        <x:v>não</x:v>
+      </x:c>
+      <x:c r="N26" s="25" t="n">
+        <x:v>14</x:v>
+      </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="13" t="str">
@@ -1156,6 +1262,12 @@
       <x:c r="L27" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M27" s="23" t="str">
+        <x:v>não</x:v>
+      </x:c>
+      <x:c r="N27" s="25" t="n">
+        <x:v>9</x:v>
+      </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="13" t="str">
@@ -1194,6 +1306,12 @@
       <x:c r="L28" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M28" s="23" t="str">
+        <x:v>não</x:v>
+      </x:c>
+      <x:c r="N28" s="25" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="13" t="str">
@@ -1232,6 +1350,12 @@
       <x:c r="L29" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M29" s="23" t="str">
+        <x:v>não</x:v>
+      </x:c>
+      <x:c r="N29" s="25" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="13" t="str">
@@ -1270,6 +1394,12 @@
       <x:c r="L30" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M30" s="23" t="str">
+        <x:v>sim</x:v>
+      </x:c>
+      <x:c r="N30" s="25" t="n">
+        <x:v>14</x:v>
+      </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="13" t="str">
@@ -1308,6 +1438,12 @@
       <x:c r="L31" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M31" s="23" t="str">
+        <x:v>não</x:v>
+      </x:c>
+      <x:c r="N31" s="25" t="n">
+        <x:v>47</x:v>
+      </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="13" t="str">
@@ -1346,6 +1482,12 @@
       <x:c r="L32" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M32" s="23" t="str">
+        <x:v>sim</x:v>
+      </x:c>
+      <x:c r="N32" s="25" t="n">
+        <x:v>55</x:v>
+      </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="13" t="str">
@@ -1384,6 +1526,12 @@
       <x:c r="L33" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M33" s="23" t="str">
+        <x:v>não</x:v>
+      </x:c>
+      <x:c r="N33" s="25" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="13" t="str">
@@ -1422,6 +1570,12 @@
       <x:c r="L34" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M34" s="23" t="str">
+        <x:v>não</x:v>
+      </x:c>
+      <x:c r="N34" s="25" t="n">
+        <x:v>1</x:v>
+      </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="13" t="str">
@@ -1460,6 +1614,12 @@
       <x:c r="L35" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M35" s="23" t="str">
+        <x:v>não</x:v>
+      </x:c>
+      <x:c r="N35" s="25" t="n">
+        <x:v>13</x:v>
+      </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="13" t="str">
@@ -1497,6 +1657,12 @@
       </x:c>
       <x:c r="L36" s="20" t="str">
         <x:v>CT-e localizado; emissão no dia ou após a cotação.</x:v>
+      </x:c>
+      <x:c r="M36" s="23" t="str">
+        <x:v>sim</x:v>
+      </x:c>
+      <x:c r="N36" s="25" t="n">
+        <x:v>300</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -1530,6 +1696,8 @@
       <x:c r="L37" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M37" s="23" t="str"/>
+      <x:c r="N37" s="25" t="str"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="13" t="str">
@@ -1556,6 +1724,8 @@
       <x:c r="L38" s="20" t="str">
         <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
+      <x:c r="M38" s="23" t="str"/>
+      <x:c r="N38" s="25" t="str"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="13" t="str">
@@ -1588,6 +1758,8 @@
       <x:c r="L39" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M39" s="23" t="str"/>
+      <x:c r="N39" s="25" t="str"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="13" t="str">
@@ -1620,6 +1792,8 @@
       <x:c r="L40" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M40" s="23" t="str"/>
+      <x:c r="N40" s="25" t="str"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="13" t="str">
@@ -1652,6 +1826,8 @@
       <x:c r="L41" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M41" s="23" t="str"/>
+      <x:c r="N41" s="25" t="str"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="13" t="str">
@@ -1684,6 +1860,8 @@
       <x:c r="L42" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M42" s="23" t="str"/>
+      <x:c r="N42" s="25" t="str"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="13" t="str">
@@ -1716,6 +1894,8 @@
       <x:c r="L43" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M43" s="23" t="str"/>
+      <x:c r="N43" s="25" t="str"/>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="13" t="str">
@@ -1748,6 +1928,8 @@
       <x:c r="L44" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
+      <x:c r="M44" s="23" t="str"/>
+      <x:c r="N44" s="25" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1756,7 +1938,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c1763c5a3804220"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14fda1a0477c4afb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1780,20 +1962,20 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="25" t="str">
+      <x:c r="A1" s="28" t="str">
         <x:v>Cotações não ganhas — Cubo x Legado</x:v>
       </x:c>
-      <x:c r="B1" s="25"/>
-      <x:c r="C1" s="25"/>
-      <x:c r="D1" s="25"/>
-      <x:c r="E1" s="25"/>
-      <x:c r="F1" s="25"/>
-      <x:c r="G1" s="25"/>
-      <x:c r="H1" s="25"/>
-      <x:c r="I1" s="25"/>
-      <x:c r="J1" s="25"/>
-      <x:c r="K1" s="25"/>
-      <x:c r="L1" s="25"/>
+      <x:c r="B1" s="28"/>
+      <x:c r="C1" s="28"/>
+      <x:c r="D1" s="28"/>
+      <x:c r="E1" s="28"/>
+      <x:c r="F1" s="28"/>
+      <x:c r="G1" s="28"/>
+      <x:c r="H1" s="28"/>
+      <x:c r="I1" s="28"/>
+      <x:c r="J1" s="28"/>
+      <x:c r="K1" s="28"/>
+      <x:c r="L1" s="28"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="6" t="str">
@@ -1812,10 +1994,10 @@
       <x:c r="L2" s="6"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="27" t="str">
+      <x:c r="A4" s="30" t="str">
         <x:v>Resumo</x:v>
       </x:c>
-      <x:c r="B4" s="27" t="str">
+      <x:c r="B4" s="30" t="str">
         <x:v>Valor</x:v>
       </x:c>
     </x:row>
@@ -1852,40 +2034,40 @@
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="30" t="str">
+      <x:c r="A11" s="33" t="str">
         <x:v>Título</x:v>
       </x:c>
-      <x:c r="B11" s="30" t="str">
+      <x:c r="B11" s="33" t="str">
         <x:v>ID card Cubo</x:v>
       </x:c>
-      <x:c r="C11" s="30" t="str">
+      <x:c r="C11" s="33" t="str">
         <x:v>Cotação</x:v>
       </x:c>
-      <x:c r="D11" s="30" t="str">
+      <x:c r="D11" s="33" t="str">
         <x:v>Status Cubo</x:v>
       </x:c>
-      <x:c r="E11" s="30" t="str">
+      <x:c r="E11" s="33" t="str">
         <x:v>Data status Cubo</x:v>
       </x:c>
-      <x:c r="F11" s="30" t="str">
+      <x:c r="F11" s="33" t="str">
         <x:v>Valor Cubo</x:v>
       </x:c>
-      <x:c r="G11" s="30" t="str">
+      <x:c r="G11" s="33" t="str">
         <x:v>CT-e</x:v>
       </x:c>
-      <x:c r="H11" s="30" t="str">
+      <x:c r="H11" s="33" t="str">
         <x:v>Valor CT-e</x:v>
       </x:c>
-      <x:c r="I11" s="30" t="str">
+      <x:c r="I11" s="33" t="str">
         <x:v>Emissão CT-e</x:v>
       </x:c>
-      <x:c r="J11" s="30" t="str">
+      <x:c r="J11" s="33" t="str">
         <x:v>Status cotação legado</x:v>
       </x:c>
-      <x:c r="K11" s="30" t="str">
+      <x:c r="K11" s="33" t="str">
         <x:v>Valor cotação legado</x:v>
       </x:c>
-      <x:c r="L11" s="30" t="str">
+      <x:c r="L11" s="33" t="str">
         <x:v>Observação</x:v>
       </x:c>
     </x:row>
@@ -5296,7 +5478,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b12e32ff82e495b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref4d4d49bfc64edb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5320,20 +5502,20 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="33" t="str">
+      <x:c r="A1" s="36" t="str">
         <x:v>Revisão — não ganhos com CT-e na data ou após status Cubo</x:v>
       </x:c>
-      <x:c r="B1" s="33"/>
-      <x:c r="C1" s="33"/>
-      <x:c r="D1" s="33"/>
-      <x:c r="E1" s="33"/>
-      <x:c r="F1" s="33"/>
-      <x:c r="G1" s="33"/>
-      <x:c r="H1" s="33"/>
-      <x:c r="I1" s="33"/>
-      <x:c r="J1" s="33"/>
-      <x:c r="K1" s="33"/>
-      <x:c r="L1" s="33"/>
+      <x:c r="B1" s="36"/>
+      <x:c r="C1" s="36"/>
+      <x:c r="D1" s="36"/>
+      <x:c r="E1" s="36"/>
+      <x:c r="F1" s="36"/>
+      <x:c r="G1" s="36"/>
+      <x:c r="H1" s="36"/>
+      <x:c r="I1" s="36"/>
+      <x:c r="J1" s="36"/>
+      <x:c r="K1" s="36"/>
+      <x:c r="L1" s="36"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="6" t="str">
@@ -5352,10 +5534,10 @@
       <x:c r="L2" s="6"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="35" t="str">
+      <x:c r="A4" s="38" t="str">
         <x:v>Resumo</x:v>
       </x:c>
-      <x:c r="B4" s="35" t="str">
+      <x:c r="B4" s="38" t="str">
         <x:v>Valor</x:v>
       </x:c>
     </x:row>
@@ -5368,40 +5550,40 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="38" t="str">
+      <x:c r="A10" s="41" t="str">
         <x:v>Título</x:v>
       </x:c>
-      <x:c r="B10" s="38" t="str">
+      <x:c r="B10" s="41" t="str">
         <x:v>ID card Cubo</x:v>
       </x:c>
-      <x:c r="C10" s="38" t="str">
+      <x:c r="C10" s="41" t="str">
         <x:v>Cotação</x:v>
       </x:c>
-      <x:c r="D10" s="38" t="str">
+      <x:c r="D10" s="41" t="str">
         <x:v>Status Cubo</x:v>
       </x:c>
-      <x:c r="E10" s="38" t="str">
+      <x:c r="E10" s="41" t="str">
         <x:v>Data status Cubo</x:v>
       </x:c>
-      <x:c r="F10" s="38" t="str">
+      <x:c r="F10" s="41" t="str">
         <x:v>Valor Cubo</x:v>
       </x:c>
-      <x:c r="G10" s="38" t="str">
+      <x:c r="G10" s="41" t="str">
         <x:v>CT-e</x:v>
       </x:c>
-      <x:c r="H10" s="38" t="str">
+      <x:c r="H10" s="41" t="str">
         <x:v>Valor CT-e</x:v>
       </x:c>
-      <x:c r="I10" s="38" t="str">
+      <x:c r="I10" s="41" t="str">
         <x:v>Emissão CT-e</x:v>
       </x:c>
-      <x:c r="J10" s="38" t="str">
+      <x:c r="J10" s="41" t="str">
         <x:v>Status cotação legado</x:v>
       </x:c>
-      <x:c r="K10" s="38" t="str">
+      <x:c r="K10" s="41" t="str">
         <x:v>Valor cotação legado</x:v>
       </x:c>
-      <x:c r="L10" s="38" t="str">
+      <x:c r="L10" s="41" t="str">
         <x:v>Observação</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
fix(crm): filtra cards pelo estagio da proposta
</commit_message>
<xml_diff>
--- a/outputs/relatorio-cotacoes-fernanda-2026-07-07-a-2026-07-31.xlsx
+++ b/outputs/relatorio-cotacoes-fernanda-2026-07-07-a-2026-07-31.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ganhos" sheetId="1" r:id="Rb41017288f5b4342"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Não ganhos" sheetId="2" r:id="R09ea195e873840ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revisão" sheetId="3" r:id="R75189d45f6854b12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ganhos" sheetId="1" r:id="Re3604f7c3b2843c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Não ganhos" sheetId="2" r:id="R2659556bd2814b33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revisão" sheetId="3" r:id="R3d19e4d693484a01"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -218,8 +218,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="NoganhosTable" displayName="NoganhosTable" ref="A11:L124" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A11:L124"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="NoganhosTable" displayName="NoganhosTable" ref="A11:L84" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A11:L84"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Título"/>
     <x:tableColumn id="2" name="ID card Cubo"/>
@@ -1938,7 +1938,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14fda1a0477c4afb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08a11a15f11748d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2006,7 +2006,7 @@
         <x:v>Cards</x:v>
       </x:c>
       <x:c r="B5" s="13" t="n">
-        <x:v>113</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2304,184 +2304,220 @@
         <x:v>Fernanda Qualisol</x:v>
       </x:c>
       <x:c r="B18" s="18" t="n">
-        <x:v>2182011</x:v>
-      </x:c>
-      <x:c r="C18" s="13" t="str"/>
+        <x:v>2183458</x:v>
+      </x:c>
+      <x:c r="C18" s="13" t="n">
+        <x:v>15285</x:v>
+      </x:c>
       <x:c r="D18" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E18" s="19" t="n">
-        <x:v>46210.48128472222</x:v>
+        <x:v>46216.70232638889</x:v>
       </x:c>
       <x:c r="F18" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>375.07</x:v>
       </x:c>
       <x:c r="G18" s="18"/>
       <x:c r="H18" s="14"/>
       <x:c r="I18" s="19"/>
-      <x:c r="J18" s="13" t="str"/>
-      <x:c r="K18" s="14"/>
+      <x:c r="J18" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K18" s="14" t="n">
+        <x:v>375.07</x:v>
+      </x:c>
       <x:c r="L18" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="13" t="str">
-        <x:v>FORP - Atendimento</x:v>
+        <x:v>Carmaço - Fiori</x:v>
       </x:c>
       <x:c r="B19" s="18" t="n">
-        <x:v>2182667</x:v>
-      </x:c>
-      <x:c r="C19" s="13" t="str"/>
+        <x:v>2191676</x:v>
+      </x:c>
+      <x:c r="C19" s="13" t="n">
+        <x:v>15316</x:v>
+      </x:c>
       <x:c r="D19" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E19" s="19" t="n">
-        <x:v>46210.777083333334</x:v>
+        <x:v>46219.57885416667</x:v>
       </x:c>
       <x:c r="F19" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>660.68</x:v>
       </x:c>
       <x:c r="G19" s="18"/>
       <x:c r="H19" s="14"/>
       <x:c r="I19" s="19"/>
-      <x:c r="J19" s="13" t="str"/>
-      <x:c r="K19" s="14"/>
+      <x:c r="J19" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K19" s="14" t="n">
+        <x:v>581.14</x:v>
+      </x:c>
       <x:c r="L19" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="13" t="str">
-        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
+        <x:v>Fernanda Qualisol</x:v>
       </x:c>
       <x:c r="B20" s="18" t="n">
-        <x:v>2181990</x:v>
-      </x:c>
-      <x:c r="C20" s="13" t="str"/>
+        <x:v>2193323</x:v>
+      </x:c>
+      <x:c r="C20" s="13" t="n">
+        <x:v>15326</x:v>
+      </x:c>
       <x:c r="D20" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E20" s="19" t="n">
-        <x:v>46211.73475694445</x:v>
+        <x:v>46219.695081018515</x:v>
       </x:c>
       <x:c r="F20" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>156.68</x:v>
       </x:c>
       <x:c r="G20" s="18"/>
       <x:c r="H20" s="14"/>
       <x:c r="I20" s="19"/>
-      <x:c r="J20" s="13" t="str"/>
-      <x:c r="K20" s="14"/>
+      <x:c r="J20" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K20" s="14" t="n">
+        <x:v>156.68</x:v>
+      </x:c>
       <x:c r="L20" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="13" t="str">
-        <x:v>Fábio Henrique</x:v>
+        <x:v>Fernanda Qualisol</x:v>
       </x:c>
       <x:c r="B21" s="18" t="n">
-        <x:v>2187342</x:v>
-      </x:c>
-      <x:c r="C21" s="13" t="str"/>
+        <x:v>2193563</x:v>
+      </x:c>
+      <x:c r="C21" s="13" t="n">
+        <x:v>15328</x:v>
+      </x:c>
       <x:c r="D21" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E21" s="19" t="n">
-        <x:v>46213.51280092593</x:v>
+        <x:v>46219.754375</x:v>
       </x:c>
       <x:c r="F21" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>434.59</x:v>
       </x:c>
       <x:c r="G21" s="18"/>
       <x:c r="H21" s="14"/>
       <x:c r="I21" s="19"/>
-      <x:c r="J21" s="13" t="str"/>
-      <x:c r="K21" s="14"/>
+      <x:c r="J21" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K21" s="14" t="n">
+        <x:v>434.59</x:v>
+      </x:c>
       <x:c r="L21" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="13" t="str">
-        <x:v>Maria Teresa Adorno</x:v>
+        <x:v>Comercial IQL-NEXUS</x:v>
       </x:c>
       <x:c r="B22" s="18" t="n">
-        <x:v>2189251</x:v>
-      </x:c>
-      <x:c r="C22" s="13" t="str"/>
+        <x:v>2193205</x:v>
+      </x:c>
+      <x:c r="C22" s="13" t="n">
+        <x:v>15324</x:v>
+      </x:c>
       <x:c r="D22" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E22" s="19" t="n">
-        <x:v>46216.51372685185</x:v>
+        <x:v>46220.549305555556</x:v>
       </x:c>
       <x:c r="F22" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>1529.67</x:v>
       </x:c>
       <x:c r="G22" s="18"/>
       <x:c r="H22" s="14"/>
       <x:c r="I22" s="19"/>
-      <x:c r="J22" s="13" t="str"/>
-      <x:c r="K22" s="14"/>
+      <x:c r="J22" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K22" s="14" t="n">
+        <x:v>1529.67</x:v>
+      </x:c>
       <x:c r="L22" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="13" t="str">
-        <x:v>Milena Montoro (comercial) Bold SJRP</x:v>
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
       </x:c>
       <x:c r="B23" s="18" t="n">
-        <x:v>2189604</x:v>
-      </x:c>
-      <x:c r="C23" s="13" t="str"/>
+        <x:v>2194690</x:v>
+      </x:c>
+      <x:c r="C23" s="13" t="n">
+        <x:v>15337</x:v>
+      </x:c>
       <x:c r="D23" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E23" s="19" t="n">
-        <x:v>46216.51372685185</x:v>
+        <x:v>46220.74028935185</x:v>
       </x:c>
       <x:c r="F23" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>164.17</x:v>
       </x:c>
       <x:c r="G23" s="18"/>
       <x:c r="H23" s="14"/>
       <x:c r="I23" s="19"/>
-      <x:c r="J23" s="13" t="str"/>
-      <x:c r="K23" s="14"/>
+      <x:c r="J23" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K23" s="14" t="n">
+        <x:v>164.17</x:v>
+      </x:c>
       <x:c r="L23" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="13" t="str">
-        <x:v>Fernanda Qualisol</x:v>
+        <x:v>Roseli - Industria Portas</x:v>
       </x:c>
       <x:c r="B24" s="18" t="n">
-        <x:v>2183458</x:v>
+        <x:v>2196088</x:v>
       </x:c>
       <x:c r="C24" s="13" t="n">
-        <x:v>15285</x:v>
+        <x:v>15341</x:v>
       </x:c>
       <x:c r="D24" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E24" s="19" t="n">
-        <x:v>46216.70232638889</x:v>
+        <x:v>46223.494039351855</x:v>
       </x:c>
       <x:c r="F24" s="14" t="n">
-        <x:v>375.07</x:v>
+        <x:v>295.86</x:v>
       </x:c>
       <x:c r="G24" s="18"/>
       <x:c r="H24" s="14"/>
       <x:c r="I24" s="19"/>
       <x:c r="J24" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K24" s="14" t="n">
-        <x:v>375.07</x:v>
+        <x:v>295.86</x:v>
       </x:c>
       <x:c r="L24" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -2489,178 +2525,214 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="13" t="str">
-        <x:v>Transporte Bautech</x:v>
+        <x:v>Rosset Cia 2 Devoluções</x:v>
       </x:c>
       <x:c r="B25" s="18" t="n">
-        <x:v>2191301</x:v>
-      </x:c>
-      <x:c r="C25" s="13" t="str"/>
+        <x:v>2190103</x:v>
+      </x:c>
+      <x:c r="C25" s="13" t="n">
+        <x:v>15300</x:v>
+      </x:c>
       <x:c r="D25" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E25" s="19" t="n">
-        <x:v>46217.57435185185</x:v>
+        <x:v>46223.590682870374</x:v>
       </x:c>
       <x:c r="F25" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>927.98</x:v>
       </x:c>
       <x:c r="G25" s="18"/>
       <x:c r="H25" s="14"/>
       <x:c r="I25" s="19"/>
-      <x:c r="J25" s="13" t="str"/>
-      <x:c r="K25" s="14"/>
+      <x:c r="J25" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K25" s="14" t="n">
+        <x:v>927.98</x:v>
+      </x:c>
       <x:c r="L25" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="13" t="str">
-        <x:v>Suelen 💕 suu</x:v>
+        <x:v>MARCEL FACAS</x:v>
       </x:c>
       <x:c r="B26" s="18" t="n">
-        <x:v>2192502</x:v>
-      </x:c>
-      <x:c r="C26" s="13" t="str"/>
+        <x:v>2191327</x:v>
+      </x:c>
+      <x:c r="C26" s="13" t="n">
+        <x:v>15306</x:v>
+      </x:c>
       <x:c r="D26" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E26" s="19" t="n">
-        <x:v>46218.60891203704</x:v>
+        <x:v>46223.7403587963</x:v>
       </x:c>
       <x:c r="F26" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>255.51</x:v>
       </x:c>
       <x:c r="G26" s="18"/>
       <x:c r="H26" s="14"/>
       <x:c r="I26" s="19"/>
-      <x:c r="J26" s="13" t="str"/>
-      <x:c r="K26" s="14"/>
+      <x:c r="J26" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K26" s="14" t="n">
+        <x:v>255.51</x:v>
+      </x:c>
       <x:c r="L26" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="13" t="str">
-        <x:v>Sterimed-Sterimais-finan</x:v>
+        <x:v>Evelyn Brito</x:v>
       </x:c>
       <x:c r="B27" s="18" t="n">
-        <x:v>2192326</x:v>
-      </x:c>
-      <x:c r="C27" s="13" t="str"/>
+        <x:v>2191363</x:v>
+      </x:c>
+      <x:c r="C27" s="13" t="n">
+        <x:v>15307</x:v>
+      </x:c>
       <x:c r="D27" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E27" s="19" t="n">
-        <x:v>46218.6983912037</x:v>
+        <x:v>46223.7403587963</x:v>
       </x:c>
       <x:c r="F27" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>493.92</x:v>
       </x:c>
       <x:c r="G27" s="18"/>
       <x:c r="H27" s="14"/>
       <x:c r="I27" s="19"/>
-      <x:c r="J27" s="13" t="str"/>
-      <x:c r="K27" s="14"/>
+      <x:c r="J27" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K27" s="14" t="n">
+        <x:v>493.92</x:v>
+      </x:c>
       <x:c r="L27" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="13" t="str">
-        <x:v>Galtron Quimica Vendas</x:v>
+        <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B28" s="18" t="n">
-        <x:v>2192650</x:v>
-      </x:c>
-      <x:c r="C28" s="13" t="str"/>
+        <x:v>2182299</x:v>
+      </x:c>
+      <x:c r="C28" s="13" t="n">
+        <x:v>15276</x:v>
+      </x:c>
       <x:c r="D28" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E28" s="19" t="n">
-        <x:v>46218.729583333334</x:v>
+        <x:v>46223.747824074075</x:v>
       </x:c>
       <x:c r="F28" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>364.03</x:v>
       </x:c>
       <x:c r="G28" s="18"/>
       <x:c r="H28" s="14"/>
       <x:c r="I28" s="19"/>
-      <x:c r="J28" s="13" t="str"/>
-      <x:c r="K28" s="14"/>
+      <x:c r="J28" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K28" s="14" t="n">
+        <x:v>364.03</x:v>
+      </x:c>
       <x:c r="L28" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="13" t="str">
-        <x:v>Ronaldo Rampazzo</x:v>
+        <x:v>VINICIUS BERNARDES TEIXEIRA</x:v>
       </x:c>
       <x:c r="B29" s="18" t="n">
-        <x:v>2192708</x:v>
-      </x:c>
-      <x:c r="C29" s="13" t="str"/>
+        <x:v>2182658</x:v>
+      </x:c>
+      <x:c r="C29" s="13" t="n">
+        <x:v>15280</x:v>
+      </x:c>
       <x:c r="D29" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E29" s="19" t="n">
-        <x:v>46218.77347222222</x:v>
+        <x:v>46223.747824074075</x:v>
       </x:c>
       <x:c r="F29" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>112.77</x:v>
       </x:c>
       <x:c r="G29" s="18"/>
       <x:c r="H29" s="14"/>
       <x:c r="I29" s="19"/>
-      <x:c r="J29" s="13" t="str"/>
-      <x:c r="K29" s="14"/>
+      <x:c r="J29" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K29" s="14" t="n">
+        <x:v>112.77</x:v>
+      </x:c>
       <x:c r="L29" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="13" t="str">
-        <x:v>Vendas TELAS MM</x:v>
+        <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B30" s="18" t="n">
-        <x:v>2192745</x:v>
-      </x:c>
-      <x:c r="C30" s="13" t="str"/>
+        <x:v>2192401</x:v>
+      </x:c>
+      <x:c r="C30" s="13" t="n">
+        <x:v>15318</x:v>
+      </x:c>
       <x:c r="D30" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E30" s="19" t="n">
-        <x:v>46218.807800925926</x:v>
+        <x:v>46223.76341435185</x:v>
       </x:c>
       <x:c r="F30" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>561.43</x:v>
       </x:c>
       <x:c r="G30" s="18"/>
       <x:c r="H30" s="14"/>
       <x:c r="I30" s="19"/>
-      <x:c r="J30" s="13" t="str"/>
-      <x:c r="K30" s="14"/>
+      <x:c r="J30" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K30" s="14" t="n">
+        <x:v>561.43</x:v>
+      </x:c>
       <x:c r="L30" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="13" t="str">
-        <x:v>Carmaço - Fiori</x:v>
+        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
       </x:c>
       <x:c r="B31" s="18" t="n">
-        <x:v>2191676</x:v>
+        <x:v>2183959</x:v>
       </x:c>
       <x:c r="C31" s="13" t="n">
-        <x:v>15316</x:v>
+        <x:v>15290</x:v>
       </x:c>
       <x:c r="D31" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E31" s="19" t="n">
-        <x:v>46219.57885416667</x:v>
+        <x:v>46223.782789351855</x:v>
       </x:c>
       <x:c r="F31" s="14" t="n">
-        <x:v>660.68</x:v>
+        <x:v>381.23</x:v>
       </x:c>
       <x:c r="G31" s="18"/>
       <x:c r="H31" s="14"/>
@@ -2669,7 +2741,7 @@
         <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K31" s="14" t="n">
-        <x:v>581.14</x:v>
+        <x:v>381.23</x:v>
       </x:c>
       <x:c r="L31" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -2677,22 +2749,22 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="13" t="str">
-        <x:v>Fernanda Qualisol</x:v>
+        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
       </x:c>
       <x:c r="B32" s="18" t="n">
-        <x:v>2193323</x:v>
+        <x:v>2182032</x:v>
       </x:c>
       <x:c r="C32" s="13" t="n">
-        <x:v>15326</x:v>
+        <x:v>15172</x:v>
       </x:c>
       <x:c r="D32" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E32" s="19" t="n">
-        <x:v>46219.695081018515</x:v>
+        <x:v>46223.784583333334</x:v>
       </x:c>
       <x:c r="F32" s="14" t="n">
-        <x:v>156.68</x:v>
+        <x:v>421.48</x:v>
       </x:c>
       <x:c r="G32" s="18"/>
       <x:c r="H32" s="14"/>
@@ -2701,7 +2773,7 @@
         <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K32" s="14" t="n">
-        <x:v>156.68</x:v>
+        <x:v>2788.47</x:v>
       </x:c>
       <x:c r="L32" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -2709,31 +2781,31 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="13" t="str">
-        <x:v>Fernanda Qualisol</x:v>
+        <x:v>Rosset Cia 2 Devoluções</x:v>
       </x:c>
       <x:c r="B33" s="18" t="n">
-        <x:v>2193563</x:v>
+        <x:v>2196879</x:v>
       </x:c>
       <x:c r="C33" s="13" t="n">
-        <x:v>15328</x:v>
+        <x:v>15344</x:v>
       </x:c>
       <x:c r="D33" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E33" s="19" t="n">
-        <x:v>46219.754375</x:v>
+        <x:v>46224.4844212963</x:v>
       </x:c>
       <x:c r="F33" s="14" t="n">
-        <x:v>434.59</x:v>
+        <x:v>927.98</x:v>
       </x:c>
       <x:c r="G33" s="18"/>
       <x:c r="H33" s="14"/>
       <x:c r="I33" s="19"/>
       <x:c r="J33" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K33" s="14" t="n">
-        <x:v>434.59</x:v>
+        <x:v>927.98</x:v>
       </x:c>
       <x:c r="L33" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -2741,83 +2813,95 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="13" t="str">
-        <x:v>leozero</x:v>
+        <x:v>longo cadastro</x:v>
       </x:c>
       <x:c r="B34" s="18" t="n">
-        <x:v>2193724</x:v>
-      </x:c>
-      <x:c r="C34" s="13" t="str"/>
+        <x:v>2197779</x:v>
+      </x:c>
+      <x:c r="C34" s="13" t="n">
+        <x:v>15346</x:v>
+      </x:c>
       <x:c r="D34" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E34" s="19" t="n">
-        <x:v>46220.46858796296</x:v>
+        <x:v>46224.60364583333</x:v>
       </x:c>
       <x:c r="F34" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>2324.41</x:v>
       </x:c>
       <x:c r="G34" s="18"/>
       <x:c r="H34" s="14"/>
       <x:c r="I34" s="19"/>
-      <x:c r="J34" s="13" t="str"/>
-      <x:c r="K34" s="14"/>
+      <x:c r="J34" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K34" s="14" t="n">
+        <x:v>2324.41</x:v>
+      </x:c>
       <x:c r="L34" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="13" t="str">
-        <x:v>Victor logística Dom Tapparo</x:v>
+        <x:v>Itamonte l +Luz Iluminação l Vanessa C.</x:v>
       </x:c>
       <x:c r="B35" s="18" t="n">
-        <x:v>2193804</x:v>
-      </x:c>
-      <x:c r="C35" s="13" t="str"/>
+        <x:v>2197933</x:v>
+      </x:c>
+      <x:c r="C35" s="13" t="n">
+        <x:v>15350</x:v>
+      </x:c>
       <x:c r="D35" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E35" s="19" t="n">
-        <x:v>46220.54813657407</x:v>
+        <x:v>46224.61032407408</x:v>
       </x:c>
       <x:c r="F35" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>244.8</x:v>
       </x:c>
       <x:c r="G35" s="18"/>
       <x:c r="H35" s="14"/>
       <x:c r="I35" s="19"/>
-      <x:c r="J35" s="13" t="str"/>
-      <x:c r="K35" s="14"/>
+      <x:c r="J35" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K35" s="14" t="n">
+        <x:v>244.8</x:v>
+      </x:c>
       <x:c r="L35" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="13" t="str">
-        <x:v>Comercial IQL-NEXUS</x:v>
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA</x:v>
       </x:c>
       <x:c r="B36" s="18" t="n">
-        <x:v>2193205</x:v>
+        <x:v>2198195</x:v>
       </x:c>
       <x:c r="C36" s="13" t="n">
-        <x:v>15324</x:v>
+        <x:v>15349</x:v>
       </x:c>
       <x:c r="D36" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E36" s="19" t="n">
-        <x:v>46220.549305555556</x:v>
+        <x:v>46224.73436342592</x:v>
       </x:c>
       <x:c r="F36" s="14" t="n">
-        <x:v>1529.67</x:v>
+        <x:v>145.3</x:v>
       </x:c>
       <x:c r="G36" s="18"/>
       <x:c r="H36" s="14"/>
       <x:c r="I36" s="19"/>
       <x:c r="J36" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K36" s="14" t="n">
-        <x:v>1529.67</x:v>
+        <x:v>145.3</x:v>
       </x:c>
       <x:c r="L36" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -2825,46 +2909,52 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="13" t="str">
-        <x:v>leozero</x:v>
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA</x:v>
       </x:c>
       <x:c r="B37" s="18" t="n">
-        <x:v>2194562</x:v>
-      </x:c>
-      <x:c r="C37" s="13" t="str"/>
+        <x:v>2198196</x:v>
+      </x:c>
+      <x:c r="C37" s="13" t="n">
+        <x:v>15353</x:v>
+      </x:c>
       <x:c r="D37" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E37" s="19" t="n">
-        <x:v>46220.668587962966</x:v>
+        <x:v>46224.73789351852</x:v>
       </x:c>
       <x:c r="F37" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>142.51</x:v>
       </x:c>
       <x:c r="G37" s="18"/>
       <x:c r="H37" s="14"/>
       <x:c r="I37" s="19"/>
-      <x:c r="J37" s="13" t="str"/>
-      <x:c r="K37" s="14"/>
+      <x:c r="J37" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K37" s="14" t="n">
+        <x:v>142.51</x:v>
+      </x:c>
       <x:c r="L37" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="13" t="str">
-        <x:v>J.a.t.t</x:v>
+        <x:v>Compras - Insertec Fornos e Refratários</x:v>
       </x:c>
       <x:c r="B38" s="18" t="n">
-        <x:v>2193326</x:v>
+        <x:v>2194633</x:v>
       </x:c>
       <x:c r="C38" s="13" t="str"/>
       <x:c r="D38" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E38" s="19" t="n">
-        <x:v>46220.71637731481</x:v>
+        <x:v>46224.77175925926</x:v>
       </x:c>
       <x:c r="F38" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>311.03</x:v>
       </x:c>
       <x:c r="G38" s="18"/>
       <x:c r="H38" s="14"/>
@@ -2877,22 +2967,22 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
+        <x:v>Fernanda Qualisol</x:v>
       </x:c>
       <x:c r="B39" s="18" t="n">
-        <x:v>2194690</x:v>
+        <x:v>2198771</x:v>
       </x:c>
       <x:c r="C39" s="13" t="n">
-        <x:v>15337</x:v>
+        <x:v>15357</x:v>
       </x:c>
       <x:c r="D39" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E39" s="19" t="n">
-        <x:v>46220.74028935185</x:v>
+        <x:v>46225.53065972222</x:v>
       </x:c>
       <x:c r="F39" s="14" t="n">
-        <x:v>164.17</x:v>
+        <x:v>239.17</x:v>
       </x:c>
       <x:c r="G39" s="18"/>
       <x:c r="H39" s="14"/>
@@ -2901,7 +2991,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K39" s="14" t="n">
-        <x:v>164.17</x:v>
+        <x:v>239.17</x:v>
       </x:c>
       <x:c r="L39" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -2909,22 +2999,22 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="13" t="str">
-        <x:v>Roseli - Industria Portas</x:v>
+        <x:v>Fernanda Qualisol</x:v>
       </x:c>
       <x:c r="B40" s="18" t="n">
-        <x:v>2196088</x:v>
+        <x:v>2199721</x:v>
       </x:c>
       <x:c r="C40" s="13" t="n">
-        <x:v>15341</x:v>
+        <x:v>15364</x:v>
       </x:c>
       <x:c r="D40" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E40" s="19" t="n">
-        <x:v>46223.494039351855</x:v>
+        <x:v>46226.506423611114</x:v>
       </x:c>
       <x:c r="F40" s="14" t="n">
-        <x:v>295.86</x:v>
+        <x:v>283.27</x:v>
       </x:c>
       <x:c r="G40" s="18"/>
       <x:c r="H40" s="14"/>
@@ -2933,7 +3023,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K40" s="14" t="n">
-        <x:v>295.86</x:v>
+        <x:v>283.27</x:v>
       </x:c>
       <x:c r="L40" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -2941,31 +3031,31 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="13" t="str">
-        <x:v>Rosset Cia 2 Devoluções</x:v>
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA</x:v>
       </x:c>
       <x:c r="B41" s="18" t="n">
-        <x:v>2190103</x:v>
+        <x:v>2199791</x:v>
       </x:c>
       <x:c r="C41" s="13" t="n">
-        <x:v>15300</x:v>
+        <x:v>15365</x:v>
       </x:c>
       <x:c r="D41" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E41" s="19" t="n">
-        <x:v>46223.590682870374</x:v>
+        <x:v>46226.51068287037</x:v>
       </x:c>
       <x:c r="F41" s="14" t="n">
-        <x:v>927.98</x:v>
+        <x:v>125.99</x:v>
       </x:c>
       <x:c r="G41" s="18"/>
       <x:c r="H41" s="14"/>
       <x:c r="I41" s="19"/>
       <x:c r="J41" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K41" s="14" t="n">
-        <x:v>927.98</x:v>
+        <x:v>125.99</x:v>
       </x:c>
       <x:c r="L41" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -2973,63 +3063,57 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="13" t="str">
-        <x:v>MARCEL FACAS</x:v>
+        <x:v>IKTEC COMERCIO DE PROD PARA TRAT DE SUPERFICIE LTDA</x:v>
       </x:c>
       <x:c r="B42" s="18" t="n">
-        <x:v>2191327</x:v>
-      </x:c>
-      <x:c r="C42" s="13" t="n">
-        <x:v>15306</x:v>
-      </x:c>
+        <x:v>2199802</x:v>
+      </x:c>
+      <x:c r="C42" s="13" t="str"/>
       <x:c r="D42" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E42" s="19" t="n">
-        <x:v>46223.7403587963</x:v>
+        <x:v>46226.51582175926</x:v>
       </x:c>
       <x:c r="F42" s="14" t="n">
-        <x:v>255.51</x:v>
+        <x:v>158.2</x:v>
       </x:c>
       <x:c r="G42" s="18"/>
       <x:c r="H42" s="14"/>
       <x:c r="I42" s="19"/>
-      <x:c r="J42" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K42" s="14" t="n">
-        <x:v>255.51</x:v>
-      </x:c>
+      <x:c r="J42" s="13" t="str"/>
+      <x:c r="K42" s="14"/>
       <x:c r="L42" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="13" t="str">
-        <x:v>Evelyn Brito</x:v>
+        <x:v>BAUTECH INDUSTRIA E COMERCIO DE TINTAS LTDA</x:v>
       </x:c>
       <x:c r="B43" s="18" t="n">
-        <x:v>2191363</x:v>
+        <x:v>2199976</x:v>
       </x:c>
       <x:c r="C43" s="13" t="n">
-        <x:v>15307</x:v>
+        <x:v>15369</x:v>
       </x:c>
       <x:c r="D43" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E43" s="19" t="n">
-        <x:v>46223.7403587963</x:v>
+        <x:v>46226.614375</x:v>
       </x:c>
       <x:c r="F43" s="14" t="n">
-        <x:v>493.92</x:v>
+        <x:v>1301.93</x:v>
       </x:c>
       <x:c r="G43" s="18"/>
       <x:c r="H43" s="14"/>
       <x:c r="I43" s="19"/>
       <x:c r="J43" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K43" s="14" t="n">
-        <x:v>493.92</x:v>
+        <x:v>1301.93</x:v>
       </x:c>
       <x:c r="L43" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3037,31 +3121,31 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
+        <x:v>GASPAR COMERCIO DE EQUIPAMENTOS E UTENSILIOS LTDA</x:v>
       </x:c>
       <x:c r="B44" s="18" t="n">
-        <x:v>2182299</x:v>
+        <x:v>2199927</x:v>
       </x:c>
       <x:c r="C44" s="13" t="n">
-        <x:v>15276</x:v>
+        <x:v>15368</x:v>
       </x:c>
       <x:c r="D44" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E44" s="19" t="n">
-        <x:v>46223.747824074075</x:v>
+        <x:v>46226.76988425926</x:v>
       </x:c>
       <x:c r="F44" s="14" t="n">
-        <x:v>364.03</x:v>
+        <x:v>298.53</x:v>
       </x:c>
       <x:c r="G44" s="18"/>
       <x:c r="H44" s="14"/>
       <x:c r="I44" s="19"/>
       <x:c r="J44" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K44" s="14" t="n">
-        <x:v>364.03</x:v>
+        <x:v>298.53</x:v>
       </x:c>
       <x:c r="L44" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3069,31 +3153,31 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="13" t="str">
-        <x:v>VINICIUS BERNARDES TEIXEIRA</x:v>
+        <x:v>Fernanda Qualisol</x:v>
       </x:c>
       <x:c r="B45" s="18" t="n">
-        <x:v>2182658</x:v>
+        <x:v>2202021</x:v>
       </x:c>
       <x:c r="C45" s="13" t="n">
-        <x:v>15280</x:v>
+        <x:v>15376</x:v>
       </x:c>
       <x:c r="D45" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E45" s="19" t="n">
-        <x:v>46223.747824074075</x:v>
+        <x:v>46227.641180555554</x:v>
       </x:c>
       <x:c r="F45" s="14" t="n">
-        <x:v>112.77</x:v>
+        <x:v>474.57</x:v>
       </x:c>
       <x:c r="G45" s="18"/>
       <x:c r="H45" s="14"/>
       <x:c r="I45" s="19"/>
       <x:c r="J45" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K45" s="14" t="n">
-        <x:v>112.77</x:v>
+        <x:v>474.57</x:v>
       </x:c>
       <x:c r="L45" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3101,22 +3185,22 @@
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
+        <x:v>ACRILICOS BRASIL LTDA</x:v>
       </x:c>
       <x:c r="B46" s="18" t="n">
-        <x:v>2192401</x:v>
+        <x:v>2182262</x:v>
       </x:c>
       <x:c r="C46" s="13" t="n">
-        <x:v>15318</x:v>
+        <x:v>15275</x:v>
       </x:c>
       <x:c r="D46" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E46" s="19" t="n">
-        <x:v>46223.76341435185</x:v>
+        <x:v>46227.72767361111</x:v>
       </x:c>
       <x:c r="F46" s="14" t="n">
-        <x:v>561.43</x:v>
+        <x:v>2456.75</x:v>
       </x:c>
       <x:c r="G46" s="18"/>
       <x:c r="H46" s="14"/>
@@ -3125,7 +3209,7 @@
         <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K46" s="14" t="n">
-        <x:v>561.43</x:v>
+        <x:v>2456.75</x:v>
       </x:c>
       <x:c r="L46" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3133,22 +3217,22 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="13" t="str">
-        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
+        <x:v>BAUTECH INDUSTRIA E COMERCIO DE TINTAS LTDA</x:v>
       </x:c>
       <x:c r="B47" s="18" t="n">
-        <x:v>2183959</x:v>
+        <x:v>2183475</x:v>
       </x:c>
       <x:c r="C47" s="13" t="n">
-        <x:v>15290</x:v>
+        <x:v>15284</x:v>
       </x:c>
       <x:c r="D47" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E47" s="19" t="n">
-        <x:v>46223.782789351855</x:v>
+        <x:v>46227.737916666665</x:v>
       </x:c>
       <x:c r="F47" s="14" t="n">
-        <x:v>381.23</x:v>
+        <x:v>4382.37</x:v>
       </x:c>
       <x:c r="G47" s="18"/>
       <x:c r="H47" s="14"/>
@@ -3157,7 +3241,7 @@
         <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K47" s="14" t="n">
-        <x:v>381.23</x:v>
+        <x:v>4382.37</x:v>
       </x:c>
       <x:c r="L47" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3165,22 +3249,22 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="13" t="str">
-        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
+        <x:v>Camila</x:v>
       </x:c>
       <x:c r="B48" s="18" t="n">
-        <x:v>2182032</x:v>
+        <x:v>2190174</x:v>
       </x:c>
       <x:c r="C48" s="13" t="n">
-        <x:v>15172</x:v>
+        <x:v>15301</x:v>
       </x:c>
       <x:c r="D48" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E48" s="19" t="n">
-        <x:v>46223.784583333334</x:v>
+        <x:v>46227.737916666665</x:v>
       </x:c>
       <x:c r="F48" s="14" t="n">
-        <x:v>421.48</x:v>
+        <x:v>2365.26</x:v>
       </x:c>
       <x:c r="G48" s="18"/>
       <x:c r="H48" s="14"/>
@@ -3189,7 +3273,7 @@
         <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K48" s="14" t="n">
-        <x:v>2788.47</x:v>
+        <x:v>2365.26</x:v>
       </x:c>
       <x:c r="L48" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3197,31 +3281,31 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="13" t="str">
-        <x:v>Rosset Cia 2 Devoluções</x:v>
+        <x:v>Bprint Gráfica</x:v>
       </x:c>
       <x:c r="B49" s="18" t="n">
-        <x:v>2196879</x:v>
+        <x:v>2198394</x:v>
       </x:c>
       <x:c r="C49" s="13" t="n">
-        <x:v>15344</x:v>
+        <x:v>15356</x:v>
       </x:c>
       <x:c r="D49" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E49" s="19" t="n">
-        <x:v>46224.4844212963</x:v>
+        <x:v>46230.57780092592</x:v>
       </x:c>
       <x:c r="F49" s="14" t="n">
-        <x:v>927.98</x:v>
+        <x:v>1185.24</x:v>
       </x:c>
       <x:c r="G49" s="18"/>
       <x:c r="H49" s="14"/>
       <x:c r="I49" s="19"/>
       <x:c r="J49" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K49" s="14" t="n">
-        <x:v>927.98</x:v>
+        <x:v>1185.24</x:v>
       </x:c>
       <x:c r="L49" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3229,31 +3313,31 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="13" t="str">
-        <x:v>longo cadastro</x:v>
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
       </x:c>
       <x:c r="B50" s="18" t="n">
-        <x:v>2197779</x:v>
+        <x:v>2191606</x:v>
       </x:c>
       <x:c r="C50" s="13" t="n">
-        <x:v>15346</x:v>
+        <x:v>15308</x:v>
       </x:c>
       <x:c r="D50" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E50" s="19" t="n">
-        <x:v>46224.60364583333</x:v>
+        <x:v>46230.67396990741</x:v>
       </x:c>
       <x:c r="F50" s="14" t="n">
-        <x:v>2324.41</x:v>
+        <x:v>160.75</x:v>
       </x:c>
       <x:c r="G50" s="18"/>
       <x:c r="H50" s="14"/>
       <x:c r="I50" s="19"/>
       <x:c r="J50" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K50" s="14" t="n">
-        <x:v>2324.41</x:v>
+        <x:v>160.75</x:v>
       </x:c>
       <x:c r="L50" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3261,48 +3345,54 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="13" t="str">
-        <x:v>Roseli</x:v>
+        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
       </x:c>
       <x:c r="B51" s="18" t="n">
-        <x:v>2197853</x:v>
-      </x:c>
-      <x:c r="C51" s="13" t="str"/>
+        <x:v>2204541</x:v>
+      </x:c>
+      <x:c r="C51" s="13" t="n">
+        <x:v>15383</x:v>
+      </x:c>
       <x:c r="D51" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E51" s="19" t="n">
-        <x:v>46224.604467592595</x:v>
+        <x:v>46230.775509259256</x:v>
       </x:c>
       <x:c r="F51" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>463.98</x:v>
       </x:c>
       <x:c r="G51" s="18"/>
       <x:c r="H51" s="14"/>
       <x:c r="I51" s="19"/>
-      <x:c r="J51" s="13" t="str"/>
-      <x:c r="K51" s="14"/>
+      <x:c r="J51" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K51" s="14" t="n">
+        <x:v>463.98</x:v>
+      </x:c>
       <x:c r="L51" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="13" t="str">
-        <x:v>Itamonte l +Luz Iluminação l Vanessa C.</x:v>
+        <x:v>Carmaço - Fiori</x:v>
       </x:c>
       <x:c r="B52" s="18" t="n">
-        <x:v>2197933</x:v>
+        <x:v>2204551</x:v>
       </x:c>
       <x:c r="C52" s="13" t="n">
-        <x:v>15350</x:v>
+        <x:v>15384</x:v>
       </x:c>
       <x:c r="D52" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E52" s="19" t="n">
-        <x:v>46224.61032407408</x:v>
+        <x:v>46230.77912037037</x:v>
       </x:c>
       <x:c r="F52" s="14" t="n">
-        <x:v>244.8</x:v>
+        <x:v>401.75</x:v>
       </x:c>
       <x:c r="G52" s="18"/>
       <x:c r="H52" s="14"/>
@@ -3311,7 +3401,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K52" s="14" t="n">
-        <x:v>244.8</x:v>
+        <x:v>401.75</x:v>
       </x:c>
       <x:c r="L52" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3319,22 +3409,22 @@
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA</x:v>
+        <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B53" s="18" t="n">
-        <x:v>2198195</x:v>
+        <x:v>2204675</x:v>
       </x:c>
       <x:c r="C53" s="13" t="n">
-        <x:v>15349</x:v>
+        <x:v>15386</x:v>
       </x:c>
       <x:c r="D53" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E53" s="19" t="n">
-        <x:v>46224.73436342592</x:v>
+        <x:v>46230.79717592592</x:v>
       </x:c>
       <x:c r="F53" s="14" t="n">
-        <x:v>145.3</x:v>
+        <x:v>1290.83</x:v>
       </x:c>
       <x:c r="G53" s="18"/>
       <x:c r="H53" s="14"/>
@@ -3343,7 +3433,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K53" s="14" t="n">
-        <x:v>145.3</x:v>
+        <x:v>1290.83</x:v>
       </x:c>
       <x:c r="L53" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3351,22 +3441,22 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA</x:v>
+        <x:v>Qualidade Almad</x:v>
       </x:c>
       <x:c r="B54" s="18" t="n">
-        <x:v>2198196</x:v>
+        <x:v>2204714</x:v>
       </x:c>
       <x:c r="C54" s="13" t="n">
-        <x:v>15353</x:v>
+        <x:v>15387</x:v>
       </x:c>
       <x:c r="D54" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E54" s="19" t="n">
-        <x:v>46224.73789351852</x:v>
+        <x:v>46231.45103009259</x:v>
       </x:c>
       <x:c r="F54" s="14" t="n">
-        <x:v>142.51</x:v>
+        <x:v>2370.92</x:v>
       </x:c>
       <x:c r="G54" s="18"/>
       <x:c r="H54" s="14"/>
@@ -3375,7 +3465,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K54" s="14" t="n">
-        <x:v>142.51</x:v>
+        <x:v>2370.92</x:v>
       </x:c>
       <x:c r="L54" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3383,100 +3473,118 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="13" t="str">
-        <x:v>Rogerio</x:v>
+        <x:v>Transporte Bautech</x:v>
       </x:c>
       <x:c r="B55" s="18" t="n">
-        <x:v>2198226</x:v>
-      </x:c>
-      <x:c r="C55" s="13" t="str"/>
+        <x:v>2205200</x:v>
+      </x:c>
+      <x:c r="C55" s="13" t="n">
+        <x:v>15388</x:v>
+      </x:c>
       <x:c r="D55" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E55" s="19" t="n">
-        <x:v>46224.760879629626</x:v>
+        <x:v>46231.503171296295</x:v>
       </x:c>
       <x:c r="F55" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>505.68</x:v>
       </x:c>
       <x:c r="G55" s="18"/>
       <x:c r="H55" s="14"/>
       <x:c r="I55" s="19"/>
-      <x:c r="J55" s="13" t="str"/>
-      <x:c r="K55" s="14"/>
+      <x:c r="J55" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K55" s="14" t="n">
+        <x:v>505.68</x:v>
+      </x:c>
       <x:c r="L55" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="13" t="str">
-        <x:v>Danval ADM</x:v>
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
       </x:c>
       <x:c r="B56" s="18" t="n">
-        <x:v>2198229</x:v>
-      </x:c>
-      <x:c r="C56" s="13" t="str"/>
+        <x:v>2205354</x:v>
+      </x:c>
+      <x:c r="C56" s="13" t="n">
+        <x:v>15394</x:v>
+      </x:c>
       <x:c r="D56" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E56" s="19" t="n">
-        <x:v>46224.760879629626</x:v>
+        <x:v>46231.60502314815</x:v>
       </x:c>
       <x:c r="F56" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>173.06</x:v>
       </x:c>
       <x:c r="G56" s="18"/>
       <x:c r="H56" s="14"/>
       <x:c r="I56" s="19"/>
-      <x:c r="J56" s="13" t="str"/>
-      <x:c r="K56" s="14"/>
+      <x:c r="J56" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K56" s="14" t="n">
+        <x:v>173.06</x:v>
+      </x:c>
       <x:c r="L56" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="13" t="str">
-        <x:v>Compras - Insertec Fornos e Refratários</x:v>
+        <x:v>Metal Max</x:v>
       </x:c>
       <x:c r="B57" s="18" t="n">
-        <x:v>2194633</x:v>
-      </x:c>
-      <x:c r="C57" s="13" t="str"/>
+        <x:v>2205212</x:v>
+      </x:c>
+      <x:c r="C57" s="13" t="n">
+        <x:v>15392</x:v>
+      </x:c>
       <x:c r="D57" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E57" s="19" t="n">
-        <x:v>46224.77175925926</x:v>
+        <x:v>46231.68457175926</x:v>
       </x:c>
       <x:c r="F57" s="14" t="n">
-        <x:v>311.03</x:v>
+        <x:v>215.53</x:v>
       </x:c>
       <x:c r="G57" s="18"/>
       <x:c r="H57" s="14"/>
       <x:c r="I57" s="19"/>
-      <x:c r="J57" s="13" t="str"/>
-      <x:c r="K57" s="14"/>
+      <x:c r="J57" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K57" s="14" t="n">
+        <x:v>215.53</x:v>
+      </x:c>
       <x:c r="L57" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="13" t="str">
-        <x:v>Fernanda Qualisol</x:v>
+        <x:v>Eder Fazzi</x:v>
       </x:c>
       <x:c r="B58" s="18" t="n">
-        <x:v>2198771</x:v>
+        <x:v>2205493</x:v>
       </x:c>
       <x:c r="C58" s="13" t="n">
-        <x:v>15357</x:v>
+        <x:v>15395</x:v>
       </x:c>
       <x:c r="D58" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E58" s="19" t="n">
-        <x:v>46225.53065972222</x:v>
+        <x:v>46231.69190972222</x:v>
       </x:c>
       <x:c r="F58" s="14" t="n">
-        <x:v>239.17</x:v>
+        <x:v>1419.63</x:v>
       </x:c>
       <x:c r="G58" s="18"/>
       <x:c r="H58" s="14"/>
@@ -3485,7 +3593,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K58" s="14" t="n">
-        <x:v>239.17</x:v>
+        <x:v>1419.63</x:v>
       </x:c>
       <x:c r="L58" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3493,57 +3601,63 @@
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="13" t="str">
-        <x:v>Nobrecar -Alex</x:v>
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
       </x:c>
       <x:c r="B59" s="18" t="n">
-        <x:v>2199033</x:v>
-      </x:c>
-      <x:c r="C59" s="13" t="str"/>
+        <x:v>2205218</x:v>
+      </x:c>
+      <x:c r="C59" s="13" t="n">
+        <x:v>15390</x:v>
+      </x:c>
       <x:c r="D59" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E59" s="19" t="n">
-        <x:v>46225.70516203704</x:v>
+        <x:v>46231.71363425926</x:v>
       </x:c>
       <x:c r="F59" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>169.45</x:v>
       </x:c>
       <x:c r="G59" s="18"/>
       <x:c r="H59" s="14"/>
       <x:c r="I59" s="19"/>
-      <x:c r="J59" s="13" t="str"/>
-      <x:c r="K59" s="14"/>
+      <x:c r="J59" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K59" s="14" t="n">
+        <x:v>169.45</x:v>
+      </x:c>
       <x:c r="L59" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="13" t="str">
-        <x:v>Fernanda Qualisol</x:v>
+        <x:v>Osni - Molina Freios</x:v>
       </x:c>
       <x:c r="B60" s="18" t="n">
-        <x:v>2199721</x:v>
+        <x:v>2201892</x:v>
       </x:c>
       <x:c r="C60" s="13" t="n">
-        <x:v>15364</x:v>
+        <x:v>15373</x:v>
       </x:c>
       <x:c r="D60" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E60" s="19" t="n">
-        <x:v>46226.506423611114</x:v>
+        <x:v>46231.74150462963</x:v>
       </x:c>
       <x:c r="F60" s="14" t="n">
-        <x:v>283.27</x:v>
+        <x:v>155.98</x:v>
       </x:c>
       <x:c r="G60" s="18"/>
       <x:c r="H60" s="14"/>
       <x:c r="I60" s="19"/>
       <x:c r="J60" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K60" s="14" t="n">
-        <x:v>283.27</x:v>
+        <x:v>155.98</x:v>
       </x:c>
       <x:c r="L60" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3551,22 +3665,22 @@
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA</x:v>
+        <x:v>Thomas Estoque R Imper</x:v>
       </x:c>
       <x:c r="B61" s="18" t="n">
-        <x:v>2199791</x:v>
+        <x:v>2205687</x:v>
       </x:c>
       <x:c r="C61" s="13" t="n">
-        <x:v>15365</x:v>
+        <x:v>15397</x:v>
       </x:c>
       <x:c r="D61" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E61" s="19" t="n">
-        <x:v>46226.51068287037</x:v>
+        <x:v>46231.78642361111</x:v>
       </x:c>
       <x:c r="F61" s="14" t="n">
-        <x:v>125.99</x:v>
+        <x:v>1806.4</x:v>
       </x:c>
       <x:c r="G61" s="18"/>
       <x:c r="H61" s="14"/>
@@ -3575,7 +3689,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K61" s="14" t="n">
-        <x:v>125.99</x:v>
+        <x:v>1806.4</x:v>
       </x:c>
       <x:c r="L61" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3583,100 +3697,118 @@
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="13" t="str">
-        <x:v>IKTEC COMERCIO DE PROD PARA TRAT DE SUPERFICIE LTDA</x:v>
+        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
       </x:c>
       <x:c r="B62" s="18" t="n">
-        <x:v>2199802</x:v>
-      </x:c>
-      <x:c r="C62" s="13" t="str"/>
+        <x:v>2206185</x:v>
+      </x:c>
+      <x:c r="C62" s="13" t="n">
+        <x:v>15401</x:v>
+      </x:c>
       <x:c r="D62" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E62" s="19" t="n">
-        <x:v>46226.51582175926</x:v>
+        <x:v>46232.56662037037</x:v>
       </x:c>
       <x:c r="F62" s="14" t="n">
-        <x:v>158.2</x:v>
+        <x:v>599.35</x:v>
       </x:c>
       <x:c r="G62" s="18"/>
       <x:c r="H62" s="14"/>
       <x:c r="I62" s="19"/>
-      <x:c r="J62" s="13" t="str"/>
-      <x:c r="K62" s="14"/>
+      <x:c r="J62" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K62" s="14" t="n">
+        <x:v>599.35</x:v>
+      </x:c>
       <x:c r="L62" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="13" t="str">
-        <x:v>🙋🏻‍♀️</x:v>
+        <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B63" s="18" t="n">
-        <x:v>2199765</x:v>
-      </x:c>
-      <x:c r="C63" s="13" t="str"/>
+        <x:v>2205674</x:v>
+      </x:c>
+      <x:c r="C63" s="13" t="n">
+        <x:v>15402</x:v>
+      </x:c>
       <x:c r="D63" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E63" s="19" t="n">
-        <x:v>46226.544270833336</x:v>
+        <x:v>46232.57876157408</x:v>
       </x:c>
       <x:c r="F63" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>2173.95</x:v>
       </x:c>
       <x:c r="G63" s="18"/>
       <x:c r="H63" s="14"/>
       <x:c r="I63" s="19"/>
-      <x:c r="J63" s="13" t="str"/>
-      <x:c r="K63" s="14"/>
+      <x:c r="J63" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K63" s="14" t="n">
+        <x:v>2173.95</x:v>
+      </x:c>
       <x:c r="L63" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="13" t="str">
-        <x:v>Pamella</x:v>
+        <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B64" s="18" t="n">
-        <x:v>2199886</x:v>
-      </x:c>
-      <x:c r="C64" s="13" t="str"/>
+        <x:v>2206284</x:v>
+      </x:c>
+      <x:c r="C64" s="13" t="n">
+        <x:v>15405</x:v>
+      </x:c>
       <x:c r="D64" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E64" s="19" t="n">
-        <x:v>46226.57403935185</x:v>
+        <x:v>46232.59909722222</x:v>
       </x:c>
       <x:c r="F64" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>568.61</x:v>
       </x:c>
       <x:c r="G64" s="18"/>
       <x:c r="H64" s="14"/>
       <x:c r="I64" s="19"/>
-      <x:c r="J64" s="13" t="str"/>
-      <x:c r="K64" s="14"/>
+      <x:c r="J64" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K64" s="14" t="n">
+        <x:v>568.61</x:v>
+      </x:c>
       <x:c r="L64" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="13" t="str">
-        <x:v>BAUTECH INDUSTRIA E COMERCIO DE TINTAS LTDA</x:v>
+        <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B65" s="18" t="n">
-        <x:v>2199976</x:v>
+        <x:v>2206293</x:v>
       </x:c>
       <x:c r="C65" s="13" t="n">
-        <x:v>15369</x:v>
+        <x:v>15406</x:v>
       </x:c>
       <x:c r="D65" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E65" s="19" t="n">
-        <x:v>46226.614375</x:v>
+        <x:v>46232.60854166667</x:v>
       </x:c>
       <x:c r="F65" s="14" t="n">
-        <x:v>1301.93</x:v>
+        <x:v>454.22</x:v>
       </x:c>
       <x:c r="G65" s="18"/>
       <x:c r="H65" s="14"/>
@@ -3685,7 +3817,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K65" s="14" t="n">
-        <x:v>1301.93</x:v>
+        <x:v>454.22</x:v>
       </x:c>
       <x:c r="L65" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3693,48 +3825,54 @@
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="13" t="str">
-        <x:v>ML PAPÉIS</x:v>
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
       </x:c>
       <x:c r="B66" s="18" t="n">
-        <x:v>2200167</x:v>
-      </x:c>
-      <x:c r="C66" s="13" t="str"/>
+        <x:v>2206603</x:v>
+      </x:c>
+      <x:c r="C66" s="13" t="n">
+        <x:v>15408</x:v>
+      </x:c>
       <x:c r="D66" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E66" s="19" t="n">
-        <x:v>46226.76613425926</x:v>
+        <x:v>46232.799525462964</x:v>
       </x:c>
       <x:c r="F66" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>124.44</x:v>
       </x:c>
       <x:c r="G66" s="18"/>
       <x:c r="H66" s="14"/>
       <x:c r="I66" s="19"/>
-      <x:c r="J66" s="13" t="str"/>
-      <x:c r="K66" s="14"/>
+      <x:c r="J66" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K66" s="14" t="n">
+        <x:v>124.44</x:v>
+      </x:c>
       <x:c r="L66" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="13" t="str">
-        <x:v>GASPAR COMERCIO DE EQUIPAMENTOS E UTENSILIOS LTDA</x:v>
+        <x:v>Vinilak Tintas Especiais</x:v>
       </x:c>
       <x:c r="B67" s="18" t="n">
-        <x:v>2199927</x:v>
+        <x:v>2207138</x:v>
       </x:c>
       <x:c r="C67" s="13" t="n">
-        <x:v>15368</x:v>
+        <x:v>15412</x:v>
       </x:c>
       <x:c r="D67" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E67" s="19" t="n">
-        <x:v>46226.76988425926</x:v>
+        <x:v>46233.56369212963</x:v>
       </x:c>
       <x:c r="F67" s="14" t="n">
-        <x:v>298.53</x:v>
+        <x:v>503.59</x:v>
       </x:c>
       <x:c r="G67" s="18"/>
       <x:c r="H67" s="14"/>
@@ -3743,7 +3881,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K67" s="14" t="n">
-        <x:v>298.53</x:v>
+        <x:v>503.59</x:v>
       </x:c>
       <x:c r="L67" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3751,74 +3889,86 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="13" t="str">
-        <x:v>Alcimara Carneiro</x:v>
+        <x:v>João Pedro | Bprint Gráfica</x:v>
       </x:c>
       <x:c r="B68" s="18" t="n">
-        <x:v>2200262</x:v>
-      </x:c>
-      <x:c r="C68" s="13" t="str"/>
+        <x:v>2207378</x:v>
+      </x:c>
+      <x:c r="C68" s="13" t="n">
+        <x:v>15414</x:v>
+      </x:c>
       <x:c r="D68" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E68" s="19" t="n">
-        <x:v>46227.46097222222</x:v>
+        <x:v>46233.572060185186</x:v>
       </x:c>
       <x:c r="F68" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>430.25</x:v>
       </x:c>
       <x:c r="G68" s="18"/>
       <x:c r="H68" s="14"/>
       <x:c r="I68" s="19"/>
-      <x:c r="J68" s="13" t="str"/>
-      <x:c r="K68" s="14"/>
+      <x:c r="J68" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K68" s="14" t="n">
+        <x:v>430.25</x:v>
+      </x:c>
       <x:c r="L68" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="13" t="str">
-        <x:v>Alcimara Carneiro</x:v>
+        <x:v>Carmaço - Fiori</x:v>
       </x:c>
       <x:c r="B69" s="18" t="n">
-        <x:v>2200261</x:v>
-      </x:c>
-      <x:c r="C69" s="13" t="str"/>
+        <x:v>2207562</x:v>
+      </x:c>
+      <x:c r="C69" s="13" t="n">
+        <x:v>15417</x:v>
+      </x:c>
       <x:c r="D69" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E69" s="19" t="n">
-        <x:v>46227.46260416666</x:v>
+        <x:v>46233.67563657407</x:v>
       </x:c>
       <x:c r="F69" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>390.31</x:v>
       </x:c>
       <x:c r="G69" s="18"/>
       <x:c r="H69" s="14"/>
       <x:c r="I69" s="19"/>
-      <x:c r="J69" s="13" t="str"/>
-      <x:c r="K69" s="14"/>
+      <x:c r="J69" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K69" s="14" t="n">
+        <x:v>390.31</x:v>
+      </x:c>
       <x:c r="L69" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="13" t="str">
-        <x:v>Fernanda Qualisol</x:v>
+        <x:v>Queren Cyrino</x:v>
       </x:c>
       <x:c r="B70" s="18" t="n">
-        <x:v>2202021</x:v>
+        <x:v>2207563</x:v>
       </x:c>
       <x:c r="C70" s="13" t="n">
-        <x:v>15376</x:v>
+        <x:v>15419</x:v>
       </x:c>
       <x:c r="D70" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E70" s="19" t="n">
-        <x:v>46227.641180555554</x:v>
+        <x:v>46233.69023148148</x:v>
       </x:c>
       <x:c r="F70" s="14" t="n">
-        <x:v>474.57</x:v>
+        <x:v>1168.34</x:v>
       </x:c>
       <x:c r="G70" s="18"/>
       <x:c r="H70" s="14"/>
@@ -3827,7 +3977,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K70" s="14" t="n">
-        <x:v>474.57</x:v>
+        <x:v>1168.34</x:v>
       </x:c>
       <x:c r="L70" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3835,54 +3985,48 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="13" t="str">
-        <x:v>ACRILICOS BRASIL LTDA</x:v>
+        <x:v>WOOD COLOR TINTAS</x:v>
       </x:c>
       <x:c r="B71" s="18" t="n">
-        <x:v>2182262</x:v>
-      </x:c>
-      <x:c r="C71" s="13" t="n">
-        <x:v>15275</x:v>
-      </x:c>
+        <x:v>2207637</x:v>
+      </x:c>
+      <x:c r="C71" s="13" t="str"/>
       <x:c r="D71" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E71" s="19" t="n">
-        <x:v>46227.72767361111</x:v>
+        <x:v>46233.700266203705</x:v>
       </x:c>
       <x:c r="F71" s="14" t="n">
-        <x:v>2456.75</x:v>
+        <x:v>404.88</x:v>
       </x:c>
       <x:c r="G71" s="18"/>
       <x:c r="H71" s="14"/>
       <x:c r="I71" s="19"/>
-      <x:c r="J71" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K71" s="14" t="n">
-        <x:v>2456.75</x:v>
-      </x:c>
+      <x:c r="J71" s="13" t="str"/>
+      <x:c r="K71" s="14"/>
       <x:c r="L71" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="13" t="str">
-        <x:v>BAUTECH INDUSTRIA E COMERCIO DE TINTAS LTDA</x:v>
+        <x:v>Juciliana</x:v>
       </x:c>
       <x:c r="B72" s="18" t="n">
-        <x:v>2183475</x:v>
+        <x:v>2206455</x:v>
       </x:c>
       <x:c r="C72" s="13" t="n">
-        <x:v>15284</x:v>
+        <x:v>15407</x:v>
       </x:c>
       <x:c r="D72" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E72" s="19" t="n">
-        <x:v>46227.737916666665</x:v>
+        <x:v>46233.70322916667</x:v>
       </x:c>
       <x:c r="F72" s="14" t="n">
-        <x:v>4382.37</x:v>
+        <x:v>251.25</x:v>
       </x:c>
       <x:c r="G72" s="18"/>
       <x:c r="H72" s="14"/>
@@ -3891,7 +4035,7 @@
         <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K72" s="14" t="n">
-        <x:v>4382.37</x:v>
+        <x:v>251.25</x:v>
       </x:c>
       <x:c r="L72" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3899,31 +4043,31 @@
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="13" t="str">
-        <x:v>Camila</x:v>
+        <x:v>FRANCHI NORTE DISTRIBUICAO LTDA</x:v>
       </x:c>
       <x:c r="B73" s="18" t="n">
-        <x:v>2190174</x:v>
+        <x:v>2205563</x:v>
       </x:c>
       <x:c r="C73" s="13" t="n">
-        <x:v>15301</x:v>
+        <x:v>15396</x:v>
       </x:c>
       <x:c r="D73" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E73" s="19" t="n">
-        <x:v>46227.737916666665</x:v>
+        <x:v>46233.765810185185</x:v>
       </x:c>
       <x:c r="F73" s="14" t="n">
-        <x:v>2365.26</x:v>
+        <x:v>250.89</x:v>
       </x:c>
       <x:c r="G73" s="18"/>
       <x:c r="H73" s="14"/>
       <x:c r="I73" s="19"/>
       <x:c r="J73" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K73" s="14" t="n">
-        <x:v>2365.26</x:v>
+        <x:v>250.89</x:v>
       </x:c>
       <x:c r="L73" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3931,31 +4075,31 @@
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="13" t="str">
-        <x:v>Bprint Gráfica</x:v>
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
       </x:c>
       <x:c r="B74" s="18" t="n">
-        <x:v>2198394</x:v>
+        <x:v>2208212</x:v>
       </x:c>
       <x:c r="C74" s="13" t="n">
-        <x:v>15356</x:v>
+        <x:v>15421</x:v>
       </x:c>
       <x:c r="D74" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E74" s="19" t="n">
-        <x:v>46230.57780092592</x:v>
+        <x:v>46234.513715277775</x:v>
       </x:c>
       <x:c r="F74" s="14" t="n">
-        <x:v>1185.24</x:v>
+        <x:v>142.51</x:v>
       </x:c>
       <x:c r="G74" s="18"/>
       <x:c r="H74" s="14"/>
       <x:c r="I74" s="19"/>
       <x:c r="J74" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K74" s="14" t="n">
-        <x:v>1185.24</x:v>
+        <x:v>142.51</x:v>
       </x:c>
       <x:c r="L74" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3963,31 +4107,31 @@
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
+        <x:v>Elisete Henck</x:v>
       </x:c>
       <x:c r="B75" s="18" t="n">
-        <x:v>2191606</x:v>
+        <x:v>2208349</x:v>
       </x:c>
       <x:c r="C75" s="13" t="n">
-        <x:v>15308</x:v>
+        <x:v>15423</x:v>
       </x:c>
       <x:c r="D75" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E75" s="19" t="n">
-        <x:v>46230.67396990741</x:v>
+        <x:v>46234.616793981484</x:v>
       </x:c>
       <x:c r="F75" s="14" t="n">
-        <x:v>160.75</x:v>
+        <x:v>107.37</x:v>
       </x:c>
       <x:c r="G75" s="18"/>
       <x:c r="H75" s="14"/>
       <x:c r="I75" s="19"/>
       <x:c r="J75" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K75" s="14" t="n">
-        <x:v>160.75</x:v>
+        <x:v>107.37</x:v>
       </x:c>
       <x:c r="L75" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3995,31 +4139,31 @@
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="13" t="str">
-        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
+        <x:v>Logistica</x:v>
       </x:c>
       <x:c r="B76" s="18" t="n">
-        <x:v>2204541</x:v>
+        <x:v>2191659</x:v>
       </x:c>
       <x:c r="C76" s="13" t="n">
-        <x:v>15383</x:v>
+        <x:v>15317</x:v>
       </x:c>
       <x:c r="D76" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E76" s="19" t="n">
-        <x:v>46230.775509259256</x:v>
+        <x:v>46234.67115740741</x:v>
       </x:c>
       <x:c r="F76" s="14" t="n">
-        <x:v>463.98</x:v>
+        <x:v>276.1</x:v>
       </x:c>
       <x:c r="G76" s="18"/>
       <x:c r="H76" s="14"/>
       <x:c r="I76" s="19"/>
       <x:c r="J76" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K76" s="14" t="n">
-        <x:v>463.98</x:v>
+        <x:v>276.1</x:v>
       </x:c>
       <x:c r="L76" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4027,31 +4171,31 @@
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="13" t="str">
-        <x:v>Carmaço - Fiori</x:v>
+        <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B77" s="18" t="n">
-        <x:v>2204551</x:v>
+        <x:v>2192512</x:v>
       </x:c>
       <x:c r="C77" s="13" t="n">
-        <x:v>15384</x:v>
+        <x:v>15319</x:v>
       </x:c>
       <x:c r="D77" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E77" s="19" t="n">
-        <x:v>46230.77912037037</x:v>
+        <x:v>46234.67115740741</x:v>
       </x:c>
       <x:c r="F77" s="14" t="n">
-        <x:v>401.75</x:v>
+        <x:v>630.36</x:v>
       </x:c>
       <x:c r="G77" s="18"/>
       <x:c r="H77" s="14"/>
       <x:c r="I77" s="19"/>
       <x:c r="J77" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K77" s="14" t="n">
-        <x:v>401.75</x:v>
+        <x:v>630.36</x:v>
       </x:c>
       <x:c r="L77" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4059,31 +4203,31 @@
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
+        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
       </x:c>
       <x:c r="B78" s="18" t="n">
-        <x:v>2204675</x:v>
+        <x:v>2193158</x:v>
       </x:c>
       <x:c r="C78" s="13" t="n">
-        <x:v>15386</x:v>
+        <x:v>15321</x:v>
       </x:c>
       <x:c r="D78" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E78" s="19" t="n">
-        <x:v>46230.79717592592</x:v>
+        <x:v>46234.67115740741</x:v>
       </x:c>
       <x:c r="F78" s="14" t="n">
-        <x:v>1290.83</x:v>
+        <x:v>226.75</x:v>
       </x:c>
       <x:c r="G78" s="18"/>
       <x:c r="H78" s="14"/>
       <x:c r="I78" s="19"/>
       <x:c r="J78" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K78" s="14" t="n">
-        <x:v>1290.83</x:v>
+        <x:v>226.75</x:v>
       </x:c>
       <x:c r="L78" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4091,31 +4235,31 @@
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="13" t="str">
-        <x:v>Qualidade Almad</x:v>
+        <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B79" s="18" t="n">
-        <x:v>2204714</x:v>
+        <x:v>2193214</x:v>
       </x:c>
       <x:c r="C79" s="13" t="n">
-        <x:v>15387</x:v>
+        <x:v>15323</x:v>
       </x:c>
       <x:c r="D79" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E79" s="19" t="n">
-        <x:v>46231.45103009259</x:v>
+        <x:v>46234.67115740741</x:v>
       </x:c>
       <x:c r="F79" s="14" t="n">
-        <x:v>2370.92</x:v>
+        <x:v>222.19</x:v>
       </x:c>
       <x:c r="G79" s="18"/>
       <x:c r="H79" s="14"/>
       <x:c r="I79" s="19"/>
       <x:c r="J79" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K79" s="14" t="n">
-        <x:v>2370.92</x:v>
+        <x:v>222.19</x:v>
       </x:c>
       <x:c r="L79" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4123,31 +4267,31 @@
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="13" t="str">
-        <x:v>Transporte Bautech</x:v>
+        <x:v>LC Plásticos</x:v>
       </x:c>
       <x:c r="B80" s="18" t="n">
-        <x:v>2205200</x:v>
+        <x:v>2193641</x:v>
       </x:c>
       <x:c r="C80" s="13" t="n">
-        <x:v>15388</x:v>
+        <x:v>15331</x:v>
       </x:c>
       <x:c r="D80" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E80" s="19" t="n">
-        <x:v>46231.503171296295</x:v>
+        <x:v>46234.67115740741</x:v>
       </x:c>
       <x:c r="F80" s="14" t="n">
-        <x:v>505.68</x:v>
+        <x:v>781.33</x:v>
       </x:c>
       <x:c r="G80" s="18"/>
       <x:c r="H80" s="14"/>
       <x:c r="I80" s="19"/>
       <x:c r="J80" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K80" s="14" t="n">
-        <x:v>505.68</x:v>
+        <x:v>781.33</x:v>
       </x:c>
       <x:c r="L80" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4155,57 +4299,63 @@
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="13" t="str">
-        <x:v>Barão</x:v>
+        <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B81" s="18" t="n">
-        <x:v>2205201</x:v>
-      </x:c>
-      <x:c r="C81" s="13" t="str"/>
+        <x:v>2194620</x:v>
+      </x:c>
+      <x:c r="C81" s="13" t="n">
+        <x:v>15335</x:v>
+      </x:c>
       <x:c r="D81" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E81" s="19" t="n">
-        <x:v>46231.511400462965</x:v>
+        <x:v>46234.67115740741</x:v>
       </x:c>
       <x:c r="F81" s="14" t="n">
-        <x:v>0</x:v>
+        <x:v>437.67</x:v>
       </x:c>
       <x:c r="G81" s="18"/>
       <x:c r="H81" s="14"/>
       <x:c r="I81" s="19"/>
-      <x:c r="J81" s="13" t="str"/>
-      <x:c r="K81" s="14"/>
+      <x:c r="J81" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K81" s="14" t="n">
+        <x:v>437.67</x:v>
+      </x:c>
       <x:c r="L81" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
+        <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B82" s="18" t="n">
-        <x:v>2205354</x:v>
+        <x:v>2194619</x:v>
       </x:c>
       <x:c r="C82" s="13" t="n">
-        <x:v>15394</x:v>
+        <x:v>15340</x:v>
       </x:c>
       <x:c r="D82" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E82" s="19" t="n">
-        <x:v>46231.60502314815</x:v>
+        <x:v>46234.681550925925</x:v>
       </x:c>
       <x:c r="F82" s="14" t="n">
-        <x:v>173.06</x:v>
+        <x:v>434.19</x:v>
       </x:c>
       <x:c r="G82" s="18"/>
       <x:c r="H82" s="14"/>
       <x:c r="I82" s="19"/>
       <x:c r="J82" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K82" s="14" t="n">
-        <x:v>173.06</x:v>
+        <x:v>434.19</x:v>
       </x:c>
       <x:c r="L82" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4213,22 +4363,22 @@
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="13" t="str">
-        <x:v>Metal Max</x:v>
+        <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B83" s="18" t="n">
-        <x:v>2205212</x:v>
+        <x:v>2208468</x:v>
       </x:c>
       <x:c r="C83" s="13" t="n">
-        <x:v>15392</x:v>
+        <x:v>15424</x:v>
       </x:c>
       <x:c r="D83" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E83" s="19" t="n">
-        <x:v>46231.68457175926</x:v>
+        <x:v>46234.737546296295</x:v>
       </x:c>
       <x:c r="F83" s="14" t="n">
-        <x:v>215.53</x:v>
+        <x:v>310.75</x:v>
       </x:c>
       <x:c r="G83" s="18"/>
       <x:c r="H83" s="14"/>
@@ -4237,7 +4387,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K83" s="14" t="n">
-        <x:v>215.53</x:v>
+        <x:v>310.75</x:v>
       </x:c>
       <x:c r="L83" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4245,22 +4395,22 @@
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="13" t="str">
-        <x:v>Eder Fazzi</x:v>
+        <x:v>Viviane Pinheiro</x:v>
       </x:c>
       <x:c r="B84" s="18" t="n">
-        <x:v>2205493</x:v>
+        <x:v>2208572</x:v>
       </x:c>
       <x:c r="C84" s="13" t="n">
-        <x:v>15395</x:v>
+        <x:v>15425</x:v>
       </x:c>
       <x:c r="D84" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E84" s="19" t="n">
-        <x:v>46231.69190972222</x:v>
+        <x:v>46234.7840625</x:v>
       </x:c>
       <x:c r="F84" s="14" t="n">
-        <x:v>1419.63</x:v>
+        <x:v>770.68</x:v>
       </x:c>
       <x:c r="G84" s="18"/>
       <x:c r="H84" s="14"/>
@@ -4269,1206 +4419,10 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K84" s="14" t="n">
-        <x:v>1419.63</x:v>
+        <x:v>770.68</x:v>
       </x:c>
       <x:c r="L84" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="85">
-      <x:c r="A85" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
-      </x:c>
-      <x:c r="B85" s="18" t="n">
-        <x:v>2205218</x:v>
-      </x:c>
-      <x:c r="C85" s="13" t="n">
-        <x:v>15390</x:v>
-      </x:c>
-      <x:c r="D85" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E85" s="19" t="n">
-        <x:v>46231.71363425926</x:v>
-      </x:c>
-      <x:c r="F85" s="14" t="n">
-        <x:v>169.45</x:v>
-      </x:c>
-      <x:c r="G85" s="18"/>
-      <x:c r="H85" s="14"/>
-      <x:c r="I85" s="19"/>
-      <x:c r="J85" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K85" s="14" t="n">
-        <x:v>169.45</x:v>
-      </x:c>
-      <x:c r="L85" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="86">
-      <x:c r="A86" s="13" t="str">
-        <x:v>Pamella</x:v>
-      </x:c>
-      <x:c r="B86" s="18" t="n">
-        <x:v>2205564</x:v>
-      </x:c>
-      <x:c r="C86" s="13" t="str"/>
-      <x:c r="D86" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E86" s="19" t="n">
-        <x:v>46231.73575231482</x:v>
-      </x:c>
-      <x:c r="F86" s="14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G86" s="18"/>
-      <x:c r="H86" s="14"/>
-      <x:c r="I86" s="19"/>
-      <x:c r="J86" s="13" t="str"/>
-      <x:c r="K86" s="14"/>
-      <x:c r="L86" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="87">
-      <x:c r="A87" s="13" t="str">
-        <x:v>Osni - Molina Freios</x:v>
-      </x:c>
-      <x:c r="B87" s="18" t="n">
-        <x:v>2201892</x:v>
-      </x:c>
-      <x:c r="C87" s="13" t="n">
-        <x:v>15373</x:v>
-      </x:c>
-      <x:c r="D87" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E87" s="19" t="n">
-        <x:v>46231.74150462963</x:v>
-      </x:c>
-      <x:c r="F87" s="14" t="n">
-        <x:v>155.98</x:v>
-      </x:c>
-      <x:c r="G87" s="18"/>
-      <x:c r="H87" s="14"/>
-      <x:c r="I87" s="19"/>
-      <x:c r="J87" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K87" s="14" t="n">
-        <x:v>155.98</x:v>
-      </x:c>
-      <x:c r="L87" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="88">
-      <x:c r="A88" s="13" t="str">
-        <x:v>Thomas Estoque R Imper</x:v>
-      </x:c>
-      <x:c r="B88" s="18" t="n">
-        <x:v>2205687</x:v>
-      </x:c>
-      <x:c r="C88" s="13" t="n">
-        <x:v>15397</x:v>
-      </x:c>
-      <x:c r="D88" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E88" s="19" t="n">
-        <x:v>46231.78642361111</x:v>
-      </x:c>
-      <x:c r="F88" s="14" t="n">
-        <x:v>1806.4</x:v>
-      </x:c>
-      <x:c r="G88" s="18"/>
-      <x:c r="H88" s="14"/>
-      <x:c r="I88" s="19"/>
-      <x:c r="J88" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K88" s="14" t="n">
-        <x:v>1806.4</x:v>
-      </x:c>
-      <x:c r="L88" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="89">
-      <x:c r="A89" s="13" t="str">
-        <x:v>Letícia Jovial 🍀</x:v>
-      </x:c>
-      <x:c r="B89" s="18" t="n">
-        <x:v>2205699</x:v>
-      </x:c>
-      <x:c r="C89" s="13" t="str"/>
-      <x:c r="D89" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E89" s="19" t="n">
-        <x:v>46232.51677083333</x:v>
-      </x:c>
-      <x:c r="F89" s="14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G89" s="18"/>
-      <x:c r="H89" s="14"/>
-      <x:c r="I89" s="19"/>
-      <x:c r="J89" s="13" t="str"/>
-      <x:c r="K89" s="14"/>
-      <x:c r="L89" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="90">
-      <x:c r="A90" s="13" t="str">
-        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
-      </x:c>
-      <x:c r="B90" s="18" t="n">
-        <x:v>2206185</x:v>
-      </x:c>
-      <x:c r="C90" s="13" t="n">
-        <x:v>15401</x:v>
-      </x:c>
-      <x:c r="D90" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E90" s="19" t="n">
-        <x:v>46232.56662037037</x:v>
-      </x:c>
-      <x:c r="F90" s="14" t="n">
-        <x:v>599.35</x:v>
-      </x:c>
-      <x:c r="G90" s="18"/>
-      <x:c r="H90" s="14"/>
-      <x:c r="I90" s="19"/>
-      <x:c r="J90" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K90" s="14" t="n">
-        <x:v>599.35</x:v>
-      </x:c>
-      <x:c r="L90" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="91">
-      <x:c r="A91" s="13" t="str">
-        <x:v>DNM Limp Witor</x:v>
-      </x:c>
-      <x:c r="B91" s="18" t="n">
-        <x:v>2206237</x:v>
-      </x:c>
-      <x:c r="C91" s="13" t="str"/>
-      <x:c r="D91" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E91" s="19" t="n">
-        <x:v>46232.568773148145</x:v>
-      </x:c>
-      <x:c r="F91" s="14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G91" s="18"/>
-      <x:c r="H91" s="14"/>
-      <x:c r="I91" s="19"/>
-      <x:c r="J91" s="13" t="str"/>
-      <x:c r="K91" s="14"/>
-      <x:c r="L91" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="92">
-      <x:c r="A92" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
-      </x:c>
-      <x:c r="B92" s="18" t="n">
-        <x:v>2205674</x:v>
-      </x:c>
-      <x:c r="C92" s="13" t="n">
-        <x:v>15402</x:v>
-      </x:c>
-      <x:c r="D92" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E92" s="19" t="n">
-        <x:v>46232.57876157408</x:v>
-      </x:c>
-      <x:c r="F92" s="14" t="n">
-        <x:v>2173.95</x:v>
-      </x:c>
-      <x:c r="G92" s="18"/>
-      <x:c r="H92" s="14"/>
-      <x:c r="I92" s="19"/>
-      <x:c r="J92" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K92" s="14" t="n">
-        <x:v>2173.95</x:v>
-      </x:c>
-      <x:c r="L92" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="93">
-      <x:c r="A93" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
-      </x:c>
-      <x:c r="B93" s="18" t="n">
-        <x:v>2206284</x:v>
-      </x:c>
-      <x:c r="C93" s="13" t="n">
-        <x:v>15405</x:v>
-      </x:c>
-      <x:c r="D93" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E93" s="19" t="n">
-        <x:v>46232.59909722222</x:v>
-      </x:c>
-      <x:c r="F93" s="14" t="n">
-        <x:v>568.61</x:v>
-      </x:c>
-      <x:c r="G93" s="18"/>
-      <x:c r="H93" s="14"/>
-      <x:c r="I93" s="19"/>
-      <x:c r="J93" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K93" s="14" t="n">
-        <x:v>568.61</x:v>
-      </x:c>
-      <x:c r="L93" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="94">
-      <x:c r="A94" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
-      </x:c>
-      <x:c r="B94" s="18" t="n">
-        <x:v>2206293</x:v>
-      </x:c>
-      <x:c r="C94" s="13" t="n">
-        <x:v>15406</x:v>
-      </x:c>
-      <x:c r="D94" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E94" s="19" t="n">
-        <x:v>46232.60854166667</x:v>
-      </x:c>
-      <x:c r="F94" s="14" t="n">
-        <x:v>454.22</x:v>
-      </x:c>
-      <x:c r="G94" s="18"/>
-      <x:c r="H94" s="14"/>
-      <x:c r="I94" s="19"/>
-      <x:c r="J94" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K94" s="14" t="n">
-        <x:v>454.22</x:v>
-      </x:c>
-      <x:c r="L94" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="95">
-      <x:c r="A95" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
-      </x:c>
-      <x:c r="B95" s="18" t="n">
-        <x:v>2206603</x:v>
-      </x:c>
-      <x:c r="C95" s="13" t="n">
-        <x:v>15408</x:v>
-      </x:c>
-      <x:c r="D95" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E95" s="19" t="n">
-        <x:v>46232.799525462964</x:v>
-      </x:c>
-      <x:c r="F95" s="14" t="n">
-        <x:v>124.44</x:v>
-      </x:c>
-      <x:c r="G95" s="18"/>
-      <x:c r="H95" s="14"/>
-      <x:c r="I95" s="19"/>
-      <x:c r="J95" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K95" s="14" t="n">
-        <x:v>124.44</x:v>
-      </x:c>
-      <x:c r="L95" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="96">
-      <x:c r="A96" s="13" t="str">
-        <x:v>Vinilak Tintas Especiais</x:v>
-      </x:c>
-      <x:c r="B96" s="18" t="n">
-        <x:v>2207138</x:v>
-      </x:c>
-      <x:c r="C96" s="13" t="n">
-        <x:v>15412</x:v>
-      </x:c>
-      <x:c r="D96" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E96" s="19" t="n">
-        <x:v>46233.56369212963</x:v>
-      </x:c>
-      <x:c r="F96" s="14" t="n">
-        <x:v>503.59</x:v>
-      </x:c>
-      <x:c r="G96" s="18"/>
-      <x:c r="H96" s="14"/>
-      <x:c r="I96" s="19"/>
-      <x:c r="J96" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K96" s="14" t="n">
-        <x:v>503.59</x:v>
-      </x:c>
-      <x:c r="L96" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="97">
-      <x:c r="A97" s="13" t="str">
-        <x:v>João Pedro | Bprint Gráfica</x:v>
-      </x:c>
-      <x:c r="B97" s="18" t="n">
-        <x:v>2207378</x:v>
-      </x:c>
-      <x:c r="C97" s="13" t="n">
-        <x:v>15414</x:v>
-      </x:c>
-      <x:c r="D97" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E97" s="19" t="n">
-        <x:v>46233.572060185186</x:v>
-      </x:c>
-      <x:c r="F97" s="14" t="n">
-        <x:v>430.25</x:v>
-      </x:c>
-      <x:c r="G97" s="18"/>
-      <x:c r="H97" s="14"/>
-      <x:c r="I97" s="19"/>
-      <x:c r="J97" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K97" s="14" t="n">
-        <x:v>430.25</x:v>
-      </x:c>
-      <x:c r="L97" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="98">
-      <x:c r="A98" s="13" t="str">
-        <x:v>Evecar Auto Mecânica</x:v>
-      </x:c>
-      <x:c r="B98" s="18" t="n">
-        <x:v>2207368</x:v>
-      </x:c>
-      <x:c r="C98" s="13" t="str"/>
-      <x:c r="D98" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E98" s="19" t="n">
-        <x:v>46233.57381944444</x:v>
-      </x:c>
-      <x:c r="F98" s="14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G98" s="18"/>
-      <x:c r="H98" s="14"/>
-      <x:c r="I98" s="19"/>
-      <x:c r="J98" s="13" t="str"/>
-      <x:c r="K98" s="14"/>
-      <x:c r="L98" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="99">
-      <x:c r="A99" s="13" t="str">
-        <x:v>Carmaço - Fiori</x:v>
-      </x:c>
-      <x:c r="B99" s="18" t="n">
-        <x:v>2207562</x:v>
-      </x:c>
-      <x:c r="C99" s="13" t="n">
-        <x:v>15417</x:v>
-      </x:c>
-      <x:c r="D99" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E99" s="19" t="n">
-        <x:v>46233.67563657407</x:v>
-      </x:c>
-      <x:c r="F99" s="14" t="n">
-        <x:v>390.31</x:v>
-      </x:c>
-      <x:c r="G99" s="18"/>
-      <x:c r="H99" s="14"/>
-      <x:c r="I99" s="19"/>
-      <x:c r="J99" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K99" s="14" t="n">
-        <x:v>390.31</x:v>
-      </x:c>
-      <x:c r="L99" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="100">
-      <x:c r="A100" s="13" t="str">
-        <x:v>Queren Cyrino</x:v>
-      </x:c>
-      <x:c r="B100" s="18" t="n">
-        <x:v>2204550</x:v>
-      </x:c>
-      <x:c r="C100" s="13" t="str"/>
-      <x:c r="D100" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E100" s="19" t="n">
-        <x:v>46233.67685185185</x:v>
-      </x:c>
-      <x:c r="F100" s="14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G100" s="18"/>
-      <x:c r="H100" s="14"/>
-      <x:c r="I100" s="19"/>
-      <x:c r="J100" s="13" t="str"/>
-      <x:c r="K100" s="14"/>
-      <x:c r="L100" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="101">
-      <x:c r="A101" s="13" t="str">
-        <x:v>Sterimed-Sterimais-finan</x:v>
-      </x:c>
-      <x:c r="B101" s="18" t="n">
-        <x:v>2206736</x:v>
-      </x:c>
-      <x:c r="C101" s="13" t="str"/>
-      <x:c r="D101" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E101" s="19" t="n">
-        <x:v>46233.677256944444</x:v>
-      </x:c>
-      <x:c r="F101" s="14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G101" s="18"/>
-      <x:c r="H101" s="14"/>
-      <x:c r="I101" s="19"/>
-      <x:c r="J101" s="13" t="str"/>
-      <x:c r="K101" s="14"/>
-      <x:c r="L101" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="102">
-      <x:c r="A102" s="13" t="str">
-        <x:v>Queren Cyrino</x:v>
-      </x:c>
-      <x:c r="B102" s="18" t="n">
-        <x:v>2207563</x:v>
-      </x:c>
-      <x:c r="C102" s="13" t="n">
-        <x:v>15419</x:v>
-      </x:c>
-      <x:c r="D102" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E102" s="19" t="n">
-        <x:v>46233.69023148148</x:v>
-      </x:c>
-      <x:c r="F102" s="14" t="n">
-        <x:v>1168.34</x:v>
-      </x:c>
-      <x:c r="G102" s="18"/>
-      <x:c r="H102" s="14"/>
-      <x:c r="I102" s="19"/>
-      <x:c r="J102" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K102" s="14" t="n">
-        <x:v>1168.34</x:v>
-      </x:c>
-      <x:c r="L102" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="103">
-      <x:c r="A103" s="13" t="str">
-        <x:v>Cabaninha kids Brinquedos Pedagógico</x:v>
-      </x:c>
-      <x:c r="B103" s="18" t="n">
-        <x:v>2207565</x:v>
-      </x:c>
-      <x:c r="C103" s="13" t="str"/>
-      <x:c r="D103" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E103" s="19" t="n">
-        <x:v>46233.694918981484</x:v>
-      </x:c>
-      <x:c r="F103" s="14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G103" s="18"/>
-      <x:c r="H103" s="14"/>
-      <x:c r="I103" s="19"/>
-      <x:c r="J103" s="13" t="str"/>
-      <x:c r="K103" s="14"/>
-      <x:c r="L103" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="104">
-      <x:c r="A104" s="13" t="str">
-        <x:v>WOOD COLOR TINTAS</x:v>
-      </x:c>
-      <x:c r="B104" s="18" t="n">
-        <x:v>2207637</x:v>
-      </x:c>
-      <x:c r="C104" s="13" t="str"/>
-      <x:c r="D104" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E104" s="19" t="n">
-        <x:v>46233.700266203705</x:v>
-      </x:c>
-      <x:c r="F104" s="14" t="n">
-        <x:v>404.88</x:v>
-      </x:c>
-      <x:c r="G104" s="18"/>
-      <x:c r="H104" s="14"/>
-      <x:c r="I104" s="19"/>
-      <x:c r="J104" s="13" t="str"/>
-      <x:c r="K104" s="14"/>
-      <x:c r="L104" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="105">
-      <x:c r="A105" s="13" t="str">
-        <x:v>Juciliana</x:v>
-      </x:c>
-      <x:c r="B105" s="18" t="n">
-        <x:v>2206455</x:v>
-      </x:c>
-      <x:c r="C105" s="13" t="n">
-        <x:v>15407</x:v>
-      </x:c>
-      <x:c r="D105" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E105" s="19" t="n">
-        <x:v>46233.70322916667</x:v>
-      </x:c>
-      <x:c r="F105" s="14" t="n">
-        <x:v>251.25</x:v>
-      </x:c>
-      <x:c r="G105" s="18"/>
-      <x:c r="H105" s="14"/>
-      <x:c r="I105" s="19"/>
-      <x:c r="J105" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K105" s="14" t="n">
-        <x:v>251.25</x:v>
-      </x:c>
-      <x:c r="L105" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="106">
-      <x:c r="A106" s="13" t="str">
-        <x:v>Alcimara Carneiro</x:v>
-      </x:c>
-      <x:c r="B106" s="18" t="n">
-        <x:v>2207534</x:v>
-      </x:c>
-      <x:c r="C106" s="13" t="str"/>
-      <x:c r="D106" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E106" s="19" t="n">
-        <x:v>46233.70322916667</x:v>
-      </x:c>
-      <x:c r="F106" s="14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G106" s="18"/>
-      <x:c r="H106" s="14"/>
-      <x:c r="I106" s="19"/>
-      <x:c r="J106" s="13" t="str"/>
-      <x:c r="K106" s="14"/>
-      <x:c r="L106" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="107">
-      <x:c r="A107" s="13" t="str">
-        <x:v>FRANCHI NORTE DISTRIBUICAO LTDA</x:v>
-      </x:c>
-      <x:c r="B107" s="18" t="n">
-        <x:v>2205563</x:v>
-      </x:c>
-      <x:c r="C107" s="13" t="n">
-        <x:v>15396</x:v>
-      </x:c>
-      <x:c r="D107" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E107" s="19" t="n">
-        <x:v>46233.765810185185</x:v>
-      </x:c>
-      <x:c r="F107" s="14" t="n">
-        <x:v>250.89</x:v>
-      </x:c>
-      <x:c r="G107" s="18"/>
-      <x:c r="H107" s="14"/>
-      <x:c r="I107" s="19"/>
-      <x:c r="J107" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K107" s="14" t="n">
-        <x:v>250.89</x:v>
-      </x:c>
-      <x:c r="L107" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="108">
-      <x:c r="A108" s="13" t="str">
-        <x:v>Michele Pereira</x:v>
-      </x:c>
-      <x:c r="B108" s="18" t="n">
-        <x:v>2204577</x:v>
-      </x:c>
-      <x:c r="C108" s="13" t="str"/>
-      <x:c r="D108" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E108" s="19" t="n">
-        <x:v>46233.8053125</x:v>
-      </x:c>
-      <x:c r="F108" s="14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G108" s="18"/>
-      <x:c r="H108" s="14"/>
-      <x:c r="I108" s="19"/>
-      <x:c r="J108" s="13" t="str"/>
-      <x:c r="K108" s="14"/>
-      <x:c r="L108" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="109">
-      <x:c r="A109" s="13" t="str">
-        <x:v>Fernanda Alves</x:v>
-      </x:c>
-      <x:c r="B109" s="18" t="n">
-        <x:v>2207830</x:v>
-      </x:c>
-      <x:c r="C109" s="13" t="str"/>
-      <x:c r="D109" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E109" s="19" t="n">
-        <x:v>46234.48326388889</x:v>
-      </x:c>
-      <x:c r="F109" s="14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G109" s="18"/>
-      <x:c r="H109" s="14"/>
-      <x:c r="I109" s="19"/>
-      <x:c r="J109" s="13" t="str"/>
-      <x:c r="K109" s="14"/>
-      <x:c r="L109" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="110">
-      <x:c r="A110" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
-      </x:c>
-      <x:c r="B110" s="18" t="n">
-        <x:v>2208212</x:v>
-      </x:c>
-      <x:c r="C110" s="13" t="n">
-        <x:v>15421</x:v>
-      </x:c>
-      <x:c r="D110" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E110" s="19" t="n">
-        <x:v>46234.513715277775</x:v>
-      </x:c>
-      <x:c r="F110" s="14" t="n">
-        <x:v>142.51</x:v>
-      </x:c>
-      <x:c r="G110" s="18"/>
-      <x:c r="H110" s="14"/>
-      <x:c r="I110" s="19"/>
-      <x:c r="J110" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K110" s="14" t="n">
-        <x:v>142.51</x:v>
-      </x:c>
-      <x:c r="L110" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="111">
-      <x:c r="A111" s="13" t="str">
-        <x:v>Elisete Henck</x:v>
-      </x:c>
-      <x:c r="B111" s="18" t="n">
-        <x:v>2208349</x:v>
-      </x:c>
-      <x:c r="C111" s="13" t="n">
-        <x:v>15423</x:v>
-      </x:c>
-      <x:c r="D111" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E111" s="19" t="n">
-        <x:v>46234.616793981484</x:v>
-      </x:c>
-      <x:c r="F111" s="14" t="n">
-        <x:v>107.37</x:v>
-      </x:c>
-      <x:c r="G111" s="18"/>
-      <x:c r="H111" s="14"/>
-      <x:c r="I111" s="19"/>
-      <x:c r="J111" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K111" s="14" t="n">
-        <x:v>107.37</x:v>
-      </x:c>
-      <x:c r="L111" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="112">
-      <x:c r="A112" s="13" t="str">
-        <x:v>Lindsey Souza</x:v>
-      </x:c>
-      <x:c r="B112" s="18" t="n">
-        <x:v>2208171</x:v>
-      </x:c>
-      <x:c r="C112" s="13" t="str"/>
-      <x:c r="D112" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E112" s="19" t="n">
-        <x:v>46234.643541666665</x:v>
-      </x:c>
-      <x:c r="F112" s="14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G112" s="18"/>
-      <x:c r="H112" s="14"/>
-      <x:c r="I112" s="19"/>
-      <x:c r="J112" s="13" t="str"/>
-      <x:c r="K112" s="14"/>
-      <x:c r="L112" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="113">
-      <x:c r="A113" s="13" t="str">
-        <x:v>Logistica</x:v>
-      </x:c>
-      <x:c r="B113" s="18" t="n">
-        <x:v>2191659</x:v>
-      </x:c>
-      <x:c r="C113" s="13" t="n">
-        <x:v>15317</x:v>
-      </x:c>
-      <x:c r="D113" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E113" s="19" t="n">
-        <x:v>46234.67115740741</x:v>
-      </x:c>
-      <x:c r="F113" s="14" t="n">
-        <x:v>276.1</x:v>
-      </x:c>
-      <x:c r="G113" s="18"/>
-      <x:c r="H113" s="14"/>
-      <x:c r="I113" s="19"/>
-      <x:c r="J113" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K113" s="14" t="n">
-        <x:v>276.1</x:v>
-      </x:c>
-      <x:c r="L113" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="114">
-      <x:c r="A114" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
-      </x:c>
-      <x:c r="B114" s="18" t="n">
-        <x:v>2192512</x:v>
-      </x:c>
-      <x:c r="C114" s="13" t="n">
-        <x:v>15319</x:v>
-      </x:c>
-      <x:c r="D114" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E114" s="19" t="n">
-        <x:v>46234.67115740741</x:v>
-      </x:c>
-      <x:c r="F114" s="14" t="n">
-        <x:v>630.36</x:v>
-      </x:c>
-      <x:c r="G114" s="18"/>
-      <x:c r="H114" s="14"/>
-      <x:c r="I114" s="19"/>
-      <x:c r="J114" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K114" s="14" t="n">
-        <x:v>630.36</x:v>
-      </x:c>
-      <x:c r="L114" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="115">
-      <x:c r="A115" s="13" t="str">
-        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
-      </x:c>
-      <x:c r="B115" s="18" t="n">
-        <x:v>2193158</x:v>
-      </x:c>
-      <x:c r="C115" s="13" t="n">
-        <x:v>15321</x:v>
-      </x:c>
-      <x:c r="D115" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E115" s="19" t="n">
-        <x:v>46234.67115740741</x:v>
-      </x:c>
-      <x:c r="F115" s="14" t="n">
-        <x:v>226.75</x:v>
-      </x:c>
-      <x:c r="G115" s="18"/>
-      <x:c r="H115" s="14"/>
-      <x:c r="I115" s="19"/>
-      <x:c r="J115" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K115" s="14" t="n">
-        <x:v>226.75</x:v>
-      </x:c>
-      <x:c r="L115" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="116">
-      <x:c r="A116" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
-      </x:c>
-      <x:c r="B116" s="18" t="n">
-        <x:v>2193214</x:v>
-      </x:c>
-      <x:c r="C116" s="13" t="n">
-        <x:v>15323</x:v>
-      </x:c>
-      <x:c r="D116" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E116" s="19" t="n">
-        <x:v>46234.67115740741</x:v>
-      </x:c>
-      <x:c r="F116" s="14" t="n">
-        <x:v>222.19</x:v>
-      </x:c>
-      <x:c r="G116" s="18"/>
-      <x:c r="H116" s="14"/>
-      <x:c r="I116" s="19"/>
-      <x:c r="J116" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K116" s="14" t="n">
-        <x:v>222.19</x:v>
-      </x:c>
-      <x:c r="L116" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="117">
-      <x:c r="A117" s="13" t="str">
-        <x:v>LC Plásticos</x:v>
-      </x:c>
-      <x:c r="B117" s="18" t="n">
-        <x:v>2193641</x:v>
-      </x:c>
-      <x:c r="C117" s="13" t="n">
-        <x:v>15331</x:v>
-      </x:c>
-      <x:c r="D117" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E117" s="19" t="n">
-        <x:v>46234.67115740741</x:v>
-      </x:c>
-      <x:c r="F117" s="14" t="n">
-        <x:v>781.33</x:v>
-      </x:c>
-      <x:c r="G117" s="18"/>
-      <x:c r="H117" s="14"/>
-      <x:c r="I117" s="19"/>
-      <x:c r="J117" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K117" s="14" t="n">
-        <x:v>781.33</x:v>
-      </x:c>
-      <x:c r="L117" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="118">
-      <x:c r="A118" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
-      </x:c>
-      <x:c r="B118" s="18" t="n">
-        <x:v>2194620</x:v>
-      </x:c>
-      <x:c r="C118" s="13" t="n">
-        <x:v>15335</x:v>
-      </x:c>
-      <x:c r="D118" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E118" s="19" t="n">
-        <x:v>46234.67115740741</x:v>
-      </x:c>
-      <x:c r="F118" s="14" t="n">
-        <x:v>437.67</x:v>
-      </x:c>
-      <x:c r="G118" s="18"/>
-      <x:c r="H118" s="14"/>
-      <x:c r="I118" s="19"/>
-      <x:c r="J118" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K118" s="14" t="n">
-        <x:v>437.67</x:v>
-      </x:c>
-      <x:c r="L118" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="119">
-      <x:c r="A119" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
-      </x:c>
-      <x:c r="B119" s="18" t="n">
-        <x:v>2194619</x:v>
-      </x:c>
-      <x:c r="C119" s="13" t="n">
-        <x:v>15340</x:v>
-      </x:c>
-      <x:c r="D119" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E119" s="19" t="n">
-        <x:v>46234.681550925925</x:v>
-      </x:c>
-      <x:c r="F119" s="14" t="n">
-        <x:v>434.19</x:v>
-      </x:c>
-      <x:c r="G119" s="18"/>
-      <x:c r="H119" s="14"/>
-      <x:c r="I119" s="19"/>
-      <x:c r="J119" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K119" s="14" t="n">
-        <x:v>434.19</x:v>
-      </x:c>
-      <x:c r="L119" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="120">
-      <x:c r="A120" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
-      </x:c>
-      <x:c r="B120" s="18" t="n">
-        <x:v>2208468</x:v>
-      </x:c>
-      <x:c r="C120" s="13" t="n">
-        <x:v>15424</x:v>
-      </x:c>
-      <x:c r="D120" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E120" s="19" t="n">
-        <x:v>46234.737546296295</x:v>
-      </x:c>
-      <x:c r="F120" s="14" t="n">
-        <x:v>310.75</x:v>
-      </x:c>
-      <x:c r="G120" s="18"/>
-      <x:c r="H120" s="14"/>
-      <x:c r="I120" s="19"/>
-      <x:c r="J120" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K120" s="14" t="n">
-        <x:v>310.75</x:v>
-      </x:c>
-      <x:c r="L120" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="121">
-      <x:c r="A121" s="13" t="str">
-        <x:v>Fernanda Qualisol</x:v>
-      </x:c>
-      <x:c r="B121" s="18" t="n">
-        <x:v>2204771</x:v>
-      </x:c>
-      <x:c r="C121" s="13" t="str"/>
-      <x:c r="D121" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E121" s="19" t="n">
-        <x:v>46234.75952546296</x:v>
-      </x:c>
-      <x:c r="F121" s="14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G121" s="18"/>
-      <x:c r="H121" s="14"/>
-      <x:c r="I121" s="19"/>
-      <x:c r="J121" s="13" t="str"/>
-      <x:c r="K121" s="14"/>
-      <x:c r="L121" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="122">
-      <x:c r="A122" s="13" t="str">
-        <x:v>Viviane Pinheiro</x:v>
-      </x:c>
-      <x:c r="B122" s="18" t="n">
-        <x:v>2208572</x:v>
-      </x:c>
-      <x:c r="C122" s="13" t="n">
-        <x:v>15425</x:v>
-      </x:c>
-      <x:c r="D122" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E122" s="19" t="n">
-        <x:v>46234.7840625</x:v>
-      </x:c>
-      <x:c r="F122" s="14" t="n">
-        <x:v>770.68</x:v>
-      </x:c>
-      <x:c r="G122" s="18"/>
-      <x:c r="H122" s="14"/>
-      <x:c r="I122" s="19"/>
-      <x:c r="J122" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K122" s="14" t="n">
-        <x:v>770.68</x:v>
-      </x:c>
-      <x:c r="L122" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="123">
-      <x:c r="A123" s="13" t="str">
-        <x:v>Sterimed-Sterimais-finan</x:v>
-      </x:c>
-      <x:c r="B123" s="18" t="n">
-        <x:v>2208182</x:v>
-      </x:c>
-      <x:c r="C123" s="13" t="n">
-        <x:v>15426</x:v>
-      </x:c>
-      <x:c r="D123" s="13" t="str">
-        <x:v>Aberto</x:v>
-      </x:c>
-      <x:c r="E123" s="19" t="n">
-        <x:v>46237.49989583333</x:v>
-      </x:c>
-      <x:c r="F123" s="14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G123" s="18"/>
-      <x:c r="H123" s="14"/>
-      <x:c r="I123" s="19"/>
-      <x:c r="J123" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K123" s="14" t="n">
-        <x:v>1128.09</x:v>
-      </x:c>
-      <x:c r="L123" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="124">
-      <x:c r="A124" s="13" t="str">
-        <x:v>Bruno luz</x:v>
-      </x:c>
-      <x:c r="B124" s="18" t="n">
-        <x:v>2207820</x:v>
-      </x:c>
-      <x:c r="C124" s="13" t="str"/>
-      <x:c r="D124" s="13" t="str">
-        <x:v>Perdido</x:v>
-      </x:c>
-      <x:c r="E124" s="19" t="n">
-        <x:v>46237.516493055555</x:v>
-      </x:c>
-      <x:c r="F124" s="14" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G124" s="18"/>
-      <x:c r="H124" s="14"/>
-      <x:c r="I124" s="19"/>
-      <x:c r="J124" s="13" t="str"/>
-      <x:c r="K124" s="14"/>
-      <x:c r="L124" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5478,7 +4432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref4d4d49bfc64edb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb185d3d2a28c4d98"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
chore(crm): regenera relatorio filtrado
</commit_message>
<xml_diff>
--- a/outputs/relatorio-cotacoes-fernanda-2026-07-07-a-2026-07-31.xlsx
+++ b/outputs/relatorio-cotacoes-fernanda-2026-07-07-a-2026-07-31.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ganhos" sheetId="1" r:id="Re3604f7c3b2843c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Não ganhos" sheetId="2" r:id="R2659556bd2814b33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revisão" sheetId="3" r:id="R3d19e4d693484a01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ganhos" sheetId="1" r:id="R5223ea5e93f84687"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Não ganhos" sheetId="2" r:id="Rf39837a1d9874011"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revisão" sheetId="3" r:id="Rca1d6a8ba90e4285"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1938,7 +1938,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R08a11a15f11748d7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb45d7ffe8c6e45bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4432,7 +4432,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb185d3d2a28c4d98"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13dabc07b8bc4012"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
fix(crm): usa data do status no periodo de ganhos
</commit_message>
<xml_diff>
--- a/outputs/relatorio-cotacoes-fernanda-2026-07-07-a-2026-07-31.xlsx
+++ b/outputs/relatorio-cotacoes-fernanda-2026-07-07-a-2026-07-31.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ganhos" sheetId="1" r:id="R5223ea5e93f84687"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Não ganhos" sheetId="2" r:id="Rf39837a1d9874011"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revisão" sheetId="3" r:id="Rca1d6a8ba90e4285"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ganhos" sheetId="1" r:id="R0f6cd408705d4644"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Não ganhos" sheetId="2" r:id="Re554c432aa1f4b38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revisão" sheetId="3" r:id="Ra51f435738884938"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -197,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GanhosTable" displayName="GanhosTable" ref="A11:L44" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A11:L44"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GanhosTable" displayName="GanhosTable" ref="A11:L48" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A11:L48"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Título"/>
     <x:tableColumn id="2" name="ID card Cubo"/>
@@ -218,8 +218,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="NoganhosTable" displayName="NoganhosTable" ref="A11:L84" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A11:L84"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="NoganhosTable" displayName="NoganhosTable" ref="A11:L98" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A11:L98"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="Título"/>
     <x:tableColumn id="2" name="ID card Cubo"/>
@@ -494,7 +494,7 @@
         <x:v>Cards</x:v>
       </x:c>
       <x:c r="B5" s="13" t="n">
-        <x:v>33</x:v>
+        <x:v>37</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -510,7 +510,7 @@
         <x:v>Valor Cubo</x:v>
       </x:c>
       <x:c r="B7" s="14" t="n">
-        <x:v>17516.13</x:v>
+        <x:v>22524.71</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1667,220 +1667,196 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
+        <x:v>Quimi Vida</x:v>
       </x:c>
       <x:c r="B37" s="18" t="n">
-        <x:v>2188035</x:v>
-      </x:c>
-      <x:c r="C37" s="13" t="n">
-        <x:v>15296</x:v>
-      </x:c>
+        <x:v>2172845</x:v>
+      </x:c>
+      <x:c r="C37" s="13" t="str"/>
       <x:c r="D37" s="13" t="str">
         <x:v>Ganho</x:v>
       </x:c>
       <x:c r="E37" s="19" t="n">
-        <x:v>46213.82513888889</x:v>
+        <x:v>46213.729409722226</x:v>
       </x:c>
       <x:c r="F37" s="14" t="n">
-        <x:v>940.17</x:v>
+        <x:v>821.17</x:v>
       </x:c>
       <x:c r="G37" s="18"/>
       <x:c r="H37" s="14"/>
       <x:c r="I37" s="19"/>
-      <x:c r="J37" s="13" t="str">
-        <x:v>APROVADA</x:v>
-      </x:c>
-      <x:c r="K37" s="14" t="n">
-        <x:v>940.17</x:v>
-      </x:c>
+      <x:c r="J37" s="13" t="str"/>
+      <x:c r="K37" s="14"/>
       <x:c r="L37" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
       <x:c r="M37" s="23" t="str"/>
       <x:c r="N37" s="25" t="str"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="13" t="str">
-        <x:v>Sterilex - Transporte</x:v>
+        <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B38" s="18" t="n">
-        <x:v>2200205</x:v>
-      </x:c>
-      <x:c r="C38" s="13" t="str"/>
+        <x:v>2188035</x:v>
+      </x:c>
+      <x:c r="C38" s="13" t="n">
+        <x:v>15296</x:v>
+      </x:c>
       <x:c r="D38" s="13" t="str">
         <x:v>Ganho</x:v>
       </x:c>
       <x:c r="E38" s="19" t="n">
-        <x:v>46226.76613425926</x:v>
+        <x:v>46213.82513888889</x:v>
       </x:c>
       <x:c r="F38" s="14" t="n">
-        <x:v>296.85</x:v>
+        <x:v>940.17</x:v>
       </x:c>
       <x:c r="G38" s="18"/>
       <x:c r="H38" s="14"/>
       <x:c r="I38" s="19"/>
-      <x:c r="J38" s="13" t="str"/>
-      <x:c r="K38" s="14"/>
+      <x:c r="J38" s="13" t="str">
+        <x:v>APROVADA</x:v>
+      </x:c>
+      <x:c r="K38" s="14" t="n">
+        <x:v>940.17</x:v>
+      </x:c>
       <x:c r="L38" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
       <x:c r="M38" s="23" t="str"/>
       <x:c r="N38" s="25" t="str"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="13" t="str">
-        <x:v>WOOD COLOR TINTAS</x:v>
+        <x:v>FLATECK AUTOMATION LTDA</x:v>
       </x:c>
       <x:c r="B39" s="18" t="n">
-        <x:v>2206231</x:v>
-      </x:c>
-      <x:c r="C39" s="13" t="n">
-        <x:v>15400</x:v>
-      </x:c>
+        <x:v>2145147</x:v>
+      </x:c>
+      <x:c r="C39" s="13" t="str"/>
       <x:c r="D39" s="13" t="str">
         <x:v>Ganho</x:v>
       </x:c>
       <x:c r="E39" s="19" t="n">
-        <x:v>46232.55829861111</x:v>
+        <x:v>46216.70232638889</x:v>
       </x:c>
       <x:c r="F39" s="14" t="n">
-        <x:v>404.88</x:v>
+        <x:v>193.23</x:v>
       </x:c>
       <x:c r="G39" s="18"/>
       <x:c r="H39" s="14"/>
       <x:c r="I39" s="19"/>
-      <x:c r="J39" s="13" t="str">
-        <x:v>APROVADA</x:v>
-      </x:c>
-      <x:c r="K39" s="14" t="n">
-        <x:v>404.88</x:v>
-      </x:c>
+      <x:c r="J39" s="13" t="str"/>
+      <x:c r="K39" s="14"/>
       <x:c r="L39" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
       <x:c r="M39" s="23" t="str"/>
       <x:c r="N39" s="25" t="str"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="13" t="str">
-        <x:v>Solvmax Adm</x:v>
+        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
       </x:c>
       <x:c r="B40" s="18" t="n">
-        <x:v>2205743</x:v>
-      </x:c>
-      <x:c r="C40" s="13" t="n">
-        <x:v>15399</x:v>
-      </x:c>
+        <x:v>2181683</x:v>
+      </x:c>
+      <x:c r="C40" s="13" t="str"/>
       <x:c r="D40" s="13" t="str">
         <x:v>Ganho</x:v>
       </x:c>
       <x:c r="E40" s="19" t="n">
-        <x:v>46232.66971064815</x:v>
+        <x:v>46216.70232638889</x:v>
       </x:c>
       <x:c r="F40" s="14" t="n">
-        <x:v>847.19</x:v>
+        <x:v>394.18</x:v>
       </x:c>
       <x:c r="G40" s="18"/>
       <x:c r="H40" s="14"/>
       <x:c r="I40" s="19"/>
-      <x:c r="J40" s="13" t="str">
-        <x:v>APROVADA</x:v>
-      </x:c>
-      <x:c r="K40" s="14" t="n">
-        <x:v>847.19</x:v>
-      </x:c>
+      <x:c r="J40" s="13" t="str"/>
+      <x:c r="K40" s="14"/>
       <x:c r="L40" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
       <x:c r="M40" s="23" t="str"/>
       <x:c r="N40" s="25" t="str"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="13" t="str">
-        <x:v>Thomas Estoque R Imper</x:v>
+        <x:v>Neto Mendes- Silux</x:v>
       </x:c>
       <x:c r="B41" s="18" t="n">
-        <x:v>2206280</x:v>
-      </x:c>
-      <x:c r="C41" s="13" t="n">
-        <x:v>15403</x:v>
-      </x:c>
+        <x:v>2180479</x:v>
+      </x:c>
+      <x:c r="C41" s="13" t="str"/>
       <x:c r="D41" s="13" t="str">
         <x:v>Ganho</x:v>
       </x:c>
       <x:c r="E41" s="19" t="n">
-        <x:v>46233.48684027778</x:v>
+        <x:v>46218.53824074074</x:v>
       </x:c>
       <x:c r="F41" s="14" t="n">
-        <x:v>712.69</x:v>
+        <x:v>3600</x:v>
       </x:c>
       <x:c r="G41" s="18"/>
       <x:c r="H41" s="14"/>
       <x:c r="I41" s="19"/>
-      <x:c r="J41" s="13" t="str">
-        <x:v>APROVADA</x:v>
-      </x:c>
-      <x:c r="K41" s="14" t="n">
-        <x:v>712.69</x:v>
-      </x:c>
+      <x:c r="J41" s="13" t="str"/>
+      <x:c r="K41" s="14"/>
       <x:c r="L41" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
       <x:c r="M41" s="23" t="str"/>
       <x:c r="N41" s="25" t="str"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="13" t="str">
-        <x:v>63.110.705 REYNALDO LUIZ CERQUEIRA DE SOUZA</x:v>
+        <x:v>Sterilex - Transporte</x:v>
       </x:c>
       <x:c r="B42" s="18" t="n">
-        <x:v>2207113</x:v>
-      </x:c>
-      <x:c r="C42" s="13" t="n">
-        <x:v>15411</x:v>
-      </x:c>
+        <x:v>2200205</x:v>
+      </x:c>
+      <x:c r="C42" s="13" t="str"/>
       <x:c r="D42" s="13" t="str">
         <x:v>Ganho</x:v>
       </x:c>
       <x:c r="E42" s="19" t="n">
-        <x:v>46233.48684027778</x:v>
+        <x:v>46226.76613425926</x:v>
       </x:c>
       <x:c r="F42" s="14" t="n">
-        <x:v>920.22</x:v>
+        <x:v>296.85</x:v>
       </x:c>
       <x:c r="G42" s="18"/>
       <x:c r="H42" s="14"/>
       <x:c r="I42" s="19"/>
-      <x:c r="J42" s="13" t="str">
-        <x:v>APROVADA</x:v>
-      </x:c>
-      <x:c r="K42" s="14" t="n">
-        <x:v>920.22</x:v>
-      </x:c>
+      <x:c r="J42" s="13" t="str"/>
+      <x:c r="K42" s="14"/>
       <x:c r="L42" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
       <x:c r="M42" s="23" t="str"/>
       <x:c r="N42" s="25" t="str"/>
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="13" t="str">
-        <x:v>Carmaço - Fiori</x:v>
+        <x:v>WOOD COLOR TINTAS</x:v>
       </x:c>
       <x:c r="B43" s="18" t="n">
-        <x:v>2207579</x:v>
+        <x:v>2206231</x:v>
       </x:c>
       <x:c r="C43" s="13" t="n">
-        <x:v>15418</x:v>
+        <x:v>15400</x:v>
       </x:c>
       <x:c r="D43" s="13" t="str">
         <x:v>Ganho</x:v>
       </x:c>
       <x:c r="E43" s="19" t="n">
-        <x:v>46233.691087962965</x:v>
+        <x:v>46232.55829861111</x:v>
       </x:c>
       <x:c r="F43" s="14" t="n">
-        <x:v>239.73</x:v>
+        <x:v>404.88</x:v>
       </x:c>
       <x:c r="G43" s="18"/>
       <x:c r="H43" s="14"/>
@@ -1889,7 +1865,7 @@
         <x:v>APROVADA</x:v>
       </x:c>
       <x:c r="K43" s="14" t="n">
-        <x:v>239.73</x:v>
+        <x:v>404.88</x:v>
       </x:c>
       <x:c r="L43" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -1899,22 +1875,22 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="13" t="str">
-        <x:v>Alisson Soratto</x:v>
+        <x:v>Solvmax Adm</x:v>
       </x:c>
       <x:c r="B44" s="18" t="n">
-        <x:v>2208211</x:v>
+        <x:v>2205743</x:v>
       </x:c>
       <x:c r="C44" s="13" t="n">
-        <x:v>15422</x:v>
+        <x:v>15399</x:v>
       </x:c>
       <x:c r="D44" s="13" t="str">
         <x:v>Ganho</x:v>
       </x:c>
       <x:c r="E44" s="19" t="n">
-        <x:v>46234.54046296296</x:v>
+        <x:v>46232.66971064815</x:v>
       </x:c>
       <x:c r="F44" s="14" t="n">
-        <x:v>135.18</x:v>
+        <x:v>847.19</x:v>
       </x:c>
       <x:c r="G44" s="18"/>
       <x:c r="H44" s="14"/>
@@ -1923,13 +1899,149 @@
         <x:v>APROVADA</x:v>
       </x:c>
       <x:c r="K44" s="14" t="n">
-        <x:v>135.18</x:v>
+        <x:v>847.19</x:v>
       </x:c>
       <x:c r="L44" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
       <x:c r="M44" s="23" t="str"/>
       <x:c r="N44" s="25" t="str"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="13" t="str">
+        <x:v>Thomas Estoque R Imper</x:v>
+      </x:c>
+      <x:c r="B45" s="18" t="n">
+        <x:v>2206280</x:v>
+      </x:c>
+      <x:c r="C45" s="13" t="n">
+        <x:v>15403</x:v>
+      </x:c>
+      <x:c r="D45" s="13" t="str">
+        <x:v>Ganho</x:v>
+      </x:c>
+      <x:c r="E45" s="19" t="n">
+        <x:v>46233.48684027778</x:v>
+      </x:c>
+      <x:c r="F45" s="14" t="n">
+        <x:v>712.69</x:v>
+      </x:c>
+      <x:c r="G45" s="18"/>
+      <x:c r="H45" s="14"/>
+      <x:c r="I45" s="19"/>
+      <x:c r="J45" s="13" t="str">
+        <x:v>APROVADA</x:v>
+      </x:c>
+      <x:c r="K45" s="14" t="n">
+        <x:v>712.69</x:v>
+      </x:c>
+      <x:c r="L45" s="20" t="str">
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+      </x:c>
+      <x:c r="M45" s="23" t="str"/>
+      <x:c r="N45" s="25" t="str"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="13" t="str">
+        <x:v>63.110.705 REYNALDO LUIZ CERQUEIRA DE SOUZA</x:v>
+      </x:c>
+      <x:c r="B46" s="18" t="n">
+        <x:v>2207113</x:v>
+      </x:c>
+      <x:c r="C46" s="13" t="n">
+        <x:v>15411</x:v>
+      </x:c>
+      <x:c r="D46" s="13" t="str">
+        <x:v>Ganho</x:v>
+      </x:c>
+      <x:c r="E46" s="19" t="n">
+        <x:v>46233.48684027778</x:v>
+      </x:c>
+      <x:c r="F46" s="14" t="n">
+        <x:v>920.22</x:v>
+      </x:c>
+      <x:c r="G46" s="18"/>
+      <x:c r="H46" s="14"/>
+      <x:c r="I46" s="19"/>
+      <x:c r="J46" s="13" t="str">
+        <x:v>APROVADA</x:v>
+      </x:c>
+      <x:c r="K46" s="14" t="n">
+        <x:v>920.22</x:v>
+      </x:c>
+      <x:c r="L46" s="20" t="str">
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+      </x:c>
+      <x:c r="M46" s="23" t="str"/>
+      <x:c r="N46" s="25" t="str"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="13" t="str">
+        <x:v>Carmaço - Fiori</x:v>
+      </x:c>
+      <x:c r="B47" s="18" t="n">
+        <x:v>2207579</x:v>
+      </x:c>
+      <x:c r="C47" s="13" t="n">
+        <x:v>15418</x:v>
+      </x:c>
+      <x:c r="D47" s="13" t="str">
+        <x:v>Ganho</x:v>
+      </x:c>
+      <x:c r="E47" s="19" t="n">
+        <x:v>46233.691087962965</x:v>
+      </x:c>
+      <x:c r="F47" s="14" t="n">
+        <x:v>239.73</x:v>
+      </x:c>
+      <x:c r="G47" s="18"/>
+      <x:c r="H47" s="14"/>
+      <x:c r="I47" s="19"/>
+      <x:c r="J47" s="13" t="str">
+        <x:v>APROVADA</x:v>
+      </x:c>
+      <x:c r="K47" s="14" t="n">
+        <x:v>239.73</x:v>
+      </x:c>
+      <x:c r="L47" s="20" t="str">
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+      </x:c>
+      <x:c r="M47" s="23" t="str"/>
+      <x:c r="N47" s="25" t="str"/>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="13" t="str">
+        <x:v>Alisson Soratto</x:v>
+      </x:c>
+      <x:c r="B48" s="18" t="n">
+        <x:v>2208211</x:v>
+      </x:c>
+      <x:c r="C48" s="13" t="n">
+        <x:v>15422</x:v>
+      </x:c>
+      <x:c r="D48" s="13" t="str">
+        <x:v>Ganho</x:v>
+      </x:c>
+      <x:c r="E48" s="19" t="n">
+        <x:v>46234.54046296296</x:v>
+      </x:c>
+      <x:c r="F48" s="14" t="n">
+        <x:v>135.18</x:v>
+      </x:c>
+      <x:c r="G48" s="18"/>
+      <x:c r="H48" s="14"/>
+      <x:c r="I48" s="19"/>
+      <x:c r="J48" s="13" t="str">
+        <x:v>APROVADA</x:v>
+      </x:c>
+      <x:c r="K48" s="14" t="n">
+        <x:v>135.18</x:v>
+      </x:c>
+      <x:c r="L48" s="20" t="str">
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+      </x:c>
+      <x:c r="M48" s="23" t="str"/>
+      <x:c r="N48" s="25" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1938,7 +2050,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb45d7ffe8c6e45bc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3c398e4708354d43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2006,7 +2118,7 @@
         <x:v>Cards</x:v>
       </x:c>
       <x:c r="B5" s="13" t="n">
-        <x:v>73</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2022,7 +2134,7 @@
         <x:v>Valor Cubo</x:v>
       </x:c>
       <x:c r="B7" s="14" t="n">
-        <x:v>46186.99</x:v>
+        <x:v>53133.86999999999</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -2301,191 +2413,161 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="13" t="str">
-        <x:v>Fernanda Qualisol</x:v>
+        <x:v>Monick Clipack</x:v>
       </x:c>
       <x:c r="B18" s="18" t="n">
-        <x:v>2183458</x:v>
-      </x:c>
-      <x:c r="C18" s="13" t="n">
-        <x:v>15285</x:v>
-      </x:c>
+        <x:v>2159444</x:v>
+      </x:c>
+      <x:c r="C18" s="13" t="str"/>
       <x:c r="D18" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E18" s="19" t="n">
-        <x:v>46216.70232638889</x:v>
+        <x:v>46210.58420138889</x:v>
       </x:c>
       <x:c r="F18" s="14" t="n">
-        <x:v>375.07</x:v>
+        <x:v>309.33</x:v>
       </x:c>
       <x:c r="G18" s="18"/>
       <x:c r="H18" s="14"/>
       <x:c r="I18" s="19"/>
-      <x:c r="J18" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K18" s="14" t="n">
-        <x:v>375.07</x:v>
-      </x:c>
+      <x:c r="J18" s="13" t="str"/>
+      <x:c r="K18" s="14"/>
       <x:c r="L18" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="13" t="str">
-        <x:v>Carmaço - Fiori</x:v>
+        <x:v>Jessica Protelim</x:v>
       </x:c>
       <x:c r="B19" s="18" t="n">
-        <x:v>2191676</x:v>
-      </x:c>
-      <x:c r="C19" s="13" t="n">
-        <x:v>15316</x:v>
-      </x:c>
+        <x:v>2160922</x:v>
+      </x:c>
+      <x:c r="C19" s="13" t="str"/>
       <x:c r="D19" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E19" s="19" t="n">
-        <x:v>46219.57885416667</x:v>
+        <x:v>46211.71430555556</x:v>
       </x:c>
       <x:c r="F19" s="14" t="n">
-        <x:v>660.68</x:v>
+        <x:v>1233.64</x:v>
       </x:c>
       <x:c r="G19" s="18"/>
       <x:c r="H19" s="14"/>
       <x:c r="I19" s="19"/>
-      <x:c r="J19" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K19" s="14" t="n">
-        <x:v>581.14</x:v>
-      </x:c>
+      <x:c r="J19" s="13" t="str"/>
+      <x:c r="K19" s="14"/>
       <x:c r="L19" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="13" t="str">
-        <x:v>Fernanda Qualisol</x:v>
+        <x:v>Bruno Cervera</x:v>
       </x:c>
       <x:c r="B20" s="18" t="n">
-        <x:v>2193323</x:v>
-      </x:c>
-      <x:c r="C20" s="13" t="n">
-        <x:v>15326</x:v>
-      </x:c>
+        <x:v>2175001</x:v>
+      </x:c>
+      <x:c r="C20" s="13" t="str"/>
       <x:c r="D20" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E20" s="19" t="n">
-        <x:v>46219.695081018515</x:v>
+        <x:v>46211.74517361111</x:v>
       </x:c>
       <x:c r="F20" s="14" t="n">
-        <x:v>156.68</x:v>
+        <x:v>255.11</x:v>
       </x:c>
       <x:c r="G20" s="18"/>
       <x:c r="H20" s="14"/>
       <x:c r="I20" s="19"/>
-      <x:c r="J20" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K20" s="14" t="n">
-        <x:v>156.68</x:v>
-      </x:c>
+      <x:c r="J20" s="13" t="str"/>
+      <x:c r="K20" s="14"/>
       <x:c r="L20" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="13" t="str">
-        <x:v>Fernanda Qualisol</x:v>
+        <x:v>Marketing Seuposto</x:v>
       </x:c>
       <x:c r="B21" s="18" t="n">
-        <x:v>2193563</x:v>
-      </x:c>
-      <x:c r="C21" s="13" t="n">
-        <x:v>15328</x:v>
-      </x:c>
+        <x:v>2176453</x:v>
+      </x:c>
+      <x:c r="C21" s="13" t="str"/>
       <x:c r="D21" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E21" s="19" t="n">
-        <x:v>46219.754375</x:v>
+        <x:v>46216.68895833333</x:v>
       </x:c>
       <x:c r="F21" s="14" t="n">
-        <x:v>434.59</x:v>
+        <x:v>250.12</x:v>
       </x:c>
       <x:c r="G21" s="18"/>
       <x:c r="H21" s="14"/>
       <x:c r="I21" s="19"/>
-      <x:c r="J21" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K21" s="14" t="n">
-        <x:v>434.59</x:v>
-      </x:c>
+      <x:c r="J21" s="13" t="str"/>
+      <x:c r="K21" s="14"/>
       <x:c r="L21" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="13" t="str">
-        <x:v>Comercial IQL-NEXUS</x:v>
+        <x:v>Qualidade Almad</x:v>
       </x:c>
       <x:c r="B22" s="18" t="n">
-        <x:v>2193205</x:v>
-      </x:c>
-      <x:c r="C22" s="13" t="n">
-        <x:v>15324</x:v>
-      </x:c>
+        <x:v>2176546</x:v>
+      </x:c>
+      <x:c r="C22" s="13" t="str"/>
       <x:c r="D22" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E22" s="19" t="n">
-        <x:v>46220.549305555556</x:v>
+        <x:v>46216.68895833333</x:v>
       </x:c>
       <x:c r="F22" s="14" t="n">
-        <x:v>1529.67</x:v>
+        <x:v>610.28</x:v>
       </x:c>
       <x:c r="G22" s="18"/>
       <x:c r="H22" s="14"/>
       <x:c r="I22" s="19"/>
-      <x:c r="J22" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K22" s="14" t="n">
-        <x:v>1529.67</x:v>
-      </x:c>
+      <x:c r="J22" s="13" t="str"/>
+      <x:c r="K22" s="14"/>
       <x:c r="L22" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
+        <x:v>Fernanda Qualisol</x:v>
       </x:c>
       <x:c r="B23" s="18" t="n">
-        <x:v>2194690</x:v>
+        <x:v>2183458</x:v>
       </x:c>
       <x:c r="C23" s="13" t="n">
-        <x:v>15337</x:v>
+        <x:v>15285</x:v>
       </x:c>
       <x:c r="D23" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E23" s="19" t="n">
-        <x:v>46220.74028935185</x:v>
+        <x:v>46216.70232638889</x:v>
       </x:c>
       <x:c r="F23" s="14" t="n">
-        <x:v>164.17</x:v>
+        <x:v>375.07</x:v>
       </x:c>
       <x:c r="G23" s="18"/>
       <x:c r="H23" s="14"/>
       <x:c r="I23" s="19"/>
       <x:c r="J23" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K23" s="14" t="n">
-        <x:v>164.17</x:v>
+        <x:v>375.07</x:v>
       </x:c>
       <x:c r="L23" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -2493,54 +2575,48 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="13" t="str">
-        <x:v>Roseli - Industria Portas</x:v>
+        <x:v>Exclusive Cristais</x:v>
       </x:c>
       <x:c r="B24" s="18" t="n">
-        <x:v>2196088</x:v>
-      </x:c>
-      <x:c r="C24" s="13" t="n">
-        <x:v>15341</x:v>
-      </x:c>
+        <x:v>2178850</x:v>
+      </x:c>
+      <x:c r="C24" s="13" t="str"/>
       <x:c r="D24" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E24" s="19" t="n">
-        <x:v>46223.494039351855</x:v>
+        <x:v>46218.782800925925</x:v>
       </x:c>
       <x:c r="F24" s="14" t="n">
-        <x:v>295.86</x:v>
+        <x:v>1251.11</x:v>
       </x:c>
       <x:c r="G24" s="18"/>
       <x:c r="H24" s="14"/>
       <x:c r="I24" s="19"/>
-      <x:c r="J24" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K24" s="14" t="n">
-        <x:v>295.86</x:v>
-      </x:c>
+      <x:c r="J24" s="13" t="str"/>
+      <x:c r="K24" s="14"/>
       <x:c r="L24" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="13" t="str">
-        <x:v>Rosset Cia 2 Devoluções</x:v>
+        <x:v>Carmaço - Fiori</x:v>
       </x:c>
       <x:c r="B25" s="18" t="n">
-        <x:v>2190103</x:v>
+        <x:v>2191676</x:v>
       </x:c>
       <x:c r="C25" s="13" t="n">
-        <x:v>15300</x:v>
+        <x:v>15316</x:v>
       </x:c>
       <x:c r="D25" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E25" s="19" t="n">
-        <x:v>46223.590682870374</x:v>
+        <x:v>46219.57885416667</x:v>
       </x:c>
       <x:c r="F25" s="14" t="n">
-        <x:v>927.98</x:v>
+        <x:v>660.68</x:v>
       </x:c>
       <x:c r="G25" s="18"/>
       <x:c r="H25" s="14"/>
@@ -2549,7 +2625,7 @@
         <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K25" s="14" t="n">
-        <x:v>927.98</x:v>
+        <x:v>581.14</x:v>
       </x:c>
       <x:c r="L25" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -2557,22 +2633,22 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="13" t="str">
-        <x:v>MARCEL FACAS</x:v>
+        <x:v>Fernanda Qualisol</x:v>
       </x:c>
       <x:c r="B26" s="18" t="n">
-        <x:v>2191327</x:v>
+        <x:v>2193323</x:v>
       </x:c>
       <x:c r="C26" s="13" t="n">
-        <x:v>15306</x:v>
+        <x:v>15326</x:v>
       </x:c>
       <x:c r="D26" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E26" s="19" t="n">
-        <x:v>46223.7403587963</x:v>
+        <x:v>46219.695081018515</x:v>
       </x:c>
       <x:c r="F26" s="14" t="n">
-        <x:v>255.51</x:v>
+        <x:v>156.68</x:v>
       </x:c>
       <x:c r="G26" s="18"/>
       <x:c r="H26" s="14"/>
@@ -2581,7 +2657,7 @@
         <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K26" s="14" t="n">
-        <x:v>255.51</x:v>
+        <x:v>156.68</x:v>
       </x:c>
       <x:c r="L26" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -2589,22 +2665,22 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="13" t="str">
-        <x:v>Evelyn Brito</x:v>
+        <x:v>Fernanda Qualisol</x:v>
       </x:c>
       <x:c r="B27" s="18" t="n">
-        <x:v>2191363</x:v>
+        <x:v>2193563</x:v>
       </x:c>
       <x:c r="C27" s="13" t="n">
-        <x:v>15307</x:v>
+        <x:v>15328</x:v>
       </x:c>
       <x:c r="D27" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E27" s="19" t="n">
-        <x:v>46223.7403587963</x:v>
+        <x:v>46219.754375</x:v>
       </x:c>
       <x:c r="F27" s="14" t="n">
-        <x:v>493.92</x:v>
+        <x:v>434.59</x:v>
       </x:c>
       <x:c r="G27" s="18"/>
       <x:c r="H27" s="14"/>
@@ -2613,7 +2689,7 @@
         <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K27" s="14" t="n">
-        <x:v>493.92</x:v>
+        <x:v>434.59</x:v>
       </x:c>
       <x:c r="L27" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -2621,22 +2697,22 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
+        <x:v>Comercial IQL-NEXUS</x:v>
       </x:c>
       <x:c r="B28" s="18" t="n">
-        <x:v>2182299</x:v>
+        <x:v>2193205</x:v>
       </x:c>
       <x:c r="C28" s="13" t="n">
-        <x:v>15276</x:v>
+        <x:v>15324</x:v>
       </x:c>
       <x:c r="D28" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E28" s="19" t="n">
-        <x:v>46223.747824074075</x:v>
+        <x:v>46220.549305555556</x:v>
       </x:c>
       <x:c r="F28" s="14" t="n">
-        <x:v>364.03</x:v>
+        <x:v>1529.67</x:v>
       </x:c>
       <x:c r="G28" s="18"/>
       <x:c r="H28" s="14"/>
@@ -2645,7 +2721,7 @@
         <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K28" s="14" t="n">
-        <x:v>364.03</x:v>
+        <x:v>1529.67</x:v>
       </x:c>
       <x:c r="L28" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -2653,31 +2729,31 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="13" t="str">
-        <x:v>VINICIUS BERNARDES TEIXEIRA</x:v>
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
       </x:c>
       <x:c r="B29" s="18" t="n">
-        <x:v>2182658</x:v>
+        <x:v>2194690</x:v>
       </x:c>
       <x:c r="C29" s="13" t="n">
-        <x:v>15280</x:v>
+        <x:v>15337</x:v>
       </x:c>
       <x:c r="D29" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E29" s="19" t="n">
-        <x:v>46223.747824074075</x:v>
+        <x:v>46220.74028935185</x:v>
       </x:c>
       <x:c r="F29" s="14" t="n">
-        <x:v>112.77</x:v>
+        <x:v>164.17</x:v>
       </x:c>
       <x:c r="G29" s="18"/>
       <x:c r="H29" s="14"/>
       <x:c r="I29" s="19"/>
       <x:c r="J29" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K29" s="14" t="n">
-        <x:v>112.77</x:v>
+        <x:v>164.17</x:v>
       </x:c>
       <x:c r="L29" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -2685,31 +2761,31 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
+        <x:v>Roseli - Industria Portas</x:v>
       </x:c>
       <x:c r="B30" s="18" t="n">
-        <x:v>2192401</x:v>
+        <x:v>2196088</x:v>
       </x:c>
       <x:c r="C30" s="13" t="n">
-        <x:v>15318</x:v>
+        <x:v>15341</x:v>
       </x:c>
       <x:c r="D30" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E30" s="19" t="n">
-        <x:v>46223.76341435185</x:v>
+        <x:v>46223.494039351855</x:v>
       </x:c>
       <x:c r="F30" s="14" t="n">
-        <x:v>561.43</x:v>
+        <x:v>295.86</x:v>
       </x:c>
       <x:c r="G30" s="18"/>
       <x:c r="H30" s="14"/>
       <x:c r="I30" s="19"/>
       <x:c r="J30" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K30" s="14" t="n">
-        <x:v>561.43</x:v>
+        <x:v>295.86</x:v>
       </x:c>
       <x:c r="L30" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -2717,127 +2793,109 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="13" t="str">
-        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
+        <x:v>Fernanda Qualisol</x:v>
       </x:c>
       <x:c r="B31" s="18" t="n">
-        <x:v>2183959</x:v>
-      </x:c>
-      <x:c r="C31" s="13" t="n">
-        <x:v>15290</x:v>
-      </x:c>
+        <x:v>2178403</x:v>
+      </x:c>
+      <x:c r="C31" s="13" t="str"/>
       <x:c r="D31" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E31" s="19" t="n">
-        <x:v>46223.782789351855</x:v>
+        <x:v>46223.51357638889</x:v>
       </x:c>
       <x:c r="F31" s="14" t="n">
-        <x:v>381.23</x:v>
+        <x:v>417.36</x:v>
       </x:c>
       <x:c r="G31" s="18"/>
       <x:c r="H31" s="14"/>
       <x:c r="I31" s="19"/>
-      <x:c r="J31" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K31" s="14" t="n">
-        <x:v>381.23</x:v>
-      </x:c>
+      <x:c r="J31" s="13" t="str"/>
+      <x:c r="K31" s="14"/>
       <x:c r="L31" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="13" t="str">
-        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
+        <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B32" s="18" t="n">
-        <x:v>2182032</x:v>
-      </x:c>
-      <x:c r="C32" s="13" t="n">
-        <x:v>15172</x:v>
-      </x:c>
+        <x:v>2178451</x:v>
+      </x:c>
+      <x:c r="C32" s="13" t="str"/>
       <x:c r="D32" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E32" s="19" t="n">
-        <x:v>46223.784583333334</x:v>
+        <x:v>46223.54821759259</x:v>
       </x:c>
       <x:c r="F32" s="14" t="n">
-        <x:v>421.48</x:v>
+        <x:v>216.87</x:v>
       </x:c>
       <x:c r="G32" s="18"/>
       <x:c r="H32" s="14"/>
       <x:c r="I32" s="19"/>
-      <x:c r="J32" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
-      </x:c>
-      <x:c r="K32" s="14" t="n">
-        <x:v>2788.47</x:v>
-      </x:c>
+      <x:c r="J32" s="13" t="str"/>
+      <x:c r="K32" s="14"/>
       <x:c r="L32" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="13" t="str">
-        <x:v>Rosset Cia 2 Devoluções</x:v>
+        <x:v>Qualisol-Carol</x:v>
       </x:c>
       <x:c r="B33" s="18" t="n">
-        <x:v>2196879</x:v>
-      </x:c>
-      <x:c r="C33" s="13" t="n">
-        <x:v>15344</x:v>
-      </x:c>
+        <x:v>2178724</x:v>
+      </x:c>
+      <x:c r="C33" s="13" t="str"/>
       <x:c r="D33" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E33" s="19" t="n">
-        <x:v>46224.4844212963</x:v>
+        <x:v>46223.54821759259</x:v>
       </x:c>
       <x:c r="F33" s="14" t="n">
-        <x:v>927.98</x:v>
+        <x:v>555.5</x:v>
       </x:c>
       <x:c r="G33" s="18"/>
       <x:c r="H33" s="14"/>
       <x:c r="I33" s="19"/>
-      <x:c r="J33" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K33" s="14" t="n">
-        <x:v>927.98</x:v>
-      </x:c>
+      <x:c r="J33" s="13" t="str"/>
+      <x:c r="K33" s="14"/>
       <x:c r="L33" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="13" t="str">
-        <x:v>longo cadastro</x:v>
+        <x:v>Rosset Cia 2 Devoluções</x:v>
       </x:c>
       <x:c r="B34" s="18" t="n">
-        <x:v>2197779</x:v>
+        <x:v>2190103</x:v>
       </x:c>
       <x:c r="C34" s="13" t="n">
-        <x:v>15346</x:v>
+        <x:v>15300</x:v>
       </x:c>
       <x:c r="D34" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E34" s="19" t="n">
-        <x:v>46224.60364583333</x:v>
+        <x:v>46223.590682870374</x:v>
       </x:c>
       <x:c r="F34" s="14" t="n">
-        <x:v>2324.41</x:v>
+        <x:v>927.98</x:v>
       </x:c>
       <x:c r="G34" s="18"/>
       <x:c r="H34" s="14"/>
       <x:c r="I34" s="19"/>
       <x:c r="J34" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K34" s="14" t="n">
-        <x:v>2324.41</x:v>
+        <x:v>927.98</x:v>
       </x:c>
       <x:c r="L34" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -2845,153 +2903,141 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="13" t="str">
-        <x:v>Itamonte l +Luz Iluminação l Vanessa C.</x:v>
+        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
       </x:c>
       <x:c r="B35" s="18" t="n">
-        <x:v>2197933</x:v>
-      </x:c>
-      <x:c r="C35" s="13" t="n">
-        <x:v>15350</x:v>
-      </x:c>
+        <x:v>2178781</x:v>
+      </x:c>
+      <x:c r="C35" s="13" t="str"/>
       <x:c r="D35" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E35" s="19" t="n">
-        <x:v>46224.61032407408</x:v>
+        <x:v>46223.72690972222</x:v>
       </x:c>
       <x:c r="F35" s="14" t="n">
-        <x:v>244.8</x:v>
+        <x:v>236.1</x:v>
       </x:c>
       <x:c r="G35" s="18"/>
       <x:c r="H35" s="14"/>
       <x:c r="I35" s="19"/>
-      <x:c r="J35" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K35" s="14" t="n">
-        <x:v>244.8</x:v>
-      </x:c>
+      <x:c r="J35" s="13" t="str"/>
+      <x:c r="K35" s="14"/>
       <x:c r="L35" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA</x:v>
+        <x:v>Suplementos Equimaster</x:v>
       </x:c>
       <x:c r="B36" s="18" t="n">
-        <x:v>2198195</x:v>
-      </x:c>
-      <x:c r="C36" s="13" t="n">
-        <x:v>15349</x:v>
-      </x:c>
+        <x:v>2178953</x:v>
+      </x:c>
+      <x:c r="C36" s="13" t="str"/>
       <x:c r="D36" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E36" s="19" t="n">
-        <x:v>46224.73436342592</x:v>
+        <x:v>46223.72690972222</x:v>
       </x:c>
       <x:c r="F36" s="14" t="n">
-        <x:v>145.3</x:v>
+        <x:v>542.59</x:v>
       </x:c>
       <x:c r="G36" s="18"/>
       <x:c r="H36" s="14"/>
       <x:c r="I36" s="19"/>
-      <x:c r="J36" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K36" s="14" t="n">
-        <x:v>145.3</x:v>
-      </x:c>
+      <x:c r="J36" s="13" t="str"/>
+      <x:c r="K36" s="14"/>
       <x:c r="L36" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA</x:v>
+        <x:v>SUCOCITRICO CUTRALE LTDA</x:v>
       </x:c>
       <x:c r="B37" s="18" t="n">
-        <x:v>2198196</x:v>
-      </x:c>
-      <x:c r="C37" s="13" t="n">
-        <x:v>15353</x:v>
-      </x:c>
+        <x:v>2179159</x:v>
+      </x:c>
+      <x:c r="C37" s="13" t="str"/>
       <x:c r="D37" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E37" s="19" t="n">
-        <x:v>46224.73789351852</x:v>
+        <x:v>46223.72690972222</x:v>
       </x:c>
       <x:c r="F37" s="14" t="n">
-        <x:v>142.51</x:v>
+        <x:v>113.65</x:v>
       </x:c>
       <x:c r="G37" s="18"/>
       <x:c r="H37" s="14"/>
       <x:c r="I37" s="19"/>
-      <x:c r="J37" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K37" s="14" t="n">
-        <x:v>142.51</x:v>
-      </x:c>
+      <x:c r="J37" s="13" t="str"/>
+      <x:c r="K37" s="14"/>
       <x:c r="L37" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="13" t="str">
-        <x:v>Compras - Insertec Fornos e Refratários</x:v>
+        <x:v>MARCEL FACAS</x:v>
       </x:c>
       <x:c r="B38" s="18" t="n">
-        <x:v>2194633</x:v>
-      </x:c>
-      <x:c r="C38" s="13" t="str"/>
+        <x:v>2191327</x:v>
+      </x:c>
+      <x:c r="C38" s="13" t="n">
+        <x:v>15306</x:v>
+      </x:c>
       <x:c r="D38" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E38" s="19" t="n">
-        <x:v>46224.77175925926</x:v>
+        <x:v>46223.7403587963</x:v>
       </x:c>
       <x:c r="F38" s="14" t="n">
-        <x:v>311.03</x:v>
+        <x:v>255.51</x:v>
       </x:c>
       <x:c r="G38" s="18"/>
       <x:c r="H38" s="14"/>
       <x:c r="I38" s="19"/>
-      <x:c r="J38" s="13" t="str"/>
-      <x:c r="K38" s="14"/>
+      <x:c r="J38" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K38" s="14" t="n">
+        <x:v>255.51</x:v>
+      </x:c>
       <x:c r="L38" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="13" t="str">
-        <x:v>Fernanda Qualisol</x:v>
+        <x:v>Evelyn Brito</x:v>
       </x:c>
       <x:c r="B39" s="18" t="n">
-        <x:v>2198771</x:v>
+        <x:v>2191363</x:v>
       </x:c>
       <x:c r="C39" s="13" t="n">
-        <x:v>15357</x:v>
+        <x:v>15307</x:v>
       </x:c>
       <x:c r="D39" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E39" s="19" t="n">
-        <x:v>46225.53065972222</x:v>
+        <x:v>46223.7403587963</x:v>
       </x:c>
       <x:c r="F39" s="14" t="n">
-        <x:v>239.17</x:v>
+        <x:v>493.92</x:v>
       </x:c>
       <x:c r="G39" s="18"/>
       <x:c r="H39" s="14"/>
       <x:c r="I39" s="19"/>
       <x:c r="J39" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K39" s="14" t="n">
-        <x:v>239.17</x:v>
+        <x:v>493.92</x:v>
       </x:c>
       <x:c r="L39" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -2999,31 +3045,31 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="13" t="str">
-        <x:v>Fernanda Qualisol</x:v>
+        <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B40" s="18" t="n">
-        <x:v>2199721</x:v>
+        <x:v>2182299</x:v>
       </x:c>
       <x:c r="C40" s="13" t="n">
-        <x:v>15364</x:v>
+        <x:v>15276</x:v>
       </x:c>
       <x:c r="D40" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E40" s="19" t="n">
-        <x:v>46226.506423611114</x:v>
+        <x:v>46223.747824074075</x:v>
       </x:c>
       <x:c r="F40" s="14" t="n">
-        <x:v>283.27</x:v>
+        <x:v>364.03</x:v>
       </x:c>
       <x:c r="G40" s="18"/>
       <x:c r="H40" s="14"/>
       <x:c r="I40" s="19"/>
       <x:c r="J40" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K40" s="14" t="n">
-        <x:v>283.27</x:v>
+        <x:v>364.03</x:v>
       </x:c>
       <x:c r="L40" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3031,31 +3077,31 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA</x:v>
+        <x:v>VINICIUS BERNARDES TEIXEIRA</x:v>
       </x:c>
       <x:c r="B41" s="18" t="n">
-        <x:v>2199791</x:v>
+        <x:v>2182658</x:v>
       </x:c>
       <x:c r="C41" s="13" t="n">
-        <x:v>15365</x:v>
+        <x:v>15280</x:v>
       </x:c>
       <x:c r="D41" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E41" s="19" t="n">
-        <x:v>46226.51068287037</x:v>
+        <x:v>46223.747824074075</x:v>
       </x:c>
       <x:c r="F41" s="14" t="n">
-        <x:v>125.99</x:v>
+        <x:v>112.77</x:v>
       </x:c>
       <x:c r="G41" s="18"/>
       <x:c r="H41" s="14"/>
       <x:c r="I41" s="19"/>
       <x:c r="J41" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K41" s="14" t="n">
-        <x:v>125.99</x:v>
+        <x:v>112.77</x:v>
       </x:c>
       <x:c r="L41" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3063,20 +3109,20 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="13" t="str">
-        <x:v>IKTEC COMERCIO DE PROD PARA TRAT DE SUPERFICIE LTDA</x:v>
+        <x:v>Fernanda Qualisol</x:v>
       </x:c>
       <x:c r="B42" s="18" t="n">
-        <x:v>2199802</x:v>
+        <x:v>2181753</x:v>
       </x:c>
       <x:c r="C42" s="13" t="str"/>
       <x:c r="D42" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E42" s="19" t="n">
-        <x:v>46226.51582175926</x:v>
+        <x:v>46223.76222222222</x:v>
       </x:c>
       <x:c r="F42" s="14" t="n">
-        <x:v>158.2</x:v>
+        <x:v>554.5</x:v>
       </x:c>
       <x:c r="G42" s="18"/>
       <x:c r="H42" s="14"/>
@@ -3089,31 +3135,31 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="13" t="str">
-        <x:v>BAUTECH INDUSTRIA E COMERCIO DE TINTAS LTDA</x:v>
+        <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B43" s="18" t="n">
-        <x:v>2199976</x:v>
+        <x:v>2192401</x:v>
       </x:c>
       <x:c r="C43" s="13" t="n">
-        <x:v>15369</x:v>
+        <x:v>15318</x:v>
       </x:c>
       <x:c r="D43" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E43" s="19" t="n">
-        <x:v>46226.614375</x:v>
+        <x:v>46223.76341435185</x:v>
       </x:c>
       <x:c r="F43" s="14" t="n">
-        <x:v>1301.93</x:v>
+        <x:v>561.43</x:v>
       </x:c>
       <x:c r="G43" s="18"/>
       <x:c r="H43" s="14"/>
       <x:c r="I43" s="19"/>
       <x:c r="J43" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K43" s="14" t="n">
-        <x:v>1301.93</x:v>
+        <x:v>561.43</x:v>
       </x:c>
       <x:c r="L43" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3121,31 +3167,31 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="13" t="str">
-        <x:v>GASPAR COMERCIO DE EQUIPAMENTOS E UTENSILIOS LTDA</x:v>
+        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
       </x:c>
       <x:c r="B44" s="18" t="n">
-        <x:v>2199927</x:v>
+        <x:v>2183959</x:v>
       </x:c>
       <x:c r="C44" s="13" t="n">
-        <x:v>15368</x:v>
+        <x:v>15290</x:v>
       </x:c>
       <x:c r="D44" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E44" s="19" t="n">
-        <x:v>46226.76988425926</x:v>
+        <x:v>46223.782789351855</x:v>
       </x:c>
       <x:c r="F44" s="14" t="n">
-        <x:v>298.53</x:v>
+        <x:v>381.23</x:v>
       </x:c>
       <x:c r="G44" s="18"/>
       <x:c r="H44" s="14"/>
       <x:c r="I44" s="19"/>
       <x:c r="J44" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K44" s="14" t="n">
-        <x:v>298.53</x:v>
+        <x:v>381.23</x:v>
       </x:c>
       <x:c r="L44" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3153,31 +3199,31 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="13" t="str">
-        <x:v>Fernanda Qualisol</x:v>
+        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
       </x:c>
       <x:c r="B45" s="18" t="n">
-        <x:v>2202021</x:v>
+        <x:v>2182032</x:v>
       </x:c>
       <x:c r="C45" s="13" t="n">
-        <x:v>15376</x:v>
+        <x:v>15172</x:v>
       </x:c>
       <x:c r="D45" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E45" s="19" t="n">
-        <x:v>46227.641180555554</x:v>
+        <x:v>46223.784583333334</x:v>
       </x:c>
       <x:c r="F45" s="14" t="n">
-        <x:v>474.57</x:v>
+        <x:v>421.48</x:v>
       </x:c>
       <x:c r="G45" s="18"/>
       <x:c r="H45" s="14"/>
       <x:c r="I45" s="19"/>
       <x:c r="J45" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K45" s="14" t="n">
-        <x:v>474.57</x:v>
+        <x:v>2788.47</x:v>
       </x:c>
       <x:c r="L45" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3185,31 +3231,31 @@
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="13" t="str">
-        <x:v>ACRILICOS BRASIL LTDA</x:v>
+        <x:v>Rosset Cia 2 Devoluções</x:v>
       </x:c>
       <x:c r="B46" s="18" t="n">
-        <x:v>2182262</x:v>
+        <x:v>2196879</x:v>
       </x:c>
       <x:c r="C46" s="13" t="n">
-        <x:v>15275</x:v>
+        <x:v>15344</x:v>
       </x:c>
       <x:c r="D46" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E46" s="19" t="n">
-        <x:v>46227.72767361111</x:v>
+        <x:v>46224.4844212963</x:v>
       </x:c>
       <x:c r="F46" s="14" t="n">
-        <x:v>2456.75</x:v>
+        <x:v>927.98</x:v>
       </x:c>
       <x:c r="G46" s="18"/>
       <x:c r="H46" s="14"/>
       <x:c r="I46" s="19"/>
       <x:c r="J46" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K46" s="14" t="n">
-        <x:v>2456.75</x:v>
+        <x:v>927.98</x:v>
       </x:c>
       <x:c r="L46" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3217,31 +3263,31 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="13" t="str">
-        <x:v>BAUTECH INDUSTRIA E COMERCIO DE TINTAS LTDA</x:v>
+        <x:v>longo cadastro</x:v>
       </x:c>
       <x:c r="B47" s="18" t="n">
-        <x:v>2183475</x:v>
+        <x:v>2197779</x:v>
       </x:c>
       <x:c r="C47" s="13" t="n">
-        <x:v>15284</x:v>
+        <x:v>15346</x:v>
       </x:c>
       <x:c r="D47" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E47" s="19" t="n">
-        <x:v>46227.737916666665</x:v>
+        <x:v>46224.60364583333</x:v>
       </x:c>
       <x:c r="F47" s="14" t="n">
-        <x:v>4382.37</x:v>
+        <x:v>2324.41</x:v>
       </x:c>
       <x:c r="G47" s="18"/>
       <x:c r="H47" s="14"/>
       <x:c r="I47" s="19"/>
       <x:c r="J47" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K47" s="14" t="n">
-        <x:v>4382.37</x:v>
+        <x:v>2324.41</x:v>
       </x:c>
       <x:c r="L47" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3249,31 +3295,31 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="13" t="str">
-        <x:v>Camila</x:v>
+        <x:v>Itamonte l +Luz Iluminação l Vanessa C.</x:v>
       </x:c>
       <x:c r="B48" s="18" t="n">
-        <x:v>2190174</x:v>
+        <x:v>2197933</x:v>
       </x:c>
       <x:c r="C48" s="13" t="n">
-        <x:v>15301</x:v>
+        <x:v>15350</x:v>
       </x:c>
       <x:c r="D48" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E48" s="19" t="n">
-        <x:v>46227.737916666665</x:v>
+        <x:v>46224.61032407408</x:v>
       </x:c>
       <x:c r="F48" s="14" t="n">
-        <x:v>2365.26</x:v>
+        <x:v>244.8</x:v>
       </x:c>
       <x:c r="G48" s="18"/>
       <x:c r="H48" s="14"/>
       <x:c r="I48" s="19"/>
       <x:c r="J48" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K48" s="14" t="n">
-        <x:v>2365.26</x:v>
+        <x:v>244.8</x:v>
       </x:c>
       <x:c r="L48" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3281,31 +3327,31 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="13" t="str">
-        <x:v>Bprint Gráfica</x:v>
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA</x:v>
       </x:c>
       <x:c r="B49" s="18" t="n">
-        <x:v>2198394</x:v>
+        <x:v>2198195</x:v>
       </x:c>
       <x:c r="C49" s="13" t="n">
-        <x:v>15356</x:v>
+        <x:v>15349</x:v>
       </x:c>
       <x:c r="D49" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E49" s="19" t="n">
-        <x:v>46230.57780092592</x:v>
+        <x:v>46224.73436342592</x:v>
       </x:c>
       <x:c r="F49" s="14" t="n">
-        <x:v>1185.24</x:v>
+        <x:v>145.3</x:v>
       </x:c>
       <x:c r="G49" s="18"/>
       <x:c r="H49" s="14"/>
       <x:c r="I49" s="19"/>
       <x:c r="J49" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K49" s="14" t="n">
-        <x:v>1185.24</x:v>
+        <x:v>145.3</x:v>
       </x:c>
       <x:c r="L49" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3313,31 +3359,31 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA</x:v>
       </x:c>
       <x:c r="B50" s="18" t="n">
-        <x:v>2191606</x:v>
+        <x:v>2198196</x:v>
       </x:c>
       <x:c r="C50" s="13" t="n">
-        <x:v>15308</x:v>
+        <x:v>15353</x:v>
       </x:c>
       <x:c r="D50" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E50" s="19" t="n">
-        <x:v>46230.67396990741</x:v>
+        <x:v>46224.73789351852</x:v>
       </x:c>
       <x:c r="F50" s="14" t="n">
-        <x:v>160.75</x:v>
+        <x:v>142.51</x:v>
       </x:c>
       <x:c r="G50" s="18"/>
       <x:c r="H50" s="14"/>
       <x:c r="I50" s="19"/>
       <x:c r="J50" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K50" s="14" t="n">
-        <x:v>160.75</x:v>
+        <x:v>142.51</x:v>
       </x:c>
       <x:c r="L50" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3345,54 +3391,48 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="13" t="str">
-        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
+        <x:v>Compras - Insertec Fornos e Refratários</x:v>
       </x:c>
       <x:c r="B51" s="18" t="n">
-        <x:v>2204541</x:v>
-      </x:c>
-      <x:c r="C51" s="13" t="n">
-        <x:v>15383</x:v>
-      </x:c>
+        <x:v>2194633</x:v>
+      </x:c>
+      <x:c r="C51" s="13" t="str"/>
       <x:c r="D51" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E51" s="19" t="n">
-        <x:v>46230.775509259256</x:v>
+        <x:v>46224.77175925926</x:v>
       </x:c>
       <x:c r="F51" s="14" t="n">
-        <x:v>463.98</x:v>
+        <x:v>311.03</x:v>
       </x:c>
       <x:c r="G51" s="18"/>
       <x:c r="H51" s="14"/>
       <x:c r="I51" s="19"/>
-      <x:c r="J51" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K51" s="14" t="n">
-        <x:v>463.98</x:v>
-      </x:c>
+      <x:c r="J51" s="13" t="str"/>
+      <x:c r="K51" s="14"/>
       <x:c r="L51" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="13" t="str">
-        <x:v>Carmaço - Fiori</x:v>
+        <x:v>Fernanda Qualisol</x:v>
       </x:c>
       <x:c r="B52" s="18" t="n">
-        <x:v>2204551</x:v>
+        <x:v>2198771</x:v>
       </x:c>
       <x:c r="C52" s="13" t="n">
-        <x:v>15384</x:v>
+        <x:v>15357</x:v>
       </x:c>
       <x:c r="D52" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E52" s="19" t="n">
-        <x:v>46230.77912037037</x:v>
+        <x:v>46225.53065972222</x:v>
       </x:c>
       <x:c r="F52" s="14" t="n">
-        <x:v>401.75</x:v>
+        <x:v>239.17</x:v>
       </x:c>
       <x:c r="G52" s="18"/>
       <x:c r="H52" s="14"/>
@@ -3401,7 +3441,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K52" s="14" t="n">
-        <x:v>401.75</x:v>
+        <x:v>239.17</x:v>
       </x:c>
       <x:c r="L52" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3409,22 +3449,22 @@
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
+        <x:v>Fernanda Qualisol</x:v>
       </x:c>
       <x:c r="B53" s="18" t="n">
-        <x:v>2204675</x:v>
+        <x:v>2199721</x:v>
       </x:c>
       <x:c r="C53" s="13" t="n">
-        <x:v>15386</x:v>
+        <x:v>15364</x:v>
       </x:c>
       <x:c r="D53" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E53" s="19" t="n">
-        <x:v>46230.79717592592</x:v>
+        <x:v>46226.506423611114</x:v>
       </x:c>
       <x:c r="F53" s="14" t="n">
-        <x:v>1290.83</x:v>
+        <x:v>283.27</x:v>
       </x:c>
       <x:c r="G53" s="18"/>
       <x:c r="H53" s="14"/>
@@ -3433,7 +3473,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K53" s="14" t="n">
-        <x:v>1290.83</x:v>
+        <x:v>283.27</x:v>
       </x:c>
       <x:c r="L53" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3441,22 +3481,22 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="13" t="str">
-        <x:v>Qualidade Almad</x:v>
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA</x:v>
       </x:c>
       <x:c r="B54" s="18" t="n">
-        <x:v>2204714</x:v>
+        <x:v>2199791</x:v>
       </x:c>
       <x:c r="C54" s="13" t="n">
-        <x:v>15387</x:v>
+        <x:v>15365</x:v>
       </x:c>
       <x:c r="D54" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E54" s="19" t="n">
-        <x:v>46231.45103009259</x:v>
+        <x:v>46226.51068287037</x:v>
       </x:c>
       <x:c r="F54" s="14" t="n">
-        <x:v>2370.92</x:v>
+        <x:v>125.99</x:v>
       </x:c>
       <x:c r="G54" s="18"/>
       <x:c r="H54" s="14"/>
@@ -3465,7 +3505,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K54" s="14" t="n">
-        <x:v>2370.92</x:v>
+        <x:v>125.99</x:v>
       </x:c>
       <x:c r="L54" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3473,54 +3513,48 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="13" t="str">
-        <x:v>Transporte Bautech</x:v>
+        <x:v>IKTEC COMERCIO DE PROD PARA TRAT DE SUPERFICIE LTDA</x:v>
       </x:c>
       <x:c r="B55" s="18" t="n">
-        <x:v>2205200</x:v>
-      </x:c>
-      <x:c r="C55" s="13" t="n">
-        <x:v>15388</x:v>
-      </x:c>
+        <x:v>2199802</x:v>
+      </x:c>
+      <x:c r="C55" s="13" t="str"/>
       <x:c r="D55" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E55" s="19" t="n">
-        <x:v>46231.503171296295</x:v>
+        <x:v>46226.51582175926</x:v>
       </x:c>
       <x:c r="F55" s="14" t="n">
-        <x:v>505.68</x:v>
+        <x:v>158.2</x:v>
       </x:c>
       <x:c r="G55" s="18"/>
       <x:c r="H55" s="14"/>
       <x:c r="I55" s="19"/>
-      <x:c r="J55" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K55" s="14" t="n">
-        <x:v>505.68</x:v>
-      </x:c>
+      <x:c r="J55" s="13" t="str"/>
+      <x:c r="K55" s="14"/>
       <x:c r="L55" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
+        <x:v>BAUTECH INDUSTRIA E COMERCIO DE TINTAS LTDA</x:v>
       </x:c>
       <x:c r="B56" s="18" t="n">
-        <x:v>2205354</x:v>
+        <x:v>2199976</x:v>
       </x:c>
       <x:c r="C56" s="13" t="n">
-        <x:v>15394</x:v>
+        <x:v>15369</x:v>
       </x:c>
       <x:c r="D56" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E56" s="19" t="n">
-        <x:v>46231.60502314815</x:v>
+        <x:v>46226.614375</x:v>
       </x:c>
       <x:c r="F56" s="14" t="n">
-        <x:v>173.06</x:v>
+        <x:v>1301.93</x:v>
       </x:c>
       <x:c r="G56" s="18"/>
       <x:c r="H56" s="14"/>
@@ -3529,7 +3563,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K56" s="14" t="n">
-        <x:v>173.06</x:v>
+        <x:v>1301.93</x:v>
       </x:c>
       <x:c r="L56" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3537,22 +3571,22 @@
     </x:row>
     <x:row r="57">
       <x:c r="A57" s="13" t="str">
-        <x:v>Metal Max</x:v>
+        <x:v>GASPAR COMERCIO DE EQUIPAMENTOS E UTENSILIOS LTDA</x:v>
       </x:c>
       <x:c r="B57" s="18" t="n">
-        <x:v>2205212</x:v>
+        <x:v>2199927</x:v>
       </x:c>
       <x:c r="C57" s="13" t="n">
-        <x:v>15392</x:v>
+        <x:v>15368</x:v>
       </x:c>
       <x:c r="D57" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E57" s="19" t="n">
-        <x:v>46231.68457175926</x:v>
+        <x:v>46226.76988425926</x:v>
       </x:c>
       <x:c r="F57" s="14" t="n">
-        <x:v>215.53</x:v>
+        <x:v>298.53</x:v>
       </x:c>
       <x:c r="G57" s="18"/>
       <x:c r="H57" s="14"/>
@@ -3561,7 +3595,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K57" s="14" t="n">
-        <x:v>215.53</x:v>
+        <x:v>298.53</x:v>
       </x:c>
       <x:c r="L57" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3569,22 +3603,22 @@
     </x:row>
     <x:row r="58">
       <x:c r="A58" s="13" t="str">
-        <x:v>Eder Fazzi</x:v>
+        <x:v>Fernanda Qualisol</x:v>
       </x:c>
       <x:c r="B58" s="18" t="n">
-        <x:v>2205493</x:v>
+        <x:v>2202021</x:v>
       </x:c>
       <x:c r="C58" s="13" t="n">
-        <x:v>15395</x:v>
+        <x:v>15376</x:v>
       </x:c>
       <x:c r="D58" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E58" s="19" t="n">
-        <x:v>46231.69190972222</x:v>
+        <x:v>46227.641180555554</x:v>
       </x:c>
       <x:c r="F58" s="14" t="n">
-        <x:v>1419.63</x:v>
+        <x:v>474.57</x:v>
       </x:c>
       <x:c r="G58" s="18"/>
       <x:c r="H58" s="14"/>
@@ -3593,7 +3627,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K58" s="14" t="n">
-        <x:v>1419.63</x:v>
+        <x:v>474.57</x:v>
       </x:c>
       <x:c r="L58" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3601,54 +3635,48 @@
     </x:row>
     <x:row r="59">
       <x:c r="A59" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
+        <x:v>Militão</x:v>
       </x:c>
       <x:c r="B59" s="18" t="n">
-        <x:v>2205218</x:v>
-      </x:c>
-      <x:c r="C59" s="13" t="n">
-        <x:v>15390</x:v>
-      </x:c>
+        <x:v>2177975</x:v>
+      </x:c>
+      <x:c r="C59" s="13" t="str"/>
       <x:c r="D59" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E59" s="19" t="n">
-        <x:v>46231.71363425926</x:v>
+        <x:v>46227.72767361111</x:v>
       </x:c>
       <x:c r="F59" s="14" t="n">
-        <x:v>169.45</x:v>
+        <x:v>400.72</x:v>
       </x:c>
       <x:c r="G59" s="18"/>
       <x:c r="H59" s="14"/>
       <x:c r="I59" s="19"/>
-      <x:c r="J59" s="13" t="str">
-        <x:v>ABERTA</x:v>
-      </x:c>
-      <x:c r="K59" s="14" t="n">
-        <x:v>169.45</x:v>
-      </x:c>
+      <x:c r="J59" s="13" t="str"/>
+      <x:c r="K59" s="14"/>
       <x:c r="L59" s="20" t="str">
-        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
       <x:c r="A60" s="13" t="str">
-        <x:v>Osni - Molina Freios</x:v>
+        <x:v>ACRILICOS BRASIL LTDA</x:v>
       </x:c>
       <x:c r="B60" s="18" t="n">
-        <x:v>2201892</x:v>
+        <x:v>2182262</x:v>
       </x:c>
       <x:c r="C60" s="13" t="n">
-        <x:v>15373</x:v>
+        <x:v>15275</x:v>
       </x:c>
       <x:c r="D60" s="13" t="str">
         <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E60" s="19" t="n">
-        <x:v>46231.74150462963</x:v>
+        <x:v>46227.72767361111</x:v>
       </x:c>
       <x:c r="F60" s="14" t="n">
-        <x:v>155.98</x:v>
+        <x:v>2456.75</x:v>
       </x:c>
       <x:c r="G60" s="18"/>
       <x:c r="H60" s="14"/>
@@ -3657,7 +3685,7 @@
         <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K60" s="14" t="n">
-        <x:v>155.98</x:v>
+        <x:v>2456.75</x:v>
       </x:c>
       <x:c r="L60" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3665,31 +3693,31 @@
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="13" t="str">
-        <x:v>Thomas Estoque R Imper</x:v>
+        <x:v>BAUTECH INDUSTRIA E COMERCIO DE TINTAS LTDA</x:v>
       </x:c>
       <x:c r="B61" s="18" t="n">
-        <x:v>2205687</x:v>
+        <x:v>2183475</x:v>
       </x:c>
       <x:c r="C61" s="13" t="n">
-        <x:v>15397</x:v>
+        <x:v>15284</x:v>
       </x:c>
       <x:c r="D61" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E61" s="19" t="n">
-        <x:v>46231.78642361111</x:v>
+        <x:v>46227.737916666665</x:v>
       </x:c>
       <x:c r="F61" s="14" t="n">
-        <x:v>1806.4</x:v>
+        <x:v>4382.37</x:v>
       </x:c>
       <x:c r="G61" s="18"/>
       <x:c r="H61" s="14"/>
       <x:c r="I61" s="19"/>
       <x:c r="J61" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K61" s="14" t="n">
-        <x:v>1806.4</x:v>
+        <x:v>4382.37</x:v>
       </x:c>
       <x:c r="L61" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3697,31 +3725,31 @@
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="13" t="str">
-        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
+        <x:v>Camila</x:v>
       </x:c>
       <x:c r="B62" s="18" t="n">
-        <x:v>2206185</x:v>
+        <x:v>2190174</x:v>
       </x:c>
       <x:c r="C62" s="13" t="n">
-        <x:v>15401</x:v>
+        <x:v>15301</x:v>
       </x:c>
       <x:c r="D62" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E62" s="19" t="n">
-        <x:v>46232.56662037037</x:v>
+        <x:v>46227.737916666665</x:v>
       </x:c>
       <x:c r="F62" s="14" t="n">
-        <x:v>599.35</x:v>
+        <x:v>2365.26</x:v>
       </x:c>
       <x:c r="G62" s="18"/>
       <x:c r="H62" s="14"/>
       <x:c r="I62" s="19"/>
       <x:c r="J62" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K62" s="14" t="n">
-        <x:v>599.35</x:v>
+        <x:v>2365.26</x:v>
       </x:c>
       <x:c r="L62" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3729,31 +3757,31 @@
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
+        <x:v>Bprint Gráfica</x:v>
       </x:c>
       <x:c r="B63" s="18" t="n">
-        <x:v>2205674</x:v>
+        <x:v>2198394</x:v>
       </x:c>
       <x:c r="C63" s="13" t="n">
-        <x:v>15402</x:v>
+        <x:v>15356</x:v>
       </x:c>
       <x:c r="D63" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E63" s="19" t="n">
-        <x:v>46232.57876157408</x:v>
+        <x:v>46230.57780092592</x:v>
       </x:c>
       <x:c r="F63" s="14" t="n">
-        <x:v>2173.95</x:v>
+        <x:v>1185.24</x:v>
       </x:c>
       <x:c r="G63" s="18"/>
       <x:c r="H63" s="14"/>
       <x:c r="I63" s="19"/>
       <x:c r="J63" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K63" s="14" t="n">
-        <x:v>2173.95</x:v>
+        <x:v>1185.24</x:v>
       </x:c>
       <x:c r="L63" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3761,31 +3789,31 @@
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
       </x:c>
       <x:c r="B64" s="18" t="n">
-        <x:v>2206284</x:v>
+        <x:v>2191606</x:v>
       </x:c>
       <x:c r="C64" s="13" t="n">
-        <x:v>15405</x:v>
+        <x:v>15308</x:v>
       </x:c>
       <x:c r="D64" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E64" s="19" t="n">
-        <x:v>46232.59909722222</x:v>
+        <x:v>46230.67396990741</x:v>
       </x:c>
       <x:c r="F64" s="14" t="n">
-        <x:v>568.61</x:v>
+        <x:v>160.75</x:v>
       </x:c>
       <x:c r="G64" s="18"/>
       <x:c r="H64" s="14"/>
       <x:c r="I64" s="19"/>
       <x:c r="J64" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K64" s="14" t="n">
-        <x:v>568.61</x:v>
+        <x:v>160.75</x:v>
       </x:c>
       <x:c r="L64" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3793,22 +3821,22 @@
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
+        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
       </x:c>
       <x:c r="B65" s="18" t="n">
-        <x:v>2206293</x:v>
+        <x:v>2204541</x:v>
       </x:c>
       <x:c r="C65" s="13" t="n">
-        <x:v>15406</x:v>
+        <x:v>15383</x:v>
       </x:c>
       <x:c r="D65" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E65" s="19" t="n">
-        <x:v>46232.60854166667</x:v>
+        <x:v>46230.775509259256</x:v>
       </x:c>
       <x:c r="F65" s="14" t="n">
-        <x:v>454.22</x:v>
+        <x:v>463.98</x:v>
       </x:c>
       <x:c r="G65" s="18"/>
       <x:c r="H65" s="14"/>
@@ -3817,7 +3845,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K65" s="14" t="n">
-        <x:v>454.22</x:v>
+        <x:v>463.98</x:v>
       </x:c>
       <x:c r="L65" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3825,22 +3853,22 @@
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
+        <x:v>Carmaço - Fiori</x:v>
       </x:c>
       <x:c r="B66" s="18" t="n">
-        <x:v>2206603</x:v>
+        <x:v>2204551</x:v>
       </x:c>
       <x:c r="C66" s="13" t="n">
-        <x:v>15408</x:v>
+        <x:v>15384</x:v>
       </x:c>
       <x:c r="D66" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E66" s="19" t="n">
-        <x:v>46232.799525462964</x:v>
+        <x:v>46230.77912037037</x:v>
       </x:c>
       <x:c r="F66" s="14" t="n">
-        <x:v>124.44</x:v>
+        <x:v>401.75</x:v>
       </x:c>
       <x:c r="G66" s="18"/>
       <x:c r="H66" s="14"/>
@@ -3849,7 +3877,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K66" s="14" t="n">
-        <x:v>124.44</x:v>
+        <x:v>401.75</x:v>
       </x:c>
       <x:c r="L66" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3857,22 +3885,22 @@
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="13" t="str">
-        <x:v>Vinilak Tintas Especiais</x:v>
+        <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B67" s="18" t="n">
-        <x:v>2207138</x:v>
+        <x:v>2204675</x:v>
       </x:c>
       <x:c r="C67" s="13" t="n">
-        <x:v>15412</x:v>
+        <x:v>15386</x:v>
       </x:c>
       <x:c r="D67" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E67" s="19" t="n">
-        <x:v>46233.56369212963</x:v>
+        <x:v>46230.79717592592</x:v>
       </x:c>
       <x:c r="F67" s="14" t="n">
-        <x:v>503.59</x:v>
+        <x:v>1290.83</x:v>
       </x:c>
       <x:c r="G67" s="18"/>
       <x:c r="H67" s="14"/>
@@ -3881,7 +3909,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K67" s="14" t="n">
-        <x:v>503.59</x:v>
+        <x:v>1290.83</x:v>
       </x:c>
       <x:c r="L67" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3889,22 +3917,22 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="13" t="str">
-        <x:v>João Pedro | Bprint Gráfica</x:v>
+        <x:v>Qualidade Almad</x:v>
       </x:c>
       <x:c r="B68" s="18" t="n">
-        <x:v>2207378</x:v>
+        <x:v>2204714</x:v>
       </x:c>
       <x:c r="C68" s="13" t="n">
-        <x:v>15414</x:v>
+        <x:v>15387</x:v>
       </x:c>
       <x:c r="D68" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E68" s="19" t="n">
-        <x:v>46233.572060185186</x:v>
+        <x:v>46231.45103009259</x:v>
       </x:c>
       <x:c r="F68" s="14" t="n">
-        <x:v>430.25</x:v>
+        <x:v>2370.92</x:v>
       </x:c>
       <x:c r="G68" s="18"/>
       <x:c r="H68" s="14"/>
@@ -3913,7 +3941,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K68" s="14" t="n">
-        <x:v>430.25</x:v>
+        <x:v>2370.92</x:v>
       </x:c>
       <x:c r="L68" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3921,22 +3949,22 @@
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="13" t="str">
-        <x:v>Carmaço - Fiori</x:v>
+        <x:v>Transporte Bautech</x:v>
       </x:c>
       <x:c r="B69" s="18" t="n">
-        <x:v>2207562</x:v>
+        <x:v>2205200</x:v>
       </x:c>
       <x:c r="C69" s="13" t="n">
-        <x:v>15417</x:v>
+        <x:v>15388</x:v>
       </x:c>
       <x:c r="D69" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E69" s="19" t="n">
-        <x:v>46233.67563657407</x:v>
+        <x:v>46231.503171296295</x:v>
       </x:c>
       <x:c r="F69" s="14" t="n">
-        <x:v>390.31</x:v>
+        <x:v>505.68</x:v>
       </x:c>
       <x:c r="G69" s="18"/>
       <x:c r="H69" s="14"/>
@@ -3945,7 +3973,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K69" s="14" t="n">
-        <x:v>390.31</x:v>
+        <x:v>505.68</x:v>
       </x:c>
       <x:c r="L69" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3953,22 +3981,22 @@
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="13" t="str">
-        <x:v>Queren Cyrino</x:v>
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
       </x:c>
       <x:c r="B70" s="18" t="n">
-        <x:v>2207563</x:v>
+        <x:v>2205354</x:v>
       </x:c>
       <x:c r="C70" s="13" t="n">
-        <x:v>15419</x:v>
+        <x:v>15394</x:v>
       </x:c>
       <x:c r="D70" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E70" s="19" t="n">
-        <x:v>46233.69023148148</x:v>
+        <x:v>46231.60502314815</x:v>
       </x:c>
       <x:c r="F70" s="14" t="n">
-        <x:v>1168.34</x:v>
+        <x:v>173.06</x:v>
       </x:c>
       <x:c r="G70" s="18"/>
       <x:c r="H70" s="14"/>
@@ -3977,7 +4005,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K70" s="14" t="n">
-        <x:v>1168.34</x:v>
+        <x:v>173.06</x:v>
       </x:c>
       <x:c r="L70" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -3985,57 +4013,63 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="13" t="str">
-        <x:v>WOOD COLOR TINTAS</x:v>
+        <x:v>Metal Max</x:v>
       </x:c>
       <x:c r="B71" s="18" t="n">
-        <x:v>2207637</x:v>
-      </x:c>
-      <x:c r="C71" s="13" t="str"/>
+        <x:v>2205212</x:v>
+      </x:c>
+      <x:c r="C71" s="13" t="n">
+        <x:v>15392</x:v>
+      </x:c>
       <x:c r="D71" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E71" s="19" t="n">
-        <x:v>46233.700266203705</x:v>
+        <x:v>46231.68457175926</x:v>
       </x:c>
       <x:c r="F71" s="14" t="n">
-        <x:v>404.88</x:v>
+        <x:v>215.53</x:v>
       </x:c>
       <x:c r="G71" s="18"/>
       <x:c r="H71" s="14"/>
       <x:c r="I71" s="19"/>
-      <x:c r="J71" s="13" t="str"/>
-      <x:c r="K71" s="14"/>
+      <x:c r="J71" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K71" s="14" t="n">
+        <x:v>215.53</x:v>
+      </x:c>
       <x:c r="L71" s="20" t="str">
-        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="13" t="str">
-        <x:v>Juciliana</x:v>
+        <x:v>Eder Fazzi</x:v>
       </x:c>
       <x:c r="B72" s="18" t="n">
-        <x:v>2206455</x:v>
+        <x:v>2205493</x:v>
       </x:c>
       <x:c r="C72" s="13" t="n">
-        <x:v>15407</x:v>
+        <x:v>15395</x:v>
       </x:c>
       <x:c r="D72" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E72" s="19" t="n">
-        <x:v>46233.70322916667</x:v>
+        <x:v>46231.69190972222</x:v>
       </x:c>
       <x:c r="F72" s="14" t="n">
-        <x:v>251.25</x:v>
+        <x:v>1419.63</x:v>
       </x:c>
       <x:c r="G72" s="18"/>
       <x:c r="H72" s="14"/>
       <x:c r="I72" s="19"/>
       <x:c r="J72" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K72" s="14" t="n">
-        <x:v>251.25</x:v>
+        <x:v>1419.63</x:v>
       </x:c>
       <x:c r="L72" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4043,22 +4077,22 @@
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="13" t="str">
-        <x:v>FRANCHI NORTE DISTRIBUICAO LTDA</x:v>
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
       </x:c>
       <x:c r="B73" s="18" t="n">
-        <x:v>2205563</x:v>
+        <x:v>2205218</x:v>
       </x:c>
       <x:c r="C73" s="13" t="n">
-        <x:v>15396</x:v>
+        <x:v>15390</x:v>
       </x:c>
       <x:c r="D73" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E73" s="19" t="n">
-        <x:v>46233.765810185185</x:v>
+        <x:v>46231.71363425926</x:v>
       </x:c>
       <x:c r="F73" s="14" t="n">
-        <x:v>250.89</x:v>
+        <x:v>169.45</x:v>
       </x:c>
       <x:c r="G73" s="18"/>
       <x:c r="H73" s="14"/>
@@ -4067,7 +4101,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K73" s="14" t="n">
-        <x:v>250.89</x:v>
+        <x:v>169.45</x:v>
       </x:c>
       <x:c r="L73" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4075,31 +4109,31 @@
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="13" t="str">
-        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
+        <x:v>Osni - Molina Freios</x:v>
       </x:c>
       <x:c r="B74" s="18" t="n">
-        <x:v>2208212</x:v>
+        <x:v>2201892</x:v>
       </x:c>
       <x:c r="C74" s="13" t="n">
-        <x:v>15421</x:v>
+        <x:v>15373</x:v>
       </x:c>
       <x:c r="D74" s="13" t="str">
-        <x:v>Aberto</x:v>
+        <x:v>Perdido</x:v>
       </x:c>
       <x:c r="E74" s="19" t="n">
-        <x:v>46234.513715277775</x:v>
+        <x:v>46231.74150462963</x:v>
       </x:c>
       <x:c r="F74" s="14" t="n">
-        <x:v>142.51</x:v>
+        <x:v>155.98</x:v>
       </x:c>
       <x:c r="G74" s="18"/>
       <x:c r="H74" s="14"/>
       <x:c r="I74" s="19"/>
       <x:c r="J74" s="13" t="str">
-        <x:v>ABERTA</x:v>
+        <x:v>NÃO APROVADA</x:v>
       </x:c>
       <x:c r="K74" s="14" t="n">
-        <x:v>142.51</x:v>
+        <x:v>155.98</x:v>
       </x:c>
       <x:c r="L74" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4107,22 +4141,22 @@
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="13" t="str">
-        <x:v>Elisete Henck</x:v>
+        <x:v>Thomas Estoque R Imper</x:v>
       </x:c>
       <x:c r="B75" s="18" t="n">
-        <x:v>2208349</x:v>
+        <x:v>2205687</x:v>
       </x:c>
       <x:c r="C75" s="13" t="n">
-        <x:v>15423</x:v>
+        <x:v>15397</x:v>
       </x:c>
       <x:c r="D75" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E75" s="19" t="n">
-        <x:v>46234.616793981484</x:v>
+        <x:v>46231.78642361111</x:v>
       </x:c>
       <x:c r="F75" s="14" t="n">
-        <x:v>107.37</x:v>
+        <x:v>1806.4</x:v>
       </x:c>
       <x:c r="G75" s="18"/>
       <x:c r="H75" s="14"/>
@@ -4131,7 +4165,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K75" s="14" t="n">
-        <x:v>107.37</x:v>
+        <x:v>1806.4</x:v>
       </x:c>
       <x:c r="L75" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4139,31 +4173,31 @@
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="13" t="str">
-        <x:v>Logistica</x:v>
+        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
       </x:c>
       <x:c r="B76" s="18" t="n">
-        <x:v>2191659</x:v>
+        <x:v>2206185</x:v>
       </x:c>
       <x:c r="C76" s="13" t="n">
-        <x:v>15317</x:v>
+        <x:v>15401</x:v>
       </x:c>
       <x:c r="D76" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E76" s="19" t="n">
-        <x:v>46234.67115740741</x:v>
+        <x:v>46232.56662037037</x:v>
       </x:c>
       <x:c r="F76" s="14" t="n">
-        <x:v>276.1</x:v>
+        <x:v>599.35</x:v>
       </x:c>
       <x:c r="G76" s="18"/>
       <x:c r="H76" s="14"/>
       <x:c r="I76" s="19"/>
       <x:c r="J76" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K76" s="14" t="n">
-        <x:v>276.1</x:v>
+        <x:v>599.35</x:v>
       </x:c>
       <x:c r="L76" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4174,28 +4208,28 @@
         <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B77" s="18" t="n">
-        <x:v>2192512</x:v>
+        <x:v>2205674</x:v>
       </x:c>
       <x:c r="C77" s="13" t="n">
-        <x:v>15319</x:v>
+        <x:v>15402</x:v>
       </x:c>
       <x:c r="D77" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E77" s="19" t="n">
-        <x:v>46234.67115740741</x:v>
+        <x:v>46232.57876157408</x:v>
       </x:c>
       <x:c r="F77" s="14" t="n">
-        <x:v>630.36</x:v>
+        <x:v>2173.95</x:v>
       </x:c>
       <x:c r="G77" s="18"/>
       <x:c r="H77" s="14"/>
       <x:c r="I77" s="19"/>
       <x:c r="J77" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K77" s="14" t="n">
-        <x:v>630.36</x:v>
+        <x:v>2173.95</x:v>
       </x:c>
       <x:c r="L77" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4203,31 +4237,31 @@
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="13" t="str">
-        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
+        <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B78" s="18" t="n">
-        <x:v>2193158</x:v>
+        <x:v>2206284</x:v>
       </x:c>
       <x:c r="C78" s="13" t="n">
-        <x:v>15321</x:v>
+        <x:v>15405</x:v>
       </x:c>
       <x:c r="D78" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E78" s="19" t="n">
-        <x:v>46234.67115740741</x:v>
+        <x:v>46232.59909722222</x:v>
       </x:c>
       <x:c r="F78" s="14" t="n">
-        <x:v>226.75</x:v>
+        <x:v>568.61</x:v>
       </x:c>
       <x:c r="G78" s="18"/>
       <x:c r="H78" s="14"/>
       <x:c r="I78" s="19"/>
       <x:c r="J78" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K78" s="14" t="n">
-        <x:v>226.75</x:v>
+        <x:v>568.61</x:v>
       </x:c>
       <x:c r="L78" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4238,28 +4272,28 @@
         <x:v>Secur Mayara</x:v>
       </x:c>
       <x:c r="B79" s="18" t="n">
-        <x:v>2193214</x:v>
+        <x:v>2206293</x:v>
       </x:c>
       <x:c r="C79" s="13" t="n">
-        <x:v>15323</x:v>
+        <x:v>15406</x:v>
       </x:c>
       <x:c r="D79" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E79" s="19" t="n">
-        <x:v>46234.67115740741</x:v>
+        <x:v>46232.60854166667</x:v>
       </x:c>
       <x:c r="F79" s="14" t="n">
-        <x:v>222.19</x:v>
+        <x:v>454.22</x:v>
       </x:c>
       <x:c r="G79" s="18"/>
       <x:c r="H79" s="14"/>
       <x:c r="I79" s="19"/>
       <x:c r="J79" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K79" s="14" t="n">
-        <x:v>222.19</x:v>
+        <x:v>454.22</x:v>
       </x:c>
       <x:c r="L79" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4267,31 +4301,31 @@
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="13" t="str">
-        <x:v>LC Plásticos</x:v>
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
       </x:c>
       <x:c r="B80" s="18" t="n">
-        <x:v>2193641</x:v>
+        <x:v>2206603</x:v>
       </x:c>
       <x:c r="C80" s="13" t="n">
-        <x:v>15331</x:v>
+        <x:v>15408</x:v>
       </x:c>
       <x:c r="D80" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E80" s="19" t="n">
-        <x:v>46234.67115740741</x:v>
+        <x:v>46232.799525462964</x:v>
       </x:c>
       <x:c r="F80" s="14" t="n">
-        <x:v>781.33</x:v>
+        <x:v>124.44</x:v>
       </x:c>
       <x:c r="G80" s="18"/>
       <x:c r="H80" s="14"/>
       <x:c r="I80" s="19"/>
       <x:c r="J80" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K80" s="14" t="n">
-        <x:v>781.33</x:v>
+        <x:v>124.44</x:v>
       </x:c>
       <x:c r="L80" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4299,31 +4333,31 @@
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
+        <x:v>Vinilak Tintas Especiais</x:v>
       </x:c>
       <x:c r="B81" s="18" t="n">
-        <x:v>2194620</x:v>
+        <x:v>2207138</x:v>
       </x:c>
       <x:c r="C81" s="13" t="n">
-        <x:v>15335</x:v>
+        <x:v>15412</x:v>
       </x:c>
       <x:c r="D81" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E81" s="19" t="n">
-        <x:v>46234.67115740741</x:v>
+        <x:v>46233.56369212963</x:v>
       </x:c>
       <x:c r="F81" s="14" t="n">
-        <x:v>437.67</x:v>
+        <x:v>503.59</x:v>
       </x:c>
       <x:c r="G81" s="18"/>
       <x:c r="H81" s="14"/>
       <x:c r="I81" s="19"/>
       <x:c r="J81" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K81" s="14" t="n">
-        <x:v>437.67</x:v>
+        <x:v>503.59</x:v>
       </x:c>
       <x:c r="L81" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4331,31 +4365,31 @@
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
+        <x:v>João Pedro | Bprint Gráfica</x:v>
       </x:c>
       <x:c r="B82" s="18" t="n">
-        <x:v>2194619</x:v>
+        <x:v>2207378</x:v>
       </x:c>
       <x:c r="C82" s="13" t="n">
-        <x:v>15340</x:v>
+        <x:v>15414</x:v>
       </x:c>
       <x:c r="D82" s="13" t="str">
-        <x:v>Perdido</x:v>
+        <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E82" s="19" t="n">
-        <x:v>46234.681550925925</x:v>
+        <x:v>46233.572060185186</x:v>
       </x:c>
       <x:c r="F82" s="14" t="n">
-        <x:v>434.19</x:v>
+        <x:v>430.25</x:v>
       </x:c>
       <x:c r="G82" s="18"/>
       <x:c r="H82" s="14"/>
       <x:c r="I82" s="19"/>
       <x:c r="J82" s="13" t="str">
-        <x:v>NÃO APROVADA</x:v>
+        <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K82" s="14" t="n">
-        <x:v>434.19</x:v>
+        <x:v>430.25</x:v>
       </x:c>
       <x:c r="L82" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4363,22 +4397,22 @@
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="13" t="str">
-        <x:v>Secur Mayara</x:v>
+        <x:v>Carmaço - Fiori</x:v>
       </x:c>
       <x:c r="B83" s="18" t="n">
-        <x:v>2208468</x:v>
+        <x:v>2207562</x:v>
       </x:c>
       <x:c r="C83" s="13" t="n">
-        <x:v>15424</x:v>
+        <x:v>15417</x:v>
       </x:c>
       <x:c r="D83" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E83" s="19" t="n">
-        <x:v>46234.737546296295</x:v>
+        <x:v>46233.67563657407</x:v>
       </x:c>
       <x:c r="F83" s="14" t="n">
-        <x:v>310.75</x:v>
+        <x:v>390.31</x:v>
       </x:c>
       <x:c r="G83" s="18"/>
       <x:c r="H83" s="14"/>
@@ -4387,7 +4421,7 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K83" s="14" t="n">
-        <x:v>310.75</x:v>
+        <x:v>390.31</x:v>
       </x:c>
       <x:c r="L83" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
@@ -4395,22 +4429,22 @@
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="13" t="str">
-        <x:v>Viviane Pinheiro</x:v>
+        <x:v>Queren Cyrino</x:v>
       </x:c>
       <x:c r="B84" s="18" t="n">
-        <x:v>2208572</x:v>
+        <x:v>2207563</x:v>
       </x:c>
       <x:c r="C84" s="13" t="n">
-        <x:v>15425</x:v>
+        <x:v>15419</x:v>
       </x:c>
       <x:c r="D84" s="13" t="str">
         <x:v>Aberto</x:v>
       </x:c>
       <x:c r="E84" s="19" t="n">
-        <x:v>46234.7840625</x:v>
+        <x:v>46233.69023148148</x:v>
       </x:c>
       <x:c r="F84" s="14" t="n">
-        <x:v>770.68</x:v>
+        <x:v>1168.34</x:v>
       </x:c>
       <x:c r="G84" s="18"/>
       <x:c r="H84" s="14"/>
@@ -4419,9 +4453,451 @@
         <x:v>ABERTA</x:v>
       </x:c>
       <x:c r="K84" s="14" t="n">
+        <x:v>1168.34</x:v>
+      </x:c>
+      <x:c r="L84" s="20" t="str">
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" s="13" t="str">
+        <x:v>WOOD COLOR TINTAS</x:v>
+      </x:c>
+      <x:c r="B85" s="18" t="n">
+        <x:v>2207637</x:v>
+      </x:c>
+      <x:c r="C85" s="13" t="str"/>
+      <x:c r="D85" s="13" t="str">
+        <x:v>Perdido</x:v>
+      </x:c>
+      <x:c r="E85" s="19" t="n">
+        <x:v>46233.700266203705</x:v>
+      </x:c>
+      <x:c r="F85" s="14" t="n">
+        <x:v>404.88</x:v>
+      </x:c>
+      <x:c r="G85" s="18"/>
+      <x:c r="H85" s="14"/>
+      <x:c r="I85" s="19"/>
+      <x:c r="J85" s="13" t="str"/>
+      <x:c r="K85" s="14"/>
+      <x:c r="L85" s="20" t="str">
+        <x:v>Card sem número de cotação identificável na timeline.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86">
+      <x:c r="A86" s="13" t="str">
+        <x:v>Juciliana</x:v>
+      </x:c>
+      <x:c r="B86" s="18" t="n">
+        <x:v>2206455</x:v>
+      </x:c>
+      <x:c r="C86" s="13" t="n">
+        <x:v>15407</x:v>
+      </x:c>
+      <x:c r="D86" s="13" t="str">
+        <x:v>Perdido</x:v>
+      </x:c>
+      <x:c r="E86" s="19" t="n">
+        <x:v>46233.70322916667</x:v>
+      </x:c>
+      <x:c r="F86" s="14" t="n">
+        <x:v>251.25</x:v>
+      </x:c>
+      <x:c r="G86" s="18"/>
+      <x:c r="H86" s="14"/>
+      <x:c r="I86" s="19"/>
+      <x:c r="J86" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K86" s="14" t="n">
+        <x:v>251.25</x:v>
+      </x:c>
+      <x:c r="L86" s="20" t="str">
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" s="13" t="str">
+        <x:v>FRANCHI NORTE DISTRIBUICAO LTDA</x:v>
+      </x:c>
+      <x:c r="B87" s="18" t="n">
+        <x:v>2205563</x:v>
+      </x:c>
+      <x:c r="C87" s="13" t="n">
+        <x:v>15396</x:v>
+      </x:c>
+      <x:c r="D87" s="13" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="E87" s="19" t="n">
+        <x:v>46233.765810185185</x:v>
+      </x:c>
+      <x:c r="F87" s="14" t="n">
+        <x:v>250.89</x:v>
+      </x:c>
+      <x:c r="G87" s="18"/>
+      <x:c r="H87" s="14"/>
+      <x:c r="I87" s="19"/>
+      <x:c r="J87" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K87" s="14" t="n">
+        <x:v>250.89</x:v>
+      </x:c>
+      <x:c r="L87" s="20" t="str">
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" s="13" t="str">
+        <x:v>NEON COMERCIAL REAGENTES ANALITICOS LTDA.</x:v>
+      </x:c>
+      <x:c r="B88" s="18" t="n">
+        <x:v>2208212</x:v>
+      </x:c>
+      <x:c r="C88" s="13" t="n">
+        <x:v>15421</x:v>
+      </x:c>
+      <x:c r="D88" s="13" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="E88" s="19" t="n">
+        <x:v>46234.513715277775</x:v>
+      </x:c>
+      <x:c r="F88" s="14" t="n">
+        <x:v>142.51</x:v>
+      </x:c>
+      <x:c r="G88" s="18"/>
+      <x:c r="H88" s="14"/>
+      <x:c r="I88" s="19"/>
+      <x:c r="J88" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K88" s="14" t="n">
+        <x:v>142.51</x:v>
+      </x:c>
+      <x:c r="L88" s="20" t="str">
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="13" t="str">
+        <x:v>Elisete Henck</x:v>
+      </x:c>
+      <x:c r="B89" s="18" t="n">
+        <x:v>2208349</x:v>
+      </x:c>
+      <x:c r="C89" s="13" t="n">
+        <x:v>15423</x:v>
+      </x:c>
+      <x:c r="D89" s="13" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="E89" s="19" t="n">
+        <x:v>46234.616793981484</x:v>
+      </x:c>
+      <x:c r="F89" s="14" t="n">
+        <x:v>107.37</x:v>
+      </x:c>
+      <x:c r="G89" s="18"/>
+      <x:c r="H89" s="14"/>
+      <x:c r="I89" s="19"/>
+      <x:c r="J89" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K89" s="14" t="n">
+        <x:v>107.37</x:v>
+      </x:c>
+      <x:c r="L89" s="20" t="str">
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="13" t="str">
+        <x:v>Logistica</x:v>
+      </x:c>
+      <x:c r="B90" s="18" t="n">
+        <x:v>2191659</x:v>
+      </x:c>
+      <x:c r="C90" s="13" t="n">
+        <x:v>15317</x:v>
+      </x:c>
+      <x:c r="D90" s="13" t="str">
+        <x:v>Perdido</x:v>
+      </x:c>
+      <x:c r="E90" s="19" t="n">
+        <x:v>46234.67115740741</x:v>
+      </x:c>
+      <x:c r="F90" s="14" t="n">
+        <x:v>276.1</x:v>
+      </x:c>
+      <x:c r="G90" s="18"/>
+      <x:c r="H90" s="14"/>
+      <x:c r="I90" s="19"/>
+      <x:c r="J90" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K90" s="14" t="n">
+        <x:v>276.1</x:v>
+      </x:c>
+      <x:c r="L90" s="20" t="str">
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" s="13" t="str">
+        <x:v>Secur Mayara</x:v>
+      </x:c>
+      <x:c r="B91" s="18" t="n">
+        <x:v>2192512</x:v>
+      </x:c>
+      <x:c r="C91" s="13" t="n">
+        <x:v>15319</x:v>
+      </x:c>
+      <x:c r="D91" s="13" t="str">
+        <x:v>Perdido</x:v>
+      </x:c>
+      <x:c r="E91" s="19" t="n">
+        <x:v>46234.67115740741</x:v>
+      </x:c>
+      <x:c r="F91" s="14" t="n">
+        <x:v>630.36</x:v>
+      </x:c>
+      <x:c r="G91" s="18"/>
+      <x:c r="H91" s="14"/>
+      <x:c r="I91" s="19"/>
+      <x:c r="J91" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K91" s="14" t="n">
+        <x:v>630.36</x:v>
+      </x:c>
+      <x:c r="L91" s="20" t="str">
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="92">
+      <x:c r="A92" s="13" t="str">
+        <x:v>WORLD COLOR - REVESTIMENTOS</x:v>
+      </x:c>
+      <x:c r="B92" s="18" t="n">
+        <x:v>2193158</x:v>
+      </x:c>
+      <x:c r="C92" s="13" t="n">
+        <x:v>15321</x:v>
+      </x:c>
+      <x:c r="D92" s="13" t="str">
+        <x:v>Perdido</x:v>
+      </x:c>
+      <x:c r="E92" s="19" t="n">
+        <x:v>46234.67115740741</x:v>
+      </x:c>
+      <x:c r="F92" s="14" t="n">
+        <x:v>226.75</x:v>
+      </x:c>
+      <x:c r="G92" s="18"/>
+      <x:c r="H92" s="14"/>
+      <x:c r="I92" s="19"/>
+      <x:c r="J92" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K92" s="14" t="n">
+        <x:v>226.75</x:v>
+      </x:c>
+      <x:c r="L92" s="20" t="str">
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" s="13" t="str">
+        <x:v>Secur Mayara</x:v>
+      </x:c>
+      <x:c r="B93" s="18" t="n">
+        <x:v>2193214</x:v>
+      </x:c>
+      <x:c r="C93" s="13" t="n">
+        <x:v>15323</x:v>
+      </x:c>
+      <x:c r="D93" s="13" t="str">
+        <x:v>Perdido</x:v>
+      </x:c>
+      <x:c r="E93" s="19" t="n">
+        <x:v>46234.67115740741</x:v>
+      </x:c>
+      <x:c r="F93" s="14" t="n">
+        <x:v>222.19</x:v>
+      </x:c>
+      <x:c r="G93" s="18"/>
+      <x:c r="H93" s="14"/>
+      <x:c r="I93" s="19"/>
+      <x:c r="J93" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K93" s="14" t="n">
+        <x:v>222.19</x:v>
+      </x:c>
+      <x:c r="L93" s="20" t="str">
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" s="13" t="str">
+        <x:v>LC Plásticos</x:v>
+      </x:c>
+      <x:c r="B94" s="18" t="n">
+        <x:v>2193641</x:v>
+      </x:c>
+      <x:c r="C94" s="13" t="n">
+        <x:v>15331</x:v>
+      </x:c>
+      <x:c r="D94" s="13" t="str">
+        <x:v>Perdido</x:v>
+      </x:c>
+      <x:c r="E94" s="19" t="n">
+        <x:v>46234.67115740741</x:v>
+      </x:c>
+      <x:c r="F94" s="14" t="n">
+        <x:v>781.33</x:v>
+      </x:c>
+      <x:c r="G94" s="18"/>
+      <x:c r="H94" s="14"/>
+      <x:c r="I94" s="19"/>
+      <x:c r="J94" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K94" s="14" t="n">
+        <x:v>781.33</x:v>
+      </x:c>
+      <x:c r="L94" s="20" t="str">
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="95">
+      <x:c r="A95" s="13" t="str">
+        <x:v>Secur Mayara</x:v>
+      </x:c>
+      <x:c r="B95" s="18" t="n">
+        <x:v>2194620</x:v>
+      </x:c>
+      <x:c r="C95" s="13" t="n">
+        <x:v>15335</x:v>
+      </x:c>
+      <x:c r="D95" s="13" t="str">
+        <x:v>Perdido</x:v>
+      </x:c>
+      <x:c r="E95" s="19" t="n">
+        <x:v>46234.67115740741</x:v>
+      </x:c>
+      <x:c r="F95" s="14" t="n">
+        <x:v>437.67</x:v>
+      </x:c>
+      <x:c r="G95" s="18"/>
+      <x:c r="H95" s="14"/>
+      <x:c r="I95" s="19"/>
+      <x:c r="J95" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K95" s="14" t="n">
+        <x:v>437.67</x:v>
+      </x:c>
+      <x:c r="L95" s="20" t="str">
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" s="13" t="str">
+        <x:v>Secur Mayara</x:v>
+      </x:c>
+      <x:c r="B96" s="18" t="n">
+        <x:v>2194619</x:v>
+      </x:c>
+      <x:c r="C96" s="13" t="n">
+        <x:v>15340</x:v>
+      </x:c>
+      <x:c r="D96" s="13" t="str">
+        <x:v>Perdido</x:v>
+      </x:c>
+      <x:c r="E96" s="19" t="n">
+        <x:v>46234.681550925925</x:v>
+      </x:c>
+      <x:c r="F96" s="14" t="n">
+        <x:v>434.19</x:v>
+      </x:c>
+      <x:c r="G96" s="18"/>
+      <x:c r="H96" s="14"/>
+      <x:c r="I96" s="19"/>
+      <x:c r="J96" s="13" t="str">
+        <x:v>NÃO APROVADA</x:v>
+      </x:c>
+      <x:c r="K96" s="14" t="n">
+        <x:v>434.19</x:v>
+      </x:c>
+      <x:c r="L96" s="20" t="str">
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" s="13" t="str">
+        <x:v>Secur Mayara</x:v>
+      </x:c>
+      <x:c r="B97" s="18" t="n">
+        <x:v>2208468</x:v>
+      </x:c>
+      <x:c r="C97" s="13" t="n">
+        <x:v>15424</x:v>
+      </x:c>
+      <x:c r="D97" s="13" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="E97" s="19" t="n">
+        <x:v>46234.737546296295</x:v>
+      </x:c>
+      <x:c r="F97" s="14" t="n">
+        <x:v>310.75</x:v>
+      </x:c>
+      <x:c r="G97" s="18"/>
+      <x:c r="H97" s="14"/>
+      <x:c r="I97" s="19"/>
+      <x:c r="J97" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K97" s="14" t="n">
+        <x:v>310.75</x:v>
+      </x:c>
+      <x:c r="L97" s="20" t="str">
+        <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" s="13" t="str">
+        <x:v>Viviane Pinheiro</x:v>
+      </x:c>
+      <x:c r="B98" s="18" t="n">
+        <x:v>2208572</x:v>
+      </x:c>
+      <x:c r="C98" s="13" t="n">
+        <x:v>15425</x:v>
+      </x:c>
+      <x:c r="D98" s="13" t="str">
+        <x:v>Aberto</x:v>
+      </x:c>
+      <x:c r="E98" s="19" t="n">
+        <x:v>46234.7840625</x:v>
+      </x:c>
+      <x:c r="F98" s="14" t="n">
         <x:v>770.68</x:v>
       </x:c>
-      <x:c r="L84" s="20" t="str">
+      <x:c r="G98" s="18"/>
+      <x:c r="H98" s="14"/>
+      <x:c r="I98" s="19"/>
+      <x:c r="J98" s="13" t="str">
+        <x:v>ABERTA</x:v>
+      </x:c>
+      <x:c r="K98" s="14" t="n">
+        <x:v>770.68</x:v>
+      </x:c>
+      <x:c r="L98" s="20" t="str">
         <x:v>Nenhum CT-e considerado: não localizado no dia ou após a cotação.</x:v>
       </x:c>
     </x:row>
@@ -4432,7 +4908,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13dabc07b8bc4012"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra0809dc7bb464742"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>